<commit_message>
Central sign-in: Portal authenticates, IT Hub roles authorise; deny unregistered or unmapped users
</commit_message>
<xml_diff>
--- a/Claude outputs/IT_Asset_Module_Test_Case_Suite.xlsx
+++ b/Claude outputs/IT_Asset_Module_Test_Case_Suite.xlsx
@@ -10,10 +10,10 @@
   <sheets>
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Test Cases" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Portal Setup &amp; Page Keys" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="IT Hub Roles &amp; Access" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Test Cases'!$A$1:$O$106</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Test Cases'!$A$1:$O$109</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1292" uniqueCount="568">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1325" uniqueCount="577">
   <si>
     <t xml:space="preserve">IT Asset Management — Test Case Suite</t>
   </si>
@@ -186,7 +186,7 @@
     <t xml:space="preserve">Example: UAT Result = Pass, UAT Tester = 'IT Asset team', UAT Date = 2026-10-20, Remarks = 'OK on Chrome / Android'.</t>
   </si>
   <si>
-    <t xml:space="preserve">Central Identity cases need the Portal admin to register IT Hub first — values on the 'Portal Setup &amp; Page Keys' sheet.</t>
+    <t xml:space="preserve">Portal sign-in cases need the Portal admin to register IT Hub, and the users created in IT Hub User Master with a role — see 'IT Hub Roles &amp; Access'.</t>
   </si>
   <si>
     <t xml:space="preserve">Test ID</t>
@@ -601,7 +601,7 @@
     <t xml:space="preserve">state=Expiring for an end date within 30 days</t>
   </si>
   <si>
-    <t xml:space="preserve">state=Expiring, daysLeft=23</t>
+    <t xml:space="preserve">state=Expiring, daysLeft=17</t>
   </si>
   <si>
     <t xml:space="preserve">CT-04</t>
@@ -861,8 +861,8 @@
     <t xml:space="preserve">Dashboard is permission-checked</t>
   </si>
   <si>
-    <t xml:space="preserve">Sign in as a user without the Asset Dashboard page and open /assets.
-[API check: GET /api/asset-dashboard without the "assets" module]</t>
+    <t xml:space="preserve">Sign in as a user whose IT Hub role has Asset Registry but not Asset Dashboard; open /assets.
+[API check: Sign in as a user whose IT Hub role lacks "Asset Dashboard"; GET /api/asset-dashboard]</t>
   </si>
   <si>
     <t xml:space="preserve">HTTP 403</t>
@@ -874,7 +874,7 @@
     <t xml:space="preserve">Login page discovers Ashika Portal sign-in</t>
   </si>
   <si>
-    <t xml:space="preserve">IT Hub registered in Ashika Portal (sso_apps); CENTRAL_SSO_* set on the server.</t>
+    <t xml:space="preserve">IT Hub registered in Ashika Portal (sso_apps); CENTRAL_SSO_* set on the server; users created in IT Hub User Master.</t>
   </si>
   <si>
     <t xml:space="preserve">Open https://ithub-uat.niytri.com/login.
@@ -913,40 +913,66 @@
     <t xml:space="preserve">SSO-04</t>
   </si>
   <si>
-    <t xml:space="preserve">Full-access Portal user signs in (authorize → code → token)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Click 'Sign in with Ashika Portal'. Sign in on the Portal as a user whose role has full access (pages *).
-[API check: Start /api/auth/central/login, Portal returns code, app exchanges it]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lands on requested page; /auth/me role=admin, identitySource=central, all modules admin</t>
+    <t xml:space="preserve">Registered IT Hub admin signs in through the Portal (authorize → code → token)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Admin › User Master: make sure the user exists (same email as the Portal) with role Admin. Click 'Sign in with Ashika Portal' and sign in on the Portal.
+[API check: Start /api/auth/central/login; Portal authenticates; IT Hub exchanges the code]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lands on requested page; /auth/me role=admin (from IT Hub), identitySource=central</t>
   </si>
   <si>
     <t xml:space="preserve">SSO-05</t>
   </si>
   <si>
-    <t xml:space="preserve">First Portal sign-in provisions a local profile without a password</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(DB / Admin › User Master) After SSO-04, open User Master and find the user.
-[API check: Check users table after SSO-04]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">User row exists, identity_source=central, password_hash empty</t>
+    <t xml:space="preserve">Portal-authenticated person NOT registered in IT Hub is refused</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sign in via the Portal as a person who is NOT in IT Hub User Master.
+[API check: Sign in via Portal as a person with no IT Hub user record]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Redirect to /login?sso_error=not_registered; no user created; no session</t>
   </si>
   <si>
     <t xml:space="preserve">SSO-06</t>
   </si>
   <si>
-    <t xml:space="preserve">View-only Portal role gets read access only to its pages</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sign in via Portal as a user whose IT Hub role has view on Asset Dashboard, Asset Registry, Licenses only.
-[API check: Sign in as Asset Viewer (pages: assets, asset_registry, asset_licenses — view)]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/auth/me shows read for those 3 modules and nothing else</t>
+    <t xml:space="preserve">Registered user with NO IT Hub role is refused</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Admin › User Master: create the user with NO role. Sign in via the Portal as that user.
+[API check: Sign in via Portal as a user present in IT Hub without any role]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Redirect to /login?sso_error=no_role; no session</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SSO-14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User disabled in IT Hub is refused even if the Portal allows</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Admin › User Master: deactivate a user. That user signs in via the Portal.
+[API check: Deactivate in User Master; sign in via Portal]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Redirect to /login?sso_error=account_disabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SSO-15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Access comes from the IT Hub role, not the Portal role</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Admin › User Master: give a user only the role 'Asset Viewer'. Sign in via the Portal as that user and check the IT Assets menu.
+[API check: Sign in via Portal as a user mapped to IT Hub role "Asset Viewer"]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/auth/me shows read on assets + asset_registry only (Portal permissions ignored)</t>
   </si>
   <si>
     <t xml:space="preserve">RBAC-01</t>
@@ -955,7 +981,7 @@
     <t xml:space="preserve">Viewer can read the asset register</t>
   </si>
   <si>
-    <t xml:space="preserve">Portal roles exist for the listed page keys (see 'Portal Setup &amp; Page Keys').</t>
+    <t xml:space="preserve">Users mapped to IT Hub roles (see 'IT Hub Roles &amp; Access').</t>
   </si>
   <si>
     <t xml:space="preserve">As the view-only user open IT Assets › Asset Registry.
@@ -981,7 +1007,7 @@
     <t xml:space="preserve">RBAC-03</t>
   </si>
   <si>
-    <t xml:space="preserve">Viewer cannot open a module not in the Portal role</t>
+    <t xml:space="preserve">Viewer cannot open a module not in the IT Hub role</t>
   </si>
   <si>
     <t xml:space="preserve">As the view-only user type /asset-contracts in the address bar.
@@ -1011,11 +1037,11 @@
     <t xml:space="preserve">RBAC-06</t>
   </si>
   <si>
-    <t xml:space="preserve">Asset Manager (edit on registry) can create and edit assets</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sign in as a user with edit on Asset Registry. Add an asset, then edit its location with a comment.
-[API check: Sign in as Asset Manager; POST /api/assets; PATCH with comment]</t>
+    <t xml:space="preserve">IT Asset Manager role can create and edit assets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sign in as a user with IT Hub role 'IT Asset Manager'. Add an asset, then edit its location with a comment.
+[API check: Sign in as a user with IT Hub role "IT Asset Manager"; add an asset; edit with comment]</t>
   </si>
   <si>
     <t xml:space="preserve">HTTP 201 then 200</t>
@@ -1024,7 +1050,7 @@
     <t xml:space="preserve">RBAC-07</t>
   </si>
   <si>
-    <t xml:space="preserve">Asset Manager can issue (asset_allocations: edit)</t>
+    <t xml:space="preserve">IT Asset Manager can issue (asset_allocations: write)</t>
   </si>
   <si>
     <t xml:space="preserve">As the same user open Handovers › Issue assets and issue the asset.
@@ -1037,7 +1063,7 @@
     <t xml:space="preserve">RBAC-08</t>
   </si>
   <si>
-    <t xml:space="preserve">Asset Manager cannot change depreciation rules (not in role)</t>
+    <t xml:space="preserve">IT Asset Manager cannot change depreciation rules (read only in role)</t>
   </si>
   <si>
     <t xml:space="preserve">As the same user open /asset-depreciation (not in role).
@@ -1047,7 +1073,7 @@
     <t xml:space="preserve">RBAC-09</t>
   </si>
   <si>
-    <t xml:space="preserve">Shared reference data: manager can read vendor list without vendor module</t>
+    <t xml:space="preserve">Shared reference data: vendor list readable with any asset access</t>
   </si>
   <si>
     <t xml:space="preserve">As the same user open Add Asset — the Vendor list loads.
@@ -1057,24 +1083,37 @@
     <t xml:space="preserve">SSO-07</t>
   </si>
   <si>
-    <t xml:space="preserve">Role change in the Portal takes effect without re-login</t>
-  </si>
-  <si>
-    <t xml:space="preserve">In the Portal give the view-only user 'edit' on asset_registry. Within 1 minute refresh IT Hub and add an asset (no re-login).
-[API check: Grant Viewer edit on asset_registry in Portal; wait for re-validation; POST /api/assets]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Create succeeds (HTTP 201)</t>
+    <t xml:space="preserve">Role change in IT Hub applies without re-login</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Admin › User Master: add role 'IT Asset Manager' to the view-only user. The user refreshes and adds an asset (no re-login).
+[API check: Admin › User Master: add "IT Asset Manager" to the viewer; viewer adds an asset]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create succeeds (HTTP 201) immediately</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SSO-16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All IT Hub roles removed → session ends</t>
+  </si>
+  <si>
+    <t xml:space="preserve">While the user is signed in, remove all their roles in User Master; the user clicks anything after a minute.
+[API check: Remove every role from the user in User Master; user clicks anything]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HTTP 401 code=central_no_role at the next check; back to login</t>
   </si>
   <si>
     <t xml:space="preserve">SSO-08</t>
   </si>
   <si>
-    <t xml:space="preserve">User disabled in the Portal is locked out immediately</t>
+    <t xml:space="preserve">User disabled in the Portal is locked out</t>
   </si>
   <si>
     <t xml:space="preserve">In the Portal disable the user. Within 1 minute click anything in IT Hub.
-[API check: Disable Viewer in Portal; next request after re-validation]</t>
+[API check: Disable the user in the Portal; next request after re-validation]</t>
   </si>
   <si>
     <t xml:space="preserve">HTTP 401 code=central_inactive; session destroyed</t>
@@ -1083,11 +1122,11 @@
     <t xml:space="preserve">SSO-09</t>
   </si>
   <si>
-    <t xml:space="preserve">Portal denies a user without access to IT Hub</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sign in via Portal as a user whose role is not tagged to IT Hub.
-[API check: Sign in as a user whose role is not tagged to IT Hub]</t>
+    <t xml:space="preserve">Portal refuses a user not allowed for IT Hub</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sign in via Portal as a user the Portal does not allow into IT Hub (if the Portal restricts apps).
+[API check: Sign in as a user the Portal does not allow for this app]</t>
   </si>
   <si>
     <t xml:space="preserve">Redirect to /login?sso_error=access_denied, no session</t>
@@ -1177,19 +1216,19 @@
     <t xml:space="preserve">RBAC-10</t>
   </si>
   <si>
-    <t xml:space="preserve">Menu &amp; page access follow the Portal role (browser)</t>
+    <t xml:space="preserve">Menu &amp; page access follow the IT Hub role (browser)</t>
   </si>
   <si>
     <t xml:space="preserve">Central Identity enabled; Portal roles configured.</t>
   </si>
   <si>
-    <t xml:space="preserve">Sign in via Portal as Asset Manager, Asset Viewer and Full-access users; open every IT Asset page.</t>
+    <t xml:space="preserve">Sign in via Portal as users mapped to IT Asset Manager, Asset Viewer and Admin; open every IT Asset page.</t>
   </si>
   <si>
     <t xml:space="preserve">Pages outside the role show 'You don't have access to this page'; Add/Edit buttons only where the role has edit.</t>
   </si>
   <si>
-    <t xml:space="preserve">Manager: edit on Registry, Contracts, Handovers; no access to Licenses, Depreciation, Audit, Vendors. Viewer: view-only Registry/Licenses. Admin: all. No console errors.</t>
+    <t xml:space="preserve">IT Asset Manager: edit everywhere except Depreciation (view). Asset Viewer: view Dashboard + Registry only. Admin: all. No console errors.</t>
   </si>
   <si>
     <t xml:space="preserve">RBAC-11</t>
@@ -1492,13 +1531,13 @@
     <t xml:space="preserve">UI-23</t>
   </si>
   <si>
-    <t xml:space="preserve">Local roles include new modules</t>
+    <t xml:space="preserve">Standard IT Asset roles present</t>
   </si>
   <si>
     <t xml:space="preserve">Admin › Roles &amp; Permissions.</t>
   </si>
   <si>
-    <t xml:space="preserve">Contracts, Depreciation, Physical Audit appear as separate modules.</t>
+    <t xml:space="preserve">IT Asset Manager, Asset Auditor, Finance (Assets), Asset Viewer exist with the access shown on the 'IT Hub Roles &amp; Access' sheet; Contracts, Depreciation, Physical Audit are separate modules.</t>
   </si>
   <si>
     <t xml:space="preserve">UI-24</t>
@@ -1531,10 +1570,10 @@
     <t xml:space="preserve">Microsoft 365 staff sign-in</t>
   </si>
   <si>
-    <t xml:space="preserve">Portal › Sign in with Microsoft (staff account with M365-enabled role).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Entra MFA prompt; lands in IT Hub with the Portal role's access.</t>
+    <t xml:space="preserve">Portal › Sign in with Microsoft (staff account registered in IT Hub with a role).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entra MFA prompt; lands in IT Hub with the access of their IT Hub role.</t>
   </si>
   <si>
     <t xml:space="preserve">UI-27</t>
@@ -1555,10 +1594,10 @@
     <t xml:space="preserve">Session ended message</t>
   </si>
   <si>
-    <t xml:space="preserve">Disable the user in the Portal while they are on a page; click anything.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Redirected to login with 'Your session was ended by the Ashika Portal'.</t>
+    <t xml:space="preserve">Disable the user in the Portal (or remove their IT Hub roles) while they are on a page; click anything.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Redirected to login with 'Your session has ended'.</t>
   </si>
   <si>
     <t xml:space="preserve">UI-29</t>
@@ -1585,7 +1624,28 @@
     <t xml:space="preserve">Pages load within 3 seconds.</t>
   </si>
   <si>
-    <t xml:space="preserve">Ashika Portal — IT Hub registration (sso_apps)</t>
+    <t xml:space="preserve">How sign-in and access work</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. The Ashika Portal checks WHO the person is (Microsoft 365 or Portal password + OTP, with MFA).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. IT Hub decides WHAT they can do — from the roles assigned in IT Hub › Admin › User Master.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. If the person is not in IT Hub User Master (same email as the Portal), sign-in is refused.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. If they are in IT Hub but have no role (and are not Admin), sign-in is refused.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. If they are deactivated in IT Hub or in the Portal, or all their roles are removed, they are signed out within a minute.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6. Local password sign-in remains only for IT Hub administrators (break-glass).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ashika Portal — register IT Hub (sso_apps)</t>
   </si>
   <si>
     <t xml:space="preserve">client_id</t>
@@ -1603,48 +1663,99 @@
     <t xml:space="preserve">client_secret</t>
   </si>
   <si>
-    <t xml:space="preserve">Generated by the Portal admin; given to the IT Hub server admin privately (never by email/chat)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">allowed_roles</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Optional — leave blank and control access through role_applications</t>
-  </si>
-  <si>
-    <t xml:space="preserve">application</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tag IT Hub roles to the 'IT Hub' application (role_applications)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Page keys used by IT Hub (put these in the Portal role's pages / access)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Page key</t>
+    <t xml:space="preserve">Generated by the Portal admin; given privately to the IT Hub server admin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Portal roles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No IT Hub-specific roles needed in the Portal; access is mapped in IT Hub</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IT Hub roles (created by db/10_asset_roles.sql — assign in Admin › User Master)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Role</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Edit (write)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">View (read only)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Use</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Admin (user role = Admin)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Everything incl. Admin, Clear All Data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">—</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IT head / application admin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IT Asset Manager</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Asset Registry, Handovers, Contracts &amp; AMC, Licenses, Vendors, Physical Audit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Asset Dashboard, Depreciation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Runs the asset desk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Asset Auditor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Asset Dashboard, Asset Registry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Physical verification team</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Finance (Assets)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Asset Dashboard, Asset Registry, Contracts &amp; AMC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fixed-asset register, AMC spend</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Asset Viewer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Management / auditors (read-only)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Screen ↔ module key (for custom roles in Admin › Roles &amp; Permissions)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Module key</t>
   </si>
   <si>
     <t xml:space="preserve">IT Hub screen</t>
   </si>
   <si>
-    <t xml:space="preserve">'view' allows</t>
-  </si>
-  <si>
-    <t xml:space="preserve">'edit' allows</t>
+    <t xml:space="preserve">View allows</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Edit allows</t>
   </si>
   <si>
     <t xml:space="preserve">assets</t>
   </si>
   <si>
-    <t xml:space="preserve">IT Assets › Asset Dashboard</t>
-  </si>
-  <si>
     <t xml:space="preserve">Dashboard</t>
   </si>
   <si>
-    <t xml:space="preserve">—</t>
-  </si>
-  <si>
     <t xml:space="preserve">asset_registry</t>
   </si>
   <si>
@@ -1654,7 +1765,7 @@
     <t xml:space="preserve">View assets, coverage, history</t>
   </si>
   <si>
-    <t xml:space="preserve">Add / edit / upload / lifecycle (maintenance, retire, dispose), finance upload, comments</t>
+    <t xml:space="preserve">Add / edit / upload / lifecycle, finance upload, comments</t>
   </si>
   <si>
     <t xml:space="preserve">asset_allocations</t>
@@ -1678,7 +1789,7 @@
     <t xml:space="preserve">View contracts and warranty coverage</t>
   </si>
   <si>
-    <t xml:space="preserve">Create / edit / renew / delete contracts, add or remove covered assets</t>
+    <t xml:space="preserve">Create / edit / renew / delete contracts, covered assets</t>
   </si>
   <si>
     <t xml:space="preserve">asset_depreciation</t>
@@ -1720,88 +1831,7 @@
     <t xml:space="preserve">Plan, start, scan, complete, cancel audits</t>
   </si>
   <si>
-    <t xml:space="preserve">pages: ["*"]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Full access</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Everything</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Everything incl. Admin, Clear All Data</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Suggested Portal roles for IT Hub</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Role (same name in Portal and IT Hub)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Portal role permissions JSON — paste as-is</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Use</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IT Hub local role (password users)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IT Hub Admin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{"pages": ["*"]}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IT head / application admin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Local: users with role Admin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IT Asset Manager</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{"pages": ["assets", "asset_registry", "asset_allocations", "asset_contracts", "asset_licenses", "asset_vendors", "asset_audits", "asset_depreciation"], "access": {"assets": "view", "asset_registry": "edit", "asset_allocations": "edit", "asset_contracts": "edit", "asset_licenses": "edit", "asset_vendors": "edit", "asset_audits": "edit", "asset_depreciation": "view"}, "pii_view": false}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Runs the asset desk</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Created by db/10_asset_roles.sql</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Asset Auditor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{"pages": ["assets", "asset_registry", "asset_audits"], "access": {"assets": "view", "asset_registry": "view", "asset_audits": "edit"}, "pii_view": false}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Physical verification team</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Finance (Assets)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{"pages": ["assets", "asset_registry", "asset_depreciation", "asset_contracts"], "access": {"assets": "view", "asset_registry": "view", "asset_depreciation": "edit", "asset_contracts": "view"}, "pii_view": false}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fixed-asset register, AMC spend</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Asset Viewer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{"pages": ["assets", "asset_registry"], "access": {"assets": "view", "asset_registry": "view"}, "pii_view": false}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Management / auditors (read-only)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">In the Portal: create each role, paste its JSON as the permissions, and tick the 'IT Hub' application (role_applications).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Every employee can always open My Assets and acknowledge their own handovers; no page key needed.</t>
+    <t xml:space="preserve">Every employee can always open My Assets and acknowledge their own handovers; no role needed beyond being able to sign in.</t>
   </si>
 </sst>
 </file>
@@ -1813,7 +1843,7 @@
     <numFmt numFmtId="165" formatCode="General"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1878,12 +1908,6 @@
       <sz val="12"/>
       <color rgb="FF1F4E9E"/>
       <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Consolas"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
@@ -1963,7 +1987,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="17">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2030,14 +2054,6 @@
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -2448,27 +2464,27 @@
         <v>21</v>
       </c>
       <c r="C11" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A11,'Test Cases'!$C$2:$C$106,$B11)</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A11,'Test Cases'!$C$2:$C$109,$B11)</f>
         <v>12</v>
       </c>
       <c r="D11" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A11,'Test Cases'!$C$2:$C$106,$B11,'Test Cases'!$J$2:$J$106,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A11,'Test Cases'!$C$2:$C$109,$B11,'Test Cases'!$J$2:$J$109,"Pass")</f>
         <v>8</v>
       </c>
       <c r="E11" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A11,'Test Cases'!$C$2:$C$106,$B11,'Test Cases'!$J$2:$J$106,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A11,'Test Cases'!$C$2:$C$109,$B11,'Test Cases'!$J$2:$J$109,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F11" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A11,'Test Cases'!$C$2:$C$106,$B11,'Test Cases'!$J$2:$J$106,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A11,'Test Cases'!$C$2:$C$109,$B11,'Test Cases'!$J$2:$J$109,"Manual (UAT)")</f>
         <v>4</v>
       </c>
       <c r="G11" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A11,'Test Cases'!$C$2:$C$106,$B11,'Test Cases'!$L$2:$L$106,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A11,'Test Cases'!$C$2:$C$109,$B11,'Test Cases'!$L$2:$L$109,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H11" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A11,'Test Cases'!$C$2:$C$106,$B11,'Test Cases'!$L$2:$L$106,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A11,'Test Cases'!$C$2:$C$109,$B11,'Test Cases'!$L$2:$L$109,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I11" s="6" t="n">
@@ -2484,27 +2500,27 @@
         <v>22</v>
       </c>
       <c r="C12" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A12,'Test Cases'!$C$2:$C$106,$B12)</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A12,'Test Cases'!$C$2:$C$109,$B12)</f>
         <v>3</v>
       </c>
       <c r="D12" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A12,'Test Cases'!$C$2:$C$106,$B12,'Test Cases'!$J$2:$J$106,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A12,'Test Cases'!$C$2:$C$109,$B12,'Test Cases'!$J$2:$J$109,"Pass")</f>
         <v>2</v>
       </c>
       <c r="E12" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A12,'Test Cases'!$C$2:$C$106,$B12,'Test Cases'!$J$2:$J$106,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A12,'Test Cases'!$C$2:$C$109,$B12,'Test Cases'!$J$2:$J$109,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F12" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A12,'Test Cases'!$C$2:$C$106,$B12,'Test Cases'!$J$2:$J$106,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A12,'Test Cases'!$C$2:$C$109,$B12,'Test Cases'!$J$2:$J$109,"Manual (UAT)")</f>
         <v>1</v>
       </c>
       <c r="G12" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A12,'Test Cases'!$C$2:$C$106,$B12,'Test Cases'!$L$2:$L$106,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A12,'Test Cases'!$C$2:$C$109,$B12,'Test Cases'!$L$2:$L$109,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H12" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A12,'Test Cases'!$C$2:$C$106,$B12,'Test Cases'!$L$2:$L$106,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A12,'Test Cases'!$C$2:$C$109,$B12,'Test Cases'!$L$2:$L$109,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I12" s="6" t="n">
@@ -2520,27 +2536,27 @@
         <v>23</v>
       </c>
       <c r="C13" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A13,'Test Cases'!$C$2:$C$106,$B13)</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A13,'Test Cases'!$C$2:$C$109,$B13)</f>
         <v>8</v>
       </c>
       <c r="D13" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A13,'Test Cases'!$C$2:$C$106,$B13,'Test Cases'!$J$2:$J$106,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A13,'Test Cases'!$C$2:$C$109,$B13,'Test Cases'!$J$2:$J$109,"Pass")</f>
         <v>6</v>
       </c>
       <c r="E13" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A13,'Test Cases'!$C$2:$C$106,$B13,'Test Cases'!$J$2:$J$106,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A13,'Test Cases'!$C$2:$C$109,$B13,'Test Cases'!$J$2:$J$109,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F13" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A13,'Test Cases'!$C$2:$C$106,$B13,'Test Cases'!$J$2:$J$106,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A13,'Test Cases'!$C$2:$C$109,$B13,'Test Cases'!$J$2:$J$109,"Manual (UAT)")</f>
         <v>2</v>
       </c>
       <c r="G13" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A13,'Test Cases'!$C$2:$C$106,$B13,'Test Cases'!$L$2:$L$106,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A13,'Test Cases'!$C$2:$C$109,$B13,'Test Cases'!$L$2:$L$109,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H13" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A13,'Test Cases'!$C$2:$C$106,$B13,'Test Cases'!$L$2:$L$106,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A13,'Test Cases'!$C$2:$C$109,$B13,'Test Cases'!$L$2:$L$109,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I13" s="6" t="n">
@@ -2556,27 +2572,27 @@
         <v>24</v>
       </c>
       <c r="C14" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A14,'Test Cases'!$C$2:$C$106,$B14)</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A14,'Test Cases'!$C$2:$C$109,$B14)</f>
         <v>4</v>
       </c>
       <c r="D14" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A14,'Test Cases'!$C$2:$C$106,$B14,'Test Cases'!$J$2:$J$106,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A14,'Test Cases'!$C$2:$C$109,$B14,'Test Cases'!$J$2:$J$109,"Pass")</f>
         <v>4</v>
       </c>
       <c r="E14" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A14,'Test Cases'!$C$2:$C$106,$B14,'Test Cases'!$J$2:$J$106,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A14,'Test Cases'!$C$2:$C$109,$B14,'Test Cases'!$J$2:$J$109,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F14" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A14,'Test Cases'!$C$2:$C$106,$B14,'Test Cases'!$J$2:$J$106,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A14,'Test Cases'!$C$2:$C$109,$B14,'Test Cases'!$J$2:$J$109,"Manual (UAT)")</f>
         <v>0</v>
       </c>
       <c r="G14" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A14,'Test Cases'!$C$2:$C$106,$B14,'Test Cases'!$L$2:$L$106,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A14,'Test Cases'!$C$2:$C$109,$B14,'Test Cases'!$L$2:$L$109,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H14" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A14,'Test Cases'!$C$2:$C$106,$B14,'Test Cases'!$L$2:$L$106,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A14,'Test Cases'!$C$2:$C$109,$B14,'Test Cases'!$L$2:$L$109,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I14" s="6" t="n">
@@ -2592,27 +2608,27 @@
         <v>25</v>
       </c>
       <c r="C15" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A15,'Test Cases'!$C$2:$C$106,$B15)</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A15,'Test Cases'!$C$2:$C$109,$B15)</f>
         <v>1</v>
       </c>
       <c r="D15" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A15,'Test Cases'!$C$2:$C$106,$B15,'Test Cases'!$J$2:$J$106,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A15,'Test Cases'!$C$2:$C$109,$B15,'Test Cases'!$J$2:$J$109,"Pass")</f>
         <v>1</v>
       </c>
       <c r="E15" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A15,'Test Cases'!$C$2:$C$106,$B15,'Test Cases'!$J$2:$J$106,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A15,'Test Cases'!$C$2:$C$109,$B15,'Test Cases'!$J$2:$J$109,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F15" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A15,'Test Cases'!$C$2:$C$106,$B15,'Test Cases'!$J$2:$J$106,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A15,'Test Cases'!$C$2:$C$109,$B15,'Test Cases'!$J$2:$J$109,"Manual (UAT)")</f>
         <v>0</v>
       </c>
       <c r="G15" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A15,'Test Cases'!$C$2:$C$106,$B15,'Test Cases'!$L$2:$L$106,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A15,'Test Cases'!$C$2:$C$109,$B15,'Test Cases'!$L$2:$L$109,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H15" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A15,'Test Cases'!$C$2:$C$106,$B15,'Test Cases'!$L$2:$L$106,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A15,'Test Cases'!$C$2:$C$109,$B15,'Test Cases'!$L$2:$L$109,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I15" s="6" t="n">
@@ -2628,27 +2644,27 @@
         <v>26</v>
       </c>
       <c r="C16" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A16,'Test Cases'!$C$2:$C$106,$B16)</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A16,'Test Cases'!$C$2:$C$109,$B16)</f>
         <v>5</v>
       </c>
       <c r="D16" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A16,'Test Cases'!$C$2:$C$106,$B16,'Test Cases'!$J$2:$J$106,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A16,'Test Cases'!$C$2:$C$109,$B16,'Test Cases'!$J$2:$J$109,"Pass")</f>
         <v>4</v>
       </c>
       <c r="E16" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A16,'Test Cases'!$C$2:$C$106,$B16,'Test Cases'!$J$2:$J$106,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A16,'Test Cases'!$C$2:$C$109,$B16,'Test Cases'!$J$2:$J$109,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F16" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A16,'Test Cases'!$C$2:$C$106,$B16,'Test Cases'!$J$2:$J$106,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A16,'Test Cases'!$C$2:$C$109,$B16,'Test Cases'!$J$2:$J$109,"Manual (UAT)")</f>
         <v>1</v>
       </c>
       <c r="G16" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A16,'Test Cases'!$C$2:$C$106,$B16,'Test Cases'!$L$2:$L$106,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A16,'Test Cases'!$C$2:$C$109,$B16,'Test Cases'!$L$2:$L$109,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H16" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A16,'Test Cases'!$C$2:$C$106,$B16,'Test Cases'!$L$2:$L$106,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A16,'Test Cases'!$C$2:$C$109,$B16,'Test Cases'!$L$2:$L$109,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I16" s="6" t="n">
@@ -2664,27 +2680,27 @@
         <v>27</v>
       </c>
       <c r="C17" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A17,'Test Cases'!$C$2:$C$106,$B17)</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A17,'Test Cases'!$C$2:$C$109,$B17)</f>
         <v>7</v>
       </c>
       <c r="D17" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A17,'Test Cases'!$C$2:$C$106,$B17,'Test Cases'!$J$2:$J$106,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A17,'Test Cases'!$C$2:$C$109,$B17,'Test Cases'!$J$2:$J$109,"Pass")</f>
         <v>5</v>
       </c>
       <c r="E17" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A17,'Test Cases'!$C$2:$C$106,$B17,'Test Cases'!$J$2:$J$106,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A17,'Test Cases'!$C$2:$C$109,$B17,'Test Cases'!$J$2:$J$109,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F17" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A17,'Test Cases'!$C$2:$C$106,$B17,'Test Cases'!$J$2:$J$106,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A17,'Test Cases'!$C$2:$C$109,$B17,'Test Cases'!$J$2:$J$109,"Manual (UAT)")</f>
         <v>2</v>
       </c>
       <c r="G17" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A17,'Test Cases'!$C$2:$C$106,$B17,'Test Cases'!$L$2:$L$106,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A17,'Test Cases'!$C$2:$C$109,$B17,'Test Cases'!$L$2:$L$109,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H17" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A17,'Test Cases'!$C$2:$C$106,$B17,'Test Cases'!$L$2:$L$106,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A17,'Test Cases'!$C$2:$C$109,$B17,'Test Cases'!$L$2:$L$109,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I17" s="6" t="n">
@@ -2700,27 +2716,27 @@
         <v>28</v>
       </c>
       <c r="C18" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A18,'Test Cases'!$C$2:$C$106,$B18)</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A18,'Test Cases'!$C$2:$C$109,$B18)</f>
         <v>9</v>
       </c>
       <c r="D18" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A18,'Test Cases'!$C$2:$C$106,$B18,'Test Cases'!$J$2:$J$106,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A18,'Test Cases'!$C$2:$C$109,$B18,'Test Cases'!$J$2:$J$109,"Pass")</f>
         <v>7</v>
       </c>
       <c r="E18" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A18,'Test Cases'!$C$2:$C$106,$B18,'Test Cases'!$J$2:$J$106,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A18,'Test Cases'!$C$2:$C$109,$B18,'Test Cases'!$J$2:$J$109,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F18" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A18,'Test Cases'!$C$2:$C$106,$B18,'Test Cases'!$J$2:$J$106,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A18,'Test Cases'!$C$2:$C$109,$B18,'Test Cases'!$J$2:$J$109,"Manual (UAT)")</f>
         <v>2</v>
       </c>
       <c r="G18" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A18,'Test Cases'!$C$2:$C$106,$B18,'Test Cases'!$L$2:$L$106,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A18,'Test Cases'!$C$2:$C$109,$B18,'Test Cases'!$L$2:$L$109,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H18" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A18,'Test Cases'!$C$2:$C$106,$B18,'Test Cases'!$L$2:$L$106,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A18,'Test Cases'!$C$2:$C$109,$B18,'Test Cases'!$L$2:$L$109,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I18" s="6" t="n">
@@ -2736,27 +2752,27 @@
         <v>29</v>
       </c>
       <c r="C19" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A19,'Test Cases'!$C$2:$C$106,$B19)</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A19,'Test Cases'!$C$2:$C$109,$B19)</f>
         <v>11</v>
       </c>
       <c r="D19" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A19,'Test Cases'!$C$2:$C$106,$B19,'Test Cases'!$J$2:$J$106,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A19,'Test Cases'!$C$2:$C$109,$B19,'Test Cases'!$J$2:$J$109,"Pass")</f>
         <v>9</v>
       </c>
       <c r="E19" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A19,'Test Cases'!$C$2:$C$106,$B19,'Test Cases'!$J$2:$J$106,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A19,'Test Cases'!$C$2:$C$109,$B19,'Test Cases'!$J$2:$J$109,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F19" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A19,'Test Cases'!$C$2:$C$106,$B19,'Test Cases'!$J$2:$J$106,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A19,'Test Cases'!$C$2:$C$109,$B19,'Test Cases'!$J$2:$J$109,"Manual (UAT)")</f>
         <v>2</v>
       </c>
       <c r="G19" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A19,'Test Cases'!$C$2:$C$106,$B19,'Test Cases'!$L$2:$L$106,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A19,'Test Cases'!$C$2:$C$109,$B19,'Test Cases'!$L$2:$L$109,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H19" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A19,'Test Cases'!$C$2:$C$106,$B19,'Test Cases'!$L$2:$L$106,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A19,'Test Cases'!$C$2:$C$109,$B19,'Test Cases'!$L$2:$L$109,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I19" s="6" t="n">
@@ -2772,27 +2788,27 @@
         <v>30</v>
       </c>
       <c r="C20" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A20,'Test Cases'!$C$2:$C$106,$B20)</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A20,'Test Cases'!$C$2:$C$109,$B20)</f>
         <v>1</v>
       </c>
       <c r="D20" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A20,'Test Cases'!$C$2:$C$106,$B20,'Test Cases'!$J$2:$J$106,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A20,'Test Cases'!$C$2:$C$109,$B20,'Test Cases'!$J$2:$J$109,"Pass")</f>
         <v>1</v>
       </c>
       <c r="E20" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A20,'Test Cases'!$C$2:$C$106,$B20,'Test Cases'!$J$2:$J$106,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A20,'Test Cases'!$C$2:$C$109,$B20,'Test Cases'!$J$2:$J$109,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F20" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A20,'Test Cases'!$C$2:$C$106,$B20,'Test Cases'!$J$2:$J$106,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A20,'Test Cases'!$C$2:$C$109,$B20,'Test Cases'!$J$2:$J$109,"Manual (UAT)")</f>
         <v>0</v>
       </c>
       <c r="G20" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A20,'Test Cases'!$C$2:$C$106,$B20,'Test Cases'!$L$2:$L$106,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A20,'Test Cases'!$C$2:$C$109,$B20,'Test Cases'!$L$2:$L$109,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H20" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A20,'Test Cases'!$C$2:$C$106,$B20,'Test Cases'!$L$2:$L$106,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A20,'Test Cases'!$C$2:$C$109,$B20,'Test Cases'!$L$2:$L$109,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I20" s="6" t="n">
@@ -2808,27 +2824,27 @@
         <v>31</v>
       </c>
       <c r="C21" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A21,'Test Cases'!$C$2:$C$106,$B21)</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A21,'Test Cases'!$C$2:$C$109,$B21)</f>
         <v>4</v>
       </c>
       <c r="D21" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A21,'Test Cases'!$C$2:$C$106,$B21,'Test Cases'!$J$2:$J$106,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A21,'Test Cases'!$C$2:$C$109,$B21,'Test Cases'!$J$2:$J$109,"Pass")</f>
         <v>2</v>
       </c>
       <c r="E21" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A21,'Test Cases'!$C$2:$C$106,$B21,'Test Cases'!$J$2:$J$106,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A21,'Test Cases'!$C$2:$C$109,$B21,'Test Cases'!$J$2:$J$109,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F21" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A21,'Test Cases'!$C$2:$C$106,$B21,'Test Cases'!$J$2:$J$106,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A21,'Test Cases'!$C$2:$C$109,$B21,'Test Cases'!$J$2:$J$109,"Manual (UAT)")</f>
         <v>2</v>
       </c>
       <c r="G21" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A21,'Test Cases'!$C$2:$C$106,$B21,'Test Cases'!$L$2:$L$106,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A21,'Test Cases'!$C$2:$C$109,$B21,'Test Cases'!$L$2:$L$109,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H21" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A21,'Test Cases'!$C$2:$C$106,$B21,'Test Cases'!$L$2:$L$106,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A21,'Test Cases'!$C$2:$C$109,$B21,'Test Cases'!$L$2:$L$109,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I21" s="6" t="n">
@@ -2844,27 +2860,27 @@
         <v>32</v>
       </c>
       <c r="C22" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A22,'Test Cases'!$C$2:$C$106,$B22)</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A22,'Test Cases'!$C$2:$C$109,$B22)</f>
         <v>3</v>
       </c>
       <c r="D22" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A22,'Test Cases'!$C$2:$C$106,$B22,'Test Cases'!$J$2:$J$106,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A22,'Test Cases'!$C$2:$C$109,$B22,'Test Cases'!$J$2:$J$109,"Pass")</f>
         <v>0</v>
       </c>
       <c r="E22" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A22,'Test Cases'!$C$2:$C$106,$B22,'Test Cases'!$J$2:$J$106,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A22,'Test Cases'!$C$2:$C$109,$B22,'Test Cases'!$J$2:$J$109,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F22" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A22,'Test Cases'!$C$2:$C$106,$B22,'Test Cases'!$J$2:$J$106,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A22,'Test Cases'!$C$2:$C$109,$B22,'Test Cases'!$J$2:$J$109,"Manual (UAT)")</f>
         <v>3</v>
       </c>
       <c r="G22" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A22,'Test Cases'!$C$2:$C$106,$B22,'Test Cases'!$L$2:$L$106,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A22,'Test Cases'!$C$2:$C$109,$B22,'Test Cases'!$L$2:$L$109,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H22" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A22,'Test Cases'!$C$2:$C$106,$B22,'Test Cases'!$L$2:$L$106,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A22,'Test Cases'!$C$2:$C$109,$B22,'Test Cases'!$L$2:$L$109,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I22" s="6" t="n">
@@ -2880,27 +2896,27 @@
         <v>33</v>
       </c>
       <c r="C23" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A23,'Test Cases'!$C$2:$C$106,$B23)</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A23,'Test Cases'!$C$2:$C$109,$B23)</f>
         <v>1</v>
       </c>
       <c r="D23" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A23,'Test Cases'!$C$2:$C$106,$B23,'Test Cases'!$J$2:$J$106,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A23,'Test Cases'!$C$2:$C$109,$B23,'Test Cases'!$J$2:$J$109,"Pass")</f>
         <v>0</v>
       </c>
       <c r="E23" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A23,'Test Cases'!$C$2:$C$106,$B23,'Test Cases'!$J$2:$J$106,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A23,'Test Cases'!$C$2:$C$109,$B23,'Test Cases'!$J$2:$J$109,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F23" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A23,'Test Cases'!$C$2:$C$106,$B23,'Test Cases'!$J$2:$J$106,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A23,'Test Cases'!$C$2:$C$109,$B23,'Test Cases'!$J$2:$J$109,"Manual (UAT)")</f>
         <v>1</v>
       </c>
       <c r="G23" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A23,'Test Cases'!$C$2:$C$106,$B23,'Test Cases'!$L$2:$L$106,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A23,'Test Cases'!$C$2:$C$109,$B23,'Test Cases'!$L$2:$L$109,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H23" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A23,'Test Cases'!$C$2:$C$106,$B23,'Test Cases'!$L$2:$L$106,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A23,'Test Cases'!$C$2:$C$109,$B23,'Test Cases'!$L$2:$L$109,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I23" s="6" t="n">
@@ -2916,27 +2932,27 @@
         <v>34</v>
       </c>
       <c r="C24" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A24,'Test Cases'!$C$2:$C$106,$B24)</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A24,'Test Cases'!$C$2:$C$109,$B24)</f>
         <v>1</v>
       </c>
       <c r="D24" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A24,'Test Cases'!$C$2:$C$106,$B24,'Test Cases'!$J$2:$J$106,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A24,'Test Cases'!$C$2:$C$109,$B24,'Test Cases'!$J$2:$J$109,"Pass")</f>
         <v>0</v>
       </c>
       <c r="E24" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A24,'Test Cases'!$C$2:$C$106,$B24,'Test Cases'!$J$2:$J$106,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A24,'Test Cases'!$C$2:$C$109,$B24,'Test Cases'!$J$2:$J$109,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F24" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A24,'Test Cases'!$C$2:$C$106,$B24,'Test Cases'!$J$2:$J$106,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A24,'Test Cases'!$C$2:$C$109,$B24,'Test Cases'!$J$2:$J$109,"Manual (UAT)")</f>
         <v>1</v>
       </c>
       <c r="G24" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A24,'Test Cases'!$C$2:$C$106,$B24,'Test Cases'!$L$2:$L$106,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A24,'Test Cases'!$C$2:$C$109,$B24,'Test Cases'!$L$2:$L$109,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H24" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A24,'Test Cases'!$C$2:$C$106,$B24,'Test Cases'!$L$2:$L$106,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A24,'Test Cases'!$C$2:$C$109,$B24,'Test Cases'!$L$2:$L$109,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I24" s="6" t="n">
@@ -2952,27 +2968,27 @@
         <v>35</v>
       </c>
       <c r="C25" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A25,'Test Cases'!$C$2:$C$106,$B25)</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A25,'Test Cases'!$C$2:$C$109,$B25)</f>
         <v>1</v>
       </c>
       <c r="D25" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A25,'Test Cases'!$C$2:$C$106,$B25,'Test Cases'!$J$2:$J$106,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A25,'Test Cases'!$C$2:$C$109,$B25,'Test Cases'!$J$2:$J$109,"Pass")</f>
         <v>0</v>
       </c>
       <c r="E25" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A25,'Test Cases'!$C$2:$C$106,$B25,'Test Cases'!$J$2:$J$106,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A25,'Test Cases'!$C$2:$C$109,$B25,'Test Cases'!$J$2:$J$109,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F25" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A25,'Test Cases'!$C$2:$C$106,$B25,'Test Cases'!$J$2:$J$106,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A25,'Test Cases'!$C$2:$C$109,$B25,'Test Cases'!$J$2:$J$109,"Manual (UAT)")</f>
         <v>1</v>
       </c>
       <c r="G25" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A25,'Test Cases'!$C$2:$C$106,$B25,'Test Cases'!$L$2:$L$106,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A25,'Test Cases'!$C$2:$C$109,$B25,'Test Cases'!$L$2:$L$109,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H25" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A25,'Test Cases'!$C$2:$C$106,$B25,'Test Cases'!$L$2:$L$106,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A25,'Test Cases'!$C$2:$C$109,$B25,'Test Cases'!$L$2:$L$109,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I25" s="6" t="n">
@@ -2988,27 +3004,27 @@
         <v>36</v>
       </c>
       <c r="C26" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A26,'Test Cases'!$C$2:$C$106,$B26)</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A26,'Test Cases'!$C$2:$C$109,$B26)</f>
         <v>2</v>
       </c>
       <c r="D26" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A26,'Test Cases'!$C$2:$C$106,$B26,'Test Cases'!$J$2:$J$106,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A26,'Test Cases'!$C$2:$C$109,$B26,'Test Cases'!$J$2:$J$109,"Pass")</f>
         <v>0</v>
       </c>
       <c r="E26" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A26,'Test Cases'!$C$2:$C$106,$B26,'Test Cases'!$J$2:$J$106,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A26,'Test Cases'!$C$2:$C$109,$B26,'Test Cases'!$J$2:$J$109,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F26" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A26,'Test Cases'!$C$2:$C$106,$B26,'Test Cases'!$J$2:$J$106,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A26,'Test Cases'!$C$2:$C$109,$B26,'Test Cases'!$J$2:$J$109,"Manual (UAT)")</f>
         <v>2</v>
       </c>
       <c r="G26" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A26,'Test Cases'!$C$2:$C$106,$B26,'Test Cases'!$L$2:$L$106,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A26,'Test Cases'!$C$2:$C$109,$B26,'Test Cases'!$L$2:$L$109,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H26" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A26,'Test Cases'!$C$2:$C$106,$B26,'Test Cases'!$L$2:$L$106,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A26,'Test Cases'!$C$2:$C$109,$B26,'Test Cases'!$L$2:$L$109,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I26" s="6" t="n">
@@ -3024,27 +3040,27 @@
         <v>37</v>
       </c>
       <c r="C27" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A27,'Test Cases'!$C$2:$C$106,$B27)</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A27,'Test Cases'!$C$2:$C$109,$B27)</f>
         <v>1</v>
       </c>
       <c r="D27" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A27,'Test Cases'!$C$2:$C$106,$B27,'Test Cases'!$J$2:$J$106,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A27,'Test Cases'!$C$2:$C$109,$B27,'Test Cases'!$J$2:$J$109,"Pass")</f>
         <v>0</v>
       </c>
       <c r="E27" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A27,'Test Cases'!$C$2:$C$106,$B27,'Test Cases'!$J$2:$J$106,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A27,'Test Cases'!$C$2:$C$109,$B27,'Test Cases'!$J$2:$J$109,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F27" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A27,'Test Cases'!$C$2:$C$106,$B27,'Test Cases'!$J$2:$J$106,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A27,'Test Cases'!$C$2:$C$109,$B27,'Test Cases'!$J$2:$J$109,"Manual (UAT)")</f>
         <v>1</v>
       </c>
       <c r="G27" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A27,'Test Cases'!$C$2:$C$106,$B27,'Test Cases'!$L$2:$L$106,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A27,'Test Cases'!$C$2:$C$109,$B27,'Test Cases'!$L$2:$L$109,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H27" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A27,'Test Cases'!$C$2:$C$106,$B27,'Test Cases'!$L$2:$L$106,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A27,'Test Cases'!$C$2:$C$109,$B27,'Test Cases'!$L$2:$L$109,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I27" s="6" t="n">
@@ -3094,32 +3110,32 @@
         <v>40</v>
       </c>
       <c r="C29" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A29,'Test Cases'!$C$2:$C$106,$B29)</f>
-        <v>18</v>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A29,'Test Cases'!$C$2:$C$109,$B29)</f>
+        <v>21</v>
       </c>
       <c r="D29" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A29,'Test Cases'!$C$2:$C$106,$B29,'Test Cases'!$J$2:$J$106,"Pass")</f>
-        <v>14</v>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A29,'Test Cases'!$C$2:$C$109,$B29,'Test Cases'!$J$2:$J$109,"Pass")</f>
+        <v>17</v>
       </c>
       <c r="E29" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A29,'Test Cases'!$C$2:$C$106,$B29,'Test Cases'!$J$2:$J$106,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A29,'Test Cases'!$C$2:$C$109,$B29,'Test Cases'!$J$2:$J$109,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F29" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A29,'Test Cases'!$C$2:$C$106,$B29,'Test Cases'!$J$2:$J$106,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A29,'Test Cases'!$C$2:$C$109,$B29,'Test Cases'!$J$2:$J$109,"Manual (UAT)")</f>
         <v>4</v>
       </c>
       <c r="G29" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A29,'Test Cases'!$C$2:$C$106,$B29,'Test Cases'!$L$2:$L$106,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A29,'Test Cases'!$C$2:$C$109,$B29,'Test Cases'!$L$2:$L$109,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H29" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A29,'Test Cases'!$C$2:$C$106,$B29,'Test Cases'!$L$2:$L$106,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A29,'Test Cases'!$C$2:$C$109,$B29,'Test Cases'!$L$2:$L$109,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I29" s="6" t="n">
         <f aca="false">C29-G29-H29</f>
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3130,27 +3146,27 @@
         <v>41</v>
       </c>
       <c r="C30" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A30,'Test Cases'!$C$2:$C$106,$B30)</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A30,'Test Cases'!$C$2:$C$109,$B30)</f>
         <v>10</v>
       </c>
       <c r="D30" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A30,'Test Cases'!$C$2:$C$106,$B30,'Test Cases'!$J$2:$J$106,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A30,'Test Cases'!$C$2:$C$109,$B30,'Test Cases'!$J$2:$J$109,"Pass")</f>
         <v>10</v>
       </c>
       <c r="E30" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A30,'Test Cases'!$C$2:$C$106,$B30,'Test Cases'!$J$2:$J$106,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A30,'Test Cases'!$C$2:$C$109,$B30,'Test Cases'!$J$2:$J$109,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F30" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A30,'Test Cases'!$C$2:$C$106,$B30,'Test Cases'!$J$2:$J$106,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A30,'Test Cases'!$C$2:$C$109,$B30,'Test Cases'!$J$2:$J$109,"Manual (UAT)")</f>
         <v>0</v>
       </c>
       <c r="G30" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A30,'Test Cases'!$C$2:$C$106,$B30,'Test Cases'!$L$2:$L$106,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A30,'Test Cases'!$C$2:$C$109,$B30,'Test Cases'!$L$2:$L$109,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H30" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A30,'Test Cases'!$C$2:$C$106,$B30,'Test Cases'!$L$2:$L$106,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A30,'Test Cases'!$C$2:$C$109,$B30,'Test Cases'!$L$2:$L$109,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I30" s="6" t="n">
@@ -3166,27 +3182,27 @@
         <v>42</v>
       </c>
       <c r="C31" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A31,'Test Cases'!$C$2:$C$106,$B31)</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A31,'Test Cases'!$C$2:$C$109,$B31)</f>
         <v>2</v>
       </c>
       <c r="D31" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A31,'Test Cases'!$C$2:$C$106,$B31,'Test Cases'!$J$2:$J$106,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A31,'Test Cases'!$C$2:$C$109,$B31,'Test Cases'!$J$2:$J$109,"Pass")</f>
         <v>2</v>
       </c>
       <c r="E31" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A31,'Test Cases'!$C$2:$C$106,$B31,'Test Cases'!$J$2:$J$106,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A31,'Test Cases'!$C$2:$C$109,$B31,'Test Cases'!$J$2:$J$109,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F31" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A31,'Test Cases'!$C$2:$C$106,$B31,'Test Cases'!$J$2:$J$106,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A31,'Test Cases'!$C$2:$C$109,$B31,'Test Cases'!$J$2:$J$109,"Manual (UAT)")</f>
         <v>0</v>
       </c>
       <c r="G31" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A31,'Test Cases'!$C$2:$C$106,$B31,'Test Cases'!$L$2:$L$106,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A31,'Test Cases'!$C$2:$C$109,$B31,'Test Cases'!$L$2:$L$109,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H31" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A31,'Test Cases'!$C$2:$C$106,$B31,'Test Cases'!$L$2:$L$106,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A31,'Test Cases'!$C$2:$C$109,$B31,'Test Cases'!$L$2:$L$109,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I31" s="6" t="n">
@@ -3202,27 +3218,27 @@
         <v>43</v>
       </c>
       <c r="C32" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A32,'Test Cases'!$C$2:$C$106,$B32)</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A32,'Test Cases'!$C$2:$C$109,$B32)</f>
         <v>1</v>
       </c>
       <c r="D32" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A32,'Test Cases'!$C$2:$C$106,$B32,'Test Cases'!$J$2:$J$106,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A32,'Test Cases'!$C$2:$C$109,$B32,'Test Cases'!$J$2:$J$109,"Pass")</f>
         <v>0</v>
       </c>
       <c r="E32" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A32,'Test Cases'!$C$2:$C$106,$B32,'Test Cases'!$J$2:$J$106,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A32,'Test Cases'!$C$2:$C$109,$B32,'Test Cases'!$J$2:$J$109,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F32" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A32,'Test Cases'!$C$2:$C$106,$B32,'Test Cases'!$J$2:$J$106,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A32,'Test Cases'!$C$2:$C$109,$B32,'Test Cases'!$J$2:$J$109,"Manual (UAT)")</f>
         <v>1</v>
       </c>
       <c r="G32" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A32,'Test Cases'!$C$2:$C$106,$B32,'Test Cases'!$L$2:$L$106,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A32,'Test Cases'!$C$2:$C$109,$B32,'Test Cases'!$L$2:$L$109,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H32" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$106,$A32,'Test Cases'!$C$2:$C$106,$B32,'Test Cases'!$L$2:$L$106,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$109,$A32,'Test Cases'!$C$2:$C$109,$B32,'Test Cases'!$L$2:$L$109,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I32" s="6" t="n">
@@ -3237,11 +3253,11 @@
       <c r="B33" s="7"/>
       <c r="C33" s="8" t="n">
         <f aca="false">SUM(C29:C32)</f>
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="D33" s="8" t="n">
         <f aca="false">SUM(D29:D32)</f>
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E33" s="8" t="n">
         <f aca="false">SUM(E29:E32)</f>
@@ -3261,7 +3277,7 @@
       </c>
       <c r="I33" s="8" t="n">
         <f aca="false">SUM(I29:I32)</f>
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3271,11 +3287,11 @@
       <c r="B34" s="9"/>
       <c r="C34" s="10" t="n">
         <f aca="false">C11+C12+C13+C14+C15+C16+C17+C18+C19+C20+C21+C22+C23+C24+C25+C26+C27+C29+C30+C31+C32</f>
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="D34" s="10" t="n">
         <f aca="false">D11+D12+D13+D14+D15+D16+D17+D18+D19+D20+D21+D22+D23+D24+D25+D26+D27+D29+D30+D31+D32</f>
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="E34" s="10" t="n">
         <f aca="false">E11+E12+E13+E14+E15+E16+E17+E18+E19+E20+E21+E22+E23+E24+E25+E26+E27+E29+E30+E31+E32</f>
@@ -3295,7 +3311,7 @@
       </c>
       <c r="I34" s="10" t="n">
         <f aca="false">I11+I12+I13+I14+I15+I16+I17+I18+I19+I20+I21+I22+I23+I24+I25+I26+I27+I29+I30+I31+I32</f>
-        <v>105</v>
+        <v>108</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3362,7 +3378,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O106"/>
+  <dimension ref="A1:O109"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -5340,7 +5356,7 @@
       <c r="N50" s="15"/>
       <c r="O50" s="15"/>
     </row>
-    <row r="51" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="51" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="14" t="s">
         <v>264</v>
       </c>
@@ -5379,7 +5395,7 @@
       <c r="N51" s="15"/>
       <c r="O51" s="15"/>
     </row>
-    <row r="52" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="14" t="s">
         <v>269</v>
       </c>
@@ -5418,7 +5434,7 @@
       <c r="N52" s="15"/>
       <c r="O52" s="15"/>
     </row>
-    <row r="53" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="14" t="s">
         <v>273</v>
       </c>
@@ -5457,7 +5473,7 @@
       <c r="N53" s="15"/>
       <c r="O53" s="15"/>
     </row>
-    <row r="54" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="54" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="14" t="s">
         <v>277</v>
       </c>
@@ -5496,7 +5512,7 @@
       <c r="N54" s="15"/>
       <c r="O54" s="15"/>
     </row>
-    <row r="55" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="55" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="14" t="s">
         <v>281</v>
       </c>
@@ -5522,7 +5538,7 @@
         <v>72</v>
       </c>
       <c r="I55" s="14" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="J55" s="14" t="s">
         <v>74</v>
@@ -5535,7 +5551,7 @@
       <c r="N55" s="15"/>
       <c r="O55" s="15"/>
     </row>
-    <row r="56" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="56" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="14" t="s">
         <v>285</v>
       </c>
@@ -5561,7 +5577,7 @@
         <v>72</v>
       </c>
       <c r="I56" s="14" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="J56" s="14" t="s">
         <v>74</v>
@@ -5574,7 +5590,7 @@
       <c r="N56" s="15"/>
       <c r="O56" s="15"/>
     </row>
-    <row r="57" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="57" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="14" t="s">
         <v>289</v>
       </c>
@@ -5582,25 +5598,25 @@
         <v>39</v>
       </c>
       <c r="C57" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D57" s="14" t="s">
         <v>290</v>
       </c>
       <c r="E57" s="14" t="s">
+        <v>266</v>
+      </c>
+      <c r="F57" s="14" t="s">
         <v>291</v>
       </c>
-      <c r="F57" s="14" t="s">
+      <c r="G57" s="14" t="s">
         <v>292</v>
-      </c>
-      <c r="G57" s="14" t="s">
-        <v>293</v>
       </c>
       <c r="H57" s="14" t="s">
         <v>72</v>
       </c>
       <c r="I57" s="14" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="J57" s="14" t="s">
         <v>74</v>
@@ -5613,33 +5629,33 @@
       <c r="N57" s="15"/>
       <c r="O57" s="15"/>
     </row>
-    <row r="58" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="58" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="14" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B58" s="14" t="s">
         <v>39</v>
       </c>
       <c r="C58" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D58" s="14" t="s">
+        <v>294</v>
+      </c>
+      <c r="E58" s="14" t="s">
+        <v>266</v>
+      </c>
+      <c r="F58" s="14" t="s">
         <v>295</v>
       </c>
-      <c r="E58" s="14" t="s">
-        <v>291</v>
-      </c>
-      <c r="F58" s="14" t="s">
+      <c r="G58" s="14" t="s">
         <v>296</v>
-      </c>
-      <c r="G58" s="14" t="s">
-        <v>297</v>
       </c>
       <c r="H58" s="14" t="s">
         <v>72</v>
       </c>
       <c r="I58" s="14" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="J58" s="14" t="s">
         <v>74</v>
@@ -5652,9 +5668,9 @@
       <c r="N58" s="15"/>
       <c r="O58" s="15"/>
     </row>
-    <row r="59" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="14" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B59" s="14" t="s">
         <v>39</v>
@@ -5663,22 +5679,22 @@
         <v>41</v>
       </c>
       <c r="D59" s="14" t="s">
+        <v>298</v>
+      </c>
+      <c r="E59" s="14" t="s">
         <v>299</v>
-      </c>
-      <c r="E59" s="14" t="s">
-        <v>291</v>
       </c>
       <c r="F59" s="14" t="s">
         <v>300</v>
       </c>
       <c r="G59" s="14" t="s">
-        <v>263</v>
+        <v>301</v>
       </c>
       <c r="H59" s="14" t="s">
         <v>72</v>
       </c>
       <c r="I59" s="14" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="J59" s="14" t="s">
         <v>74</v>
@@ -5693,7 +5709,7 @@
     </row>
     <row r="60" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="14" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B60" s="14" t="s">
         <v>39</v>
@@ -5702,16 +5718,16 @@
         <v>41</v>
       </c>
       <c r="D60" s="14" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="E60" s="14" t="s">
-        <v>291</v>
+        <v>299</v>
       </c>
       <c r="F60" s="14" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="G60" s="14" t="s">
-        <v>263</v>
+        <v>305</v>
       </c>
       <c r="H60" s="14" t="s">
         <v>72</v>
@@ -5732,7 +5748,7 @@
     </row>
     <row r="61" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="14" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="B61" s="14" t="s">
         <v>39</v>
@@ -5741,13 +5757,13 @@
         <v>41</v>
       </c>
       <c r="D61" s="14" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="E61" s="14" t="s">
-        <v>291</v>
+        <v>299</v>
       </c>
       <c r="F61" s="14" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="G61" s="14" t="s">
         <v>263</v>
@@ -5769,9 +5785,9 @@
       <c r="N61" s="15"/>
       <c r="O61" s="15"/>
     </row>
-    <row r="62" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="62" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="14" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B62" s="14" t="s">
         <v>39</v>
@@ -5780,22 +5796,22 @@
         <v>41</v>
       </c>
       <c r="D62" s="14" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="E62" s="14" t="s">
-        <v>291</v>
+        <v>299</v>
       </c>
       <c r="F62" s="14" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="G62" s="14" t="s">
-        <v>310</v>
+        <v>263</v>
       </c>
       <c r="H62" s="14" t="s">
         <v>72</v>
       </c>
       <c r="I62" s="14" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="J62" s="14" t="s">
         <v>74</v>
@@ -5810,7 +5826,7 @@
     </row>
     <row r="63" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="14" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B63" s="14" t="s">
         <v>39</v>
@@ -5819,22 +5835,22 @@
         <v>41</v>
       </c>
       <c r="D63" s="14" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E63" s="14" t="s">
-        <v>291</v>
+        <v>299</v>
       </c>
       <c r="F63" s="14" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="G63" s="14" t="s">
-        <v>314</v>
+        <v>263</v>
       </c>
       <c r="H63" s="14" t="s">
         <v>72</v>
       </c>
       <c r="I63" s="14" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="J63" s="14" t="s">
         <v>74</v>
@@ -5847,7 +5863,7 @@
       <c r="N63" s="15"/>
       <c r="O63" s="15"/>
     </row>
-    <row r="64" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="64" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="14" t="s">
         <v>315</v>
       </c>
@@ -5861,19 +5877,19 @@
         <v>316</v>
       </c>
       <c r="E64" s="14" t="s">
-        <v>291</v>
+        <v>299</v>
       </c>
       <c r="F64" s="14" t="s">
         <v>317</v>
       </c>
       <c r="G64" s="14" t="s">
-        <v>263</v>
+        <v>318</v>
       </c>
       <c r="H64" s="14" t="s">
         <v>72</v>
       </c>
       <c r="I64" s="14" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="J64" s="14" t="s">
         <v>74</v>
@@ -5888,7 +5904,7 @@
     </row>
     <row r="65" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="14" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B65" s="14" t="s">
         <v>39</v>
@@ -5897,16 +5913,16 @@
         <v>41</v>
       </c>
       <c r="D65" s="14" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="E65" s="14" t="s">
-        <v>291</v>
+        <v>299</v>
       </c>
       <c r="F65" s="14" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G65" s="14" t="s">
-        <v>293</v>
+        <v>322</v>
       </c>
       <c r="H65" s="14" t="s">
         <v>72</v>
@@ -5925,33 +5941,33 @@
       <c r="N65" s="15"/>
       <c r="O65" s="15"/>
     </row>
-    <row r="66" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="66" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="14" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B66" s="14" t="s">
         <v>39</v>
       </c>
       <c r="C66" s="14" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D66" s="14" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="E66" s="14" t="s">
-        <v>266</v>
+        <v>299</v>
       </c>
       <c r="F66" s="14" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="G66" s="14" t="s">
-        <v>324</v>
+        <v>263</v>
       </c>
       <c r="H66" s="14" t="s">
         <v>72</v>
       </c>
       <c r="I66" s="14" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="J66" s="14" t="s">
         <v>74</v>
@@ -5964,27 +5980,27 @@
       <c r="N66" s="15"/>
       <c r="O66" s="15"/>
     </row>
-    <row r="67" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="67" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="14" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B67" s="14" t="s">
         <v>39</v>
       </c>
       <c r="C67" s="14" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D67" s="14" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E67" s="14" t="s">
-        <v>266</v>
+        <v>299</v>
       </c>
       <c r="F67" s="14" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="G67" s="14" t="s">
-        <v>328</v>
+        <v>301</v>
       </c>
       <c r="H67" s="14" t="s">
         <v>72</v>
@@ -6003,7 +6019,7 @@
       <c r="N67" s="15"/>
       <c r="O67" s="15"/>
     </row>
-    <row r="68" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="68" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="14" t="s">
         <v>329</v>
       </c>
@@ -6042,7 +6058,7 @@
       <c r="N68" s="15"/>
       <c r="O68" s="15"/>
     </row>
-    <row r="69" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="69" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="14" t="s">
         <v>333</v>
       </c>
@@ -6068,7 +6084,7 @@
         <v>72</v>
       </c>
       <c r="I69" s="14" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="J69" s="14" t="s">
         <v>74</v>
@@ -6081,7 +6097,7 @@
       <c r="N69" s="15"/>
       <c r="O69" s="15"/>
     </row>
-    <row r="70" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="70" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="14" t="s">
         <v>337</v>
       </c>
@@ -6107,7 +6123,7 @@
         <v>72</v>
       </c>
       <c r="I70" s="14" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="J70" s="14" t="s">
         <v>74</v>
@@ -6120,7 +6136,7 @@
       <c r="N70" s="15"/>
       <c r="O70" s="15"/>
     </row>
-    <row r="71" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="71" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="14" t="s">
         <v>341</v>
       </c>
@@ -6159,7 +6175,7 @@
       <c r="N71" s="15"/>
       <c r="O71" s="15"/>
     </row>
-    <row r="72" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="72" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="14" t="s">
         <v>345</v>
       </c>
@@ -6198,7 +6214,7 @@
       <c r="N72" s="15"/>
       <c r="O72" s="15"/>
     </row>
-    <row r="73" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="73" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="14" t="s">
         <v>349</v>
       </c>
@@ -6206,25 +6222,25 @@
         <v>39</v>
       </c>
       <c r="C73" s="14" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D73" s="14" t="s">
         <v>350</v>
       </c>
       <c r="E73" s="14" t="s">
+        <v>266</v>
+      </c>
+      <c r="F73" s="14" t="s">
         <v>351</v>
       </c>
-      <c r="F73" s="14" t="s">
+      <c r="G73" s="14" t="s">
         <v>352</v>
-      </c>
-      <c r="G73" s="14" t="s">
-        <v>353</v>
       </c>
       <c r="H73" s="14" t="s">
         <v>72</v>
       </c>
       <c r="I73" s="14" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="J73" s="14" t="s">
         <v>74</v>
@@ -6237,27 +6253,27 @@
       <c r="N73" s="15"/>
       <c r="O73" s="15"/>
     </row>
-    <row r="74" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="74" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="14" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="B74" s="14" t="s">
         <v>39</v>
       </c>
       <c r="C74" s="14" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D74" s="14" t="s">
+        <v>354</v>
+      </c>
+      <c r="E74" s="14" t="s">
+        <v>266</v>
+      </c>
+      <c r="F74" s="14" t="s">
         <v>355</v>
       </c>
-      <c r="E74" s="14" t="s">
-        <v>351</v>
-      </c>
-      <c r="F74" s="14" t="s">
+      <c r="G74" s="14" t="s">
         <v>356</v>
-      </c>
-      <c r="G74" s="14" t="s">
-        <v>357</v>
       </c>
       <c r="H74" s="14" t="s">
         <v>72</v>
@@ -6276,39 +6292,39 @@
       <c r="N74" s="15"/>
       <c r="O74" s="15"/>
     </row>
-    <row r="75" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="75" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="14" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="B75" s="14" t="s">
         <v>39</v>
       </c>
       <c r="C75" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D75" s="14" t="s">
+        <v>358</v>
+      </c>
+      <c r="E75" s="14" t="s">
+        <v>266</v>
+      </c>
+      <c r="F75" s="14" t="s">
         <v>359</v>
       </c>
-      <c r="E75" s="14" t="s">
+      <c r="G75" s="14" t="s">
         <v>360</v>
-      </c>
-      <c r="F75" s="14" t="s">
-        <v>361</v>
-      </c>
-      <c r="G75" s="14" t="s">
-        <v>362</v>
       </c>
       <c r="H75" s="14" t="s">
         <v>72</v>
       </c>
       <c r="I75" s="14" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="J75" s="14" t="s">
         <v>74</v>
       </c>
       <c r="K75" s="14" t="s">
-        <v>363</v>
+        <v>75</v>
       </c>
       <c r="L75" s="15"/>
       <c r="M75" s="15"/>
@@ -6317,25 +6333,25 @@
     </row>
     <row r="76" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="14" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="B76" s="14" t="s">
         <v>39</v>
       </c>
       <c r="C76" s="14" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D76" s="14" t="s">
+        <v>362</v>
+      </c>
+      <c r="E76" s="14" t="s">
+        <v>363</v>
+      </c>
+      <c r="F76" s="14" t="s">
+        <v>364</v>
+      </c>
+      <c r="G76" s="14" t="s">
         <v>365</v>
-      </c>
-      <c r="E76" s="14" t="s">
-        <v>360</v>
-      </c>
-      <c r="F76" s="14" t="s">
-        <v>366</v>
-      </c>
-      <c r="G76" s="14" t="s">
-        <v>367</v>
       </c>
       <c r="H76" s="14" t="s">
         <v>72</v>
@@ -6347,119 +6363,125 @@
         <v>74</v>
       </c>
       <c r="K76" s="14" t="s">
-        <v>368</v>
+        <v>75</v>
       </c>
       <c r="L76" s="15"/>
       <c r="M76" s="15"/>
       <c r="N76" s="15"/>
       <c r="O76" s="15"/>
     </row>
-    <row r="77" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="77" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="14" t="s">
+        <v>366</v>
+      </c>
+      <c r="B77" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="C77" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="D77" s="14" t="s">
+        <v>367</v>
+      </c>
+      <c r="E77" s="14" t="s">
+        <v>363</v>
+      </c>
+      <c r="F77" s="14" t="s">
+        <v>368</v>
+      </c>
+      <c r="G77" s="14" t="s">
         <v>369</v>
-      </c>
-      <c r="B77" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="C77" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="D77" s="14" t="s">
-        <v>370</v>
-      </c>
-      <c r="E77" s="14" t="s">
-        <v>371</v>
-      </c>
-      <c r="F77" s="14" t="s">
-        <v>372</v>
-      </c>
-      <c r="G77" s="14" t="s">
-        <v>373</v>
       </c>
       <c r="H77" s="14" t="s">
         <v>72</v>
       </c>
       <c r="I77" s="14" t="s">
-        <v>374</v>
+        <v>73</v>
       </c>
       <c r="J77" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="K77" s="14"/>
+        <v>74</v>
+      </c>
+      <c r="K77" s="14" t="s">
+        <v>75</v>
+      </c>
       <c r="L77" s="15"/>
       <c r="M77" s="15"/>
       <c r="N77" s="15"/>
       <c r="O77" s="15"/>
     </row>
-    <row r="78" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="78" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="14" t="s">
-        <v>375</v>
+        <v>370</v>
       </c>
       <c r="B78" s="14" t="s">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="C78" s="14" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="D78" s="14" t="s">
-        <v>376</v>
+        <v>371</v>
       </c>
       <c r="E78" s="14" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="F78" s="14" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="G78" s="14" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
       <c r="H78" s="14" t="s">
         <v>72</v>
       </c>
       <c r="I78" s="14" t="s">
-        <v>374</v>
+        <v>73</v>
       </c>
       <c r="J78" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="K78" s="14"/>
+        <v>74</v>
+      </c>
+      <c r="K78" s="14" t="s">
+        <v>375</v>
+      </c>
       <c r="L78" s="15"/>
       <c r="M78" s="15"/>
       <c r="N78" s="15"/>
       <c r="O78" s="15"/>
     </row>
-    <row r="79" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="79" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="14" t="s">
+        <v>376</v>
+      </c>
+      <c r="B79" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="C79" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="D79" s="14" t="s">
+        <v>377</v>
+      </c>
+      <c r="E79" s="14" t="s">
+        <v>372</v>
+      </c>
+      <c r="F79" s="14" t="s">
+        <v>378</v>
+      </c>
+      <c r="G79" s="14" t="s">
         <v>379</v>
-      </c>
-      <c r="B79" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="C79" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="D79" s="14" t="s">
-        <v>380</v>
-      </c>
-      <c r="E79" s="14" t="s">
-        <v>371</v>
-      </c>
-      <c r="F79" s="14" t="s">
-        <v>381</v>
-      </c>
-      <c r="G79" s="14" t="s">
-        <v>382</v>
       </c>
       <c r="H79" s="14" t="s">
         <v>72</v>
       </c>
       <c r="I79" s="14" t="s">
-        <v>374</v>
+        <v>73</v>
       </c>
       <c r="J79" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="K79" s="14"/>
+        <v>74</v>
+      </c>
+      <c r="K79" s="14" t="s">
+        <v>380</v>
+      </c>
       <c r="L79" s="15"/>
       <c r="M79" s="15"/>
       <c r="N79" s="15"/>
@@ -6467,31 +6489,31 @@
     </row>
     <row r="80" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="14" t="s">
+        <v>381</v>
+      </c>
+      <c r="B80" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="C80" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="D80" s="14" t="s">
+        <v>382</v>
+      </c>
+      <c r="E80" s="14" t="s">
         <v>383</v>
       </c>
-      <c r="B80" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="C80" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="D80" s="14" t="s">
+      <c r="F80" s="14" t="s">
         <v>384</v>
       </c>
-      <c r="E80" s="14" t="s">
-        <v>371</v>
-      </c>
-      <c r="F80" s="14" t="s">
+      <c r="G80" s="14" t="s">
         <v>385</v>
       </c>
-      <c r="G80" s="14" t="s">
+      <c r="H80" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="I80" s="14" t="s">
         <v>386</v>
-      </c>
-      <c r="H80" s="14" t="s">
-        <v>158</v>
-      </c>
-      <c r="I80" s="14" t="s">
-        <v>374</v>
       </c>
       <c r="J80" s="14" t="s">
         <v>16</v>
@@ -6510,13 +6532,13 @@
         <v>20</v>
       </c>
       <c r="C81" s="14" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="D81" s="14" t="s">
         <v>388</v>
       </c>
       <c r="E81" s="14" t="s">
-        <v>371</v>
+        <v>383</v>
       </c>
       <c r="F81" s="14" t="s">
         <v>389</v>
@@ -6525,10 +6547,10 @@
         <v>390</v>
       </c>
       <c r="H81" s="14" t="s">
-        <v>158</v>
+        <v>72</v>
       </c>
       <c r="I81" s="14" t="s">
-        <v>374</v>
+        <v>386</v>
       </c>
       <c r="J81" s="14" t="s">
         <v>16</v>
@@ -6547,13 +6569,13 @@
         <v>20</v>
       </c>
       <c r="C82" s="14" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="D82" s="14" t="s">
         <v>392</v>
       </c>
       <c r="E82" s="14" t="s">
-        <v>371</v>
+        <v>383</v>
       </c>
       <c r="F82" s="14" t="s">
         <v>393</v>
@@ -6562,10 +6584,10 @@
         <v>394</v>
       </c>
       <c r="H82" s="14" t="s">
-        <v>158</v>
+        <v>72</v>
       </c>
       <c r="I82" s="14" t="s">
-        <v>374</v>
+        <v>386</v>
       </c>
       <c r="J82" s="14" t="s">
         <v>16</v>
@@ -6590,7 +6612,7 @@
         <v>396</v>
       </c>
       <c r="E83" s="14" t="s">
-        <v>371</v>
+        <v>383</v>
       </c>
       <c r="F83" s="14" t="s">
         <v>397</v>
@@ -6599,10 +6621,10 @@
         <v>398</v>
       </c>
       <c r="H83" s="14" t="s">
-        <v>72</v>
+        <v>158</v>
       </c>
       <c r="I83" s="14" t="s">
-        <v>399</v>
+        <v>386</v>
       </c>
       <c r="J83" s="14" t="s">
         <v>16</v>
@@ -6615,7 +6637,7 @@
     </row>
     <row r="84" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="14" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="B84" s="14" t="s">
         <v>20</v>
@@ -6624,22 +6646,22 @@
         <v>21</v>
       </c>
       <c r="D84" s="14" t="s">
+        <v>400</v>
+      </c>
+      <c r="E84" s="14" t="s">
+        <v>383</v>
+      </c>
+      <c r="F84" s="14" t="s">
         <v>401</v>
       </c>
-      <c r="E84" s="14" t="s">
-        <v>371</v>
-      </c>
-      <c r="F84" s="14" t="s">
+      <c r="G84" s="14" t="s">
         <v>402</v>
       </c>
-      <c r="G84" s="14" t="s">
-        <v>403</v>
-      </c>
       <c r="H84" s="14" t="s">
-        <v>72</v>
+        <v>158</v>
       </c>
       <c r="I84" s="14" t="s">
-        <v>404</v>
+        <v>386</v>
       </c>
       <c r="J84" s="14" t="s">
         <v>16</v>
@@ -6652,31 +6674,31 @@
     </row>
     <row r="85" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="14" t="s">
+        <v>403</v>
+      </c>
+      <c r="B85" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="C85" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="D85" s="14" t="s">
+        <v>404</v>
+      </c>
+      <c r="E85" s="14" t="s">
+        <v>383</v>
+      </c>
+      <c r="F85" s="14" t="s">
         <v>405</v>
       </c>
-      <c r="B85" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="C85" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="D85" s="14" t="s">
+      <c r="G85" s="14" t="s">
         <v>406</v>
-      </c>
-      <c r="E85" s="14" t="s">
-        <v>371</v>
-      </c>
-      <c r="F85" s="14" t="s">
-        <v>407</v>
-      </c>
-      <c r="G85" s="14" t="s">
-        <v>408</v>
       </c>
       <c r="H85" s="14" t="s">
         <v>158</v>
       </c>
       <c r="I85" s="14" t="s">
-        <v>374</v>
+        <v>386</v>
       </c>
       <c r="J85" s="14" t="s">
         <v>16</v>
@@ -6689,31 +6711,31 @@
     </row>
     <row r="86" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="14" t="s">
+        <v>407</v>
+      </c>
+      <c r="B86" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="C86" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="D86" s="14" t="s">
+        <v>408</v>
+      </c>
+      <c r="E86" s="14" t="s">
+        <v>383</v>
+      </c>
+      <c r="F86" s="14" t="s">
         <v>409</v>
       </c>
-      <c r="B86" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="C86" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="D86" s="14" t="s">
+      <c r="G86" s="14" t="s">
         <v>410</v>
       </c>
-      <c r="E86" s="14" t="s">
-        <v>371</v>
-      </c>
-      <c r="F86" s="14" t="s">
+      <c r="H86" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="I86" s="14" t="s">
         <v>411</v>
-      </c>
-      <c r="G86" s="14" t="s">
-        <v>412</v>
-      </c>
-      <c r="H86" s="14" t="s">
-        <v>158</v>
-      </c>
-      <c r="I86" s="14" t="s">
-        <v>374</v>
       </c>
       <c r="J86" s="14" t="s">
         <v>16</v>
@@ -6726,31 +6748,31 @@
     </row>
     <row r="87" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="14" t="s">
+        <v>412</v>
+      </c>
+      <c r="B87" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="C87" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="D87" s="14" t="s">
         <v>413</v>
       </c>
-      <c r="B87" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="C87" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="D87" s="14" t="s">
+      <c r="E87" s="14" t="s">
+        <v>383</v>
+      </c>
+      <c r="F87" s="14" t="s">
         <v>414</v>
       </c>
-      <c r="E87" s="14" t="s">
-        <v>371</v>
-      </c>
-      <c r="F87" s="14" t="s">
+      <c r="G87" s="14" t="s">
         <v>415</v>
       </c>
-      <c r="G87" s="14" t="s">
+      <c r="H87" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="I87" s="14" t="s">
         <v>416</v>
-      </c>
-      <c r="H87" s="14" t="s">
-        <v>158</v>
-      </c>
-      <c r="I87" s="14" t="s">
-        <v>374</v>
       </c>
       <c r="J87" s="14" t="s">
         <v>16</v>
@@ -6769,13 +6791,13 @@
         <v>20</v>
       </c>
       <c r="C88" s="14" t="s">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="D88" s="14" t="s">
         <v>418</v>
       </c>
       <c r="E88" s="14" t="s">
-        <v>371</v>
+        <v>383</v>
       </c>
       <c r="F88" s="14" t="s">
         <v>419</v>
@@ -6784,10 +6806,10 @@
         <v>420</v>
       </c>
       <c r="H88" s="14" t="s">
-        <v>72</v>
+        <v>158</v>
       </c>
       <c r="I88" s="14" t="s">
-        <v>421</v>
+        <v>386</v>
       </c>
       <c r="J88" s="14" t="s">
         <v>16</v>
@@ -6800,31 +6822,31 @@
     </row>
     <row r="89" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="14" t="s">
+        <v>421</v>
+      </c>
+      <c r="B89" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="C89" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="D89" s="14" t="s">
         <v>422</v>
       </c>
-      <c r="B89" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="C89" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="D89" s="14" t="s">
+      <c r="E89" s="14" t="s">
+        <v>383</v>
+      </c>
+      <c r="F89" s="14" t="s">
         <v>423</v>
       </c>
-      <c r="E89" s="14" t="s">
-        <v>371</v>
-      </c>
-      <c r="F89" s="14" t="s">
+      <c r="G89" s="14" t="s">
         <v>424</v>
-      </c>
-      <c r="G89" s="14" t="s">
-        <v>425</v>
       </c>
       <c r="H89" s="14" t="s">
         <v>158</v>
       </c>
       <c r="I89" s="14" t="s">
-        <v>374</v>
+        <v>386</v>
       </c>
       <c r="J89" s="14" t="s">
         <v>16</v>
@@ -6837,31 +6859,31 @@
     </row>
     <row r="90" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="14" t="s">
+        <v>425</v>
+      </c>
+      <c r="B90" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="C90" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="D90" s="14" t="s">
         <v>426</v>
       </c>
-      <c r="B90" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="C90" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="D90" s="14" t="s">
+      <c r="E90" s="14" t="s">
+        <v>383</v>
+      </c>
+      <c r="F90" s="14" t="s">
         <v>427</v>
       </c>
-      <c r="E90" s="14" t="s">
-        <v>371</v>
-      </c>
-      <c r="F90" s="14" t="s">
+      <c r="G90" s="14" t="s">
         <v>428</v>
-      </c>
-      <c r="G90" s="14" t="s">
-        <v>429</v>
       </c>
       <c r="H90" s="14" t="s">
         <v>158</v>
       </c>
       <c r="I90" s="14" t="s">
-        <v>374</v>
+        <v>386</v>
       </c>
       <c r="J90" s="14" t="s">
         <v>16</v>
@@ -6874,31 +6896,31 @@
     </row>
     <row r="91" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="14" t="s">
+        <v>429</v>
+      </c>
+      <c r="B91" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="C91" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="D91" s="14" t="s">
         <v>430</v>
       </c>
-      <c r="B91" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="C91" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="D91" s="14" t="s">
+      <c r="E91" s="14" t="s">
+        <v>383</v>
+      </c>
+      <c r="F91" s="14" t="s">
         <v>431</v>
       </c>
-      <c r="E91" s="14" t="s">
-        <v>371</v>
-      </c>
-      <c r="F91" s="14" t="s">
+      <c r="G91" s="14" t="s">
         <v>432</v>
       </c>
-      <c r="G91" s="14" t="s">
+      <c r="H91" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="I91" s="14" t="s">
         <v>433</v>
-      </c>
-      <c r="H91" s="14" t="s">
-        <v>158</v>
-      </c>
-      <c r="I91" s="14" t="s">
-        <v>374</v>
       </c>
       <c r="J91" s="14" t="s">
         <v>16</v>
@@ -6917,13 +6939,13 @@
         <v>20</v>
       </c>
       <c r="C92" s="14" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D92" s="14" t="s">
         <v>435</v>
       </c>
       <c r="E92" s="14" t="s">
-        <v>371</v>
+        <v>383</v>
       </c>
       <c r="F92" s="14" t="s">
         <v>436</v>
@@ -6935,7 +6957,7 @@
         <v>158</v>
       </c>
       <c r="I92" s="14" t="s">
-        <v>374</v>
+        <v>386</v>
       </c>
       <c r="J92" s="14" t="s">
         <v>16</v>
@@ -6954,13 +6976,13 @@
         <v>20</v>
       </c>
       <c r="C93" s="14" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D93" s="14" t="s">
         <v>439</v>
       </c>
       <c r="E93" s="14" t="s">
-        <v>371</v>
+        <v>383</v>
       </c>
       <c r="F93" s="14" t="s">
         <v>440</v>
@@ -6972,7 +6994,7 @@
         <v>158</v>
       </c>
       <c r="I93" s="14" t="s">
-        <v>374</v>
+        <v>386</v>
       </c>
       <c r="J93" s="14" t="s">
         <v>16</v>
@@ -6991,13 +7013,13 @@
         <v>20</v>
       </c>
       <c r="C94" s="14" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D94" s="14" t="s">
         <v>443</v>
       </c>
       <c r="E94" s="14" t="s">
-        <v>371</v>
+        <v>383</v>
       </c>
       <c r="F94" s="14" t="s">
         <v>444</v>
@@ -7009,7 +7031,7 @@
         <v>158</v>
       </c>
       <c r="I94" s="14" t="s">
-        <v>374</v>
+        <v>386</v>
       </c>
       <c r="J94" s="14" t="s">
         <v>16</v>
@@ -7028,13 +7050,13 @@
         <v>20</v>
       </c>
       <c r="C95" s="14" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D95" s="14" t="s">
         <v>447</v>
       </c>
       <c r="E95" s="14" t="s">
-        <v>371</v>
+        <v>383</v>
       </c>
       <c r="F95" s="14" t="s">
         <v>448</v>
@@ -7043,10 +7065,10 @@
         <v>449</v>
       </c>
       <c r="H95" s="14" t="s">
-        <v>450</v>
+        <v>158</v>
       </c>
       <c r="I95" s="14" t="s">
-        <v>399</v>
+        <v>386</v>
       </c>
       <c r="J95" s="14" t="s">
         <v>16</v>
@@ -7059,31 +7081,31 @@
     </row>
     <row r="96" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="14" t="s">
+        <v>450</v>
+      </c>
+      <c r="B96" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="C96" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="D96" s="14" t="s">
         <v>451</v>
       </c>
-      <c r="B96" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="C96" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="D96" s="14" t="s">
+      <c r="E96" s="14" t="s">
+        <v>383</v>
+      </c>
+      <c r="F96" s="14" t="s">
         <v>452</v>
       </c>
-      <c r="E96" s="14" t="s">
-        <v>371</v>
-      </c>
-      <c r="F96" s="14" t="s">
+      <c r="G96" s="14" t="s">
         <v>453</v>
       </c>
-      <c r="G96" s="14" t="s">
-        <v>454</v>
-      </c>
       <c r="H96" s="14" t="s">
-        <v>72</v>
+        <v>158</v>
       </c>
       <c r="I96" s="14" t="s">
-        <v>374</v>
+        <v>386</v>
       </c>
       <c r="J96" s="14" t="s">
         <v>16</v>
@@ -7096,31 +7118,31 @@
     </row>
     <row r="97" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="14" t="s">
+        <v>454</v>
+      </c>
+      <c r="B97" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="C97" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="D97" s="14" t="s">
         <v>455</v>
       </c>
-      <c r="B97" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="C97" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="D97" s="14" t="s">
+      <c r="E97" s="14" t="s">
+        <v>383</v>
+      </c>
+      <c r="F97" s="14" t="s">
         <v>456</v>
       </c>
-      <c r="E97" s="14" t="s">
-        <v>371</v>
-      </c>
-      <c r="F97" s="14" t="s">
+      <c r="G97" s="14" t="s">
         <v>457</v>
       </c>
-      <c r="G97" s="14" t="s">
-        <v>458</v>
-      </c>
       <c r="H97" s="14" t="s">
-        <v>450</v>
+        <v>158</v>
       </c>
       <c r="I97" s="14" t="s">
-        <v>399</v>
+        <v>386</v>
       </c>
       <c r="J97" s="14" t="s">
         <v>16</v>
@@ -7131,33 +7153,33 @@
       <c r="N97" s="15"/>
       <c r="O97" s="15"/>
     </row>
-    <row r="98" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="98" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="14" t="s">
+        <v>458</v>
+      </c>
+      <c r="B98" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="C98" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="D98" s="14" t="s">
         <v>459</v>
       </c>
-      <c r="B98" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="C98" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="D98" s="14" t="s">
+      <c r="E98" s="14" t="s">
+        <v>383</v>
+      </c>
+      <c r="F98" s="14" t="s">
         <v>460</v>
       </c>
-      <c r="E98" s="14" t="s">
-        <v>371</v>
-      </c>
-      <c r="F98" s="14" t="s">
+      <c r="G98" s="14" t="s">
         <v>461</v>
       </c>
-      <c r="G98" s="14" t="s">
+      <c r="H98" s="14" t="s">
         <v>462</v>
       </c>
-      <c r="H98" s="14" t="s">
-        <v>158</v>
-      </c>
       <c r="I98" s="14" t="s">
-        <v>374</v>
+        <v>411</v>
       </c>
       <c r="J98" s="14" t="s">
         <v>16</v>
@@ -7173,16 +7195,16 @@
         <v>463</v>
       </c>
       <c r="B99" s="14" t="s">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="C99" s="14" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="D99" s="14" t="s">
         <v>464</v>
       </c>
       <c r="E99" s="14" t="s">
-        <v>371</v>
+        <v>383</v>
       </c>
       <c r="F99" s="14" t="s">
         <v>465</v>
@@ -7191,10 +7213,10 @@
         <v>466</v>
       </c>
       <c r="H99" s="14" t="s">
-        <v>158</v>
+        <v>72</v>
       </c>
       <c r="I99" s="14" t="s">
-        <v>404</v>
+        <v>386</v>
       </c>
       <c r="J99" s="14" t="s">
         <v>16</v>
@@ -7213,13 +7235,13 @@
         <v>20</v>
       </c>
       <c r="C100" s="14" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="D100" s="14" t="s">
         <v>468</v>
       </c>
       <c r="E100" s="14" t="s">
-        <v>371</v>
+        <v>383</v>
       </c>
       <c r="F100" s="14" t="s">
         <v>469</v>
@@ -7228,10 +7250,10 @@
         <v>470</v>
       </c>
       <c r="H100" s="14" t="s">
-        <v>158</v>
+        <v>462</v>
       </c>
       <c r="I100" s="14" t="s">
-        <v>399</v>
+        <v>411</v>
       </c>
       <c r="J100" s="14" t="s">
         <v>16</v>
@@ -7242,7 +7264,7 @@
       <c r="N100" s="15"/>
       <c r="O100" s="15"/>
     </row>
-    <row r="101" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="101" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="14" t="s">
         <v>471</v>
       </c>
@@ -7250,13 +7272,13 @@
         <v>20</v>
       </c>
       <c r="C101" s="14" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D101" s="14" t="s">
         <v>472</v>
       </c>
       <c r="E101" s="14" t="s">
-        <v>371</v>
+        <v>383</v>
       </c>
       <c r="F101" s="14" t="s">
         <v>473</v>
@@ -7265,10 +7287,10 @@
         <v>474</v>
       </c>
       <c r="H101" s="14" t="s">
-        <v>450</v>
+        <v>158</v>
       </c>
       <c r="I101" s="14" t="s">
-        <v>399</v>
+        <v>386</v>
       </c>
       <c r="J101" s="14" t="s">
         <v>16</v>
@@ -7279,7 +7301,7 @@
       <c r="N101" s="15"/>
       <c r="O101" s="15"/>
     </row>
-    <row r="102" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="102" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="14" t="s">
         <v>475</v>
       </c>
@@ -7287,13 +7309,13 @@
         <v>39</v>
       </c>
       <c r="C102" s="14" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="D102" s="14" t="s">
         <v>476</v>
       </c>
       <c r="E102" s="14" t="s">
-        <v>371</v>
+        <v>383</v>
       </c>
       <c r="F102" s="14" t="s">
         <v>477</v>
@@ -7302,10 +7324,10 @@
         <v>478</v>
       </c>
       <c r="H102" s="14" t="s">
-        <v>72</v>
+        <v>158</v>
       </c>
       <c r="I102" s="14" t="s">
-        <v>404</v>
+        <v>416</v>
       </c>
       <c r="J102" s="14" t="s">
         <v>16</v>
@@ -7321,16 +7343,16 @@
         <v>479</v>
       </c>
       <c r="B103" s="14" t="s">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="C103" s="14" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D103" s="14" t="s">
         <v>480</v>
       </c>
       <c r="E103" s="14" t="s">
-        <v>371</v>
+        <v>383</v>
       </c>
       <c r="F103" s="14" t="s">
         <v>481</v>
@@ -7339,10 +7361,10 @@
         <v>482</v>
       </c>
       <c r="H103" s="14" t="s">
-        <v>72</v>
+        <v>158</v>
       </c>
       <c r="I103" s="14" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="J103" s="14" t="s">
         <v>16</v>
@@ -7358,16 +7380,16 @@
         <v>483</v>
       </c>
       <c r="B104" s="14" t="s">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="C104" s="14" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D104" s="14" t="s">
         <v>484</v>
       </c>
       <c r="E104" s="14" t="s">
-        <v>371</v>
+        <v>383</v>
       </c>
       <c r="F104" s="14" t="s">
         <v>485</v>
@@ -7376,10 +7398,10 @@
         <v>486</v>
       </c>
       <c r="H104" s="14" t="s">
-        <v>72</v>
+        <v>462</v>
       </c>
       <c r="I104" s="14" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="J104" s="14" t="s">
         <v>16</v>
@@ -7404,7 +7426,7 @@
         <v>488</v>
       </c>
       <c r="E105" s="14" t="s">
-        <v>371</v>
+        <v>383</v>
       </c>
       <c r="F105" s="14" t="s">
         <v>489</v>
@@ -7413,10 +7435,10 @@
         <v>490</v>
       </c>
       <c r="H105" s="14" t="s">
-        <v>158</v>
+        <v>72</v>
       </c>
       <c r="I105" s="14" t="s">
-        <v>404</v>
+        <v>416</v>
       </c>
       <c r="J105" s="14" t="s">
         <v>16</v>
@@ -7432,16 +7454,16 @@
         <v>491</v>
       </c>
       <c r="B106" s="14" t="s">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="C106" s="14" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="D106" s="14" t="s">
         <v>492</v>
       </c>
       <c r="E106" s="14" t="s">
-        <v>371</v>
+        <v>383</v>
       </c>
       <c r="F106" s="14" t="s">
         <v>493</v>
@@ -7450,10 +7472,10 @@
         <v>494</v>
       </c>
       <c r="H106" s="14" t="s">
-        <v>158</v>
+        <v>72</v>
       </c>
       <c r="I106" s="14" t="s">
-        <v>37</v>
+        <v>416</v>
       </c>
       <c r="J106" s="14" t="s">
         <v>16</v>
@@ -7464,9 +7486,120 @@
       <c r="N106" s="15"/>
       <c r="O106" s="15"/>
     </row>
+    <row r="107" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A107" s="14" t="s">
+        <v>495</v>
+      </c>
+      <c r="B107" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="C107" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="D107" s="14" t="s">
+        <v>496</v>
+      </c>
+      <c r="E107" s="14" t="s">
+        <v>383</v>
+      </c>
+      <c r="F107" s="14" t="s">
+        <v>497</v>
+      </c>
+      <c r="G107" s="14" t="s">
+        <v>498</v>
+      </c>
+      <c r="H107" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="I107" s="14" t="s">
+        <v>416</v>
+      </c>
+      <c r="J107" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="K107" s="14"/>
+      <c r="L107" s="15"/>
+      <c r="M107" s="15"/>
+      <c r="N107" s="15"/>
+      <c r="O107" s="15"/>
+    </row>
+    <row r="108" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A108" s="14" t="s">
+        <v>499</v>
+      </c>
+      <c r="B108" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="C108" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="D108" s="14" t="s">
+        <v>500</v>
+      </c>
+      <c r="E108" s="14" t="s">
+        <v>383</v>
+      </c>
+      <c r="F108" s="14" t="s">
+        <v>501</v>
+      </c>
+      <c r="G108" s="14" t="s">
+        <v>502</v>
+      </c>
+      <c r="H108" s="14" t="s">
+        <v>158</v>
+      </c>
+      <c r="I108" s="14" t="s">
+        <v>416</v>
+      </c>
+      <c r="J108" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="K108" s="14"/>
+      <c r="L108" s="15"/>
+      <c r="M108" s="15"/>
+      <c r="N108" s="15"/>
+      <c r="O108" s="15"/>
+    </row>
+    <row r="109" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A109" s="14" t="s">
+        <v>503</v>
+      </c>
+      <c r="B109" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="C109" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="D109" s="14" t="s">
+        <v>504</v>
+      </c>
+      <c r="E109" s="14" t="s">
+        <v>383</v>
+      </c>
+      <c r="F109" s="14" t="s">
+        <v>505</v>
+      </c>
+      <c r="G109" s="14" t="s">
+        <v>506</v>
+      </c>
+      <c r="H109" s="14" t="s">
+        <v>158</v>
+      </c>
+      <c r="I109" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="J109" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="K109" s="14"/>
+      <c r="L109" s="15"/>
+      <c r="M109" s="15"/>
+      <c r="N109" s="15"/>
+      <c r="O109" s="15"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O106"/>
-  <conditionalFormatting sqref="J2:J106">
+  <autoFilter ref="A1:O109"/>
+  <conditionalFormatting sqref="J2:J109">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
       <formula>"Pass"</formula>
     </cfRule>
@@ -7477,7 +7610,7 @@
       <formula>"Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L2:L106">
+  <conditionalFormatting sqref="L2:L109">
     <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
       <formula>"Pass"</formula>
     </cfRule>
@@ -7489,11 +7622,11 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L2:L106" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L2:L109" type="list">
       <formula1>"Pass,Fail,Blocked,Not Run"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H2:H106" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H2:H109" type="list">
       <formula1>"High,Medium,Low"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -7514,303 +7647,310 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="44"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="16" t="s">
-        <v>495</v>
+        <v>507</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="13" t="s">
+        <v>508</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
-        <v>496</v>
-      </c>
-      <c r="B3" s="13" t="s">
-        <v>497</v>
+      <c r="A3" s="13" t="s">
+        <v>509</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
-        <v>498</v>
-      </c>
-      <c r="B4" s="13" t="s">
-        <v>499</v>
+      <c r="A4" s="13" t="s">
+        <v>510</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
-        <v>500</v>
-      </c>
-      <c r="B5" s="13" t="s">
-        <v>501</v>
+      <c r="A5" s="13" t="s">
+        <v>511</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
-        <v>502</v>
-      </c>
-      <c r="B6" s="13" t="s">
-        <v>503</v>
+      <c r="A6" s="13" t="s">
+        <v>512</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
-        <v>504</v>
-      </c>
-      <c r="B7" s="13" t="s">
-        <v>505</v>
+      <c r="A7" s="13" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="16" t="s">
+        <v>514</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="16" t="s">
-        <v>506</v>
+      <c r="A10" s="2" t="s">
+        <v>515</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>516</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="9" t="s">
-        <v>507</v>
-      </c>
-      <c r="B11" s="9" t="s">
-        <v>508</v>
-      </c>
-      <c r="C11" s="9" t="s">
-        <v>509</v>
-      </c>
-      <c r="D11" s="9" t="s">
-        <v>510</v>
+      <c r="A11" s="2" t="s">
+        <v>517</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>518</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="14" t="s">
-        <v>511</v>
-      </c>
-      <c r="B12" s="14" t="s">
-        <v>512</v>
-      </c>
-      <c r="C12" s="14" t="s">
-        <v>513</v>
-      </c>
-      <c r="D12" s="14" t="s">
-        <v>514</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="14" t="s">
-        <v>515</v>
-      </c>
-      <c r="B13" s="14" t="s">
-        <v>516</v>
-      </c>
-      <c r="C13" s="14" t="s">
-        <v>517</v>
-      </c>
-      <c r="D13" s="14" t="s">
-        <v>518</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="14" t="s">
+      <c r="A12" s="2" t="s">
         <v>519</v>
       </c>
-      <c r="B14" s="14" t="s">
+      <c r="B12" s="13" t="s">
         <v>520</v>
       </c>
-      <c r="C14" s="14" t="s">
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="2" t="s">
         <v>521</v>
       </c>
-      <c r="D14" s="14" t="s">
+      <c r="B13" s="13" t="s">
         <v>522</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="14" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="16" t="s">
         <v>523</v>
       </c>
-      <c r="B15" s="14" t="s">
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="9" t="s">
         <v>524</v>
       </c>
-      <c r="C15" s="14" t="s">
+      <c r="B16" s="9" t="s">
         <v>525</v>
       </c>
-      <c r="D15" s="14" t="s">
+      <c r="C16" s="9" t="s">
         <v>526</v>
       </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="14" t="s">
+      <c r="D16" s="9" t="s">
         <v>527</v>
       </c>
-      <c r="B16" s="14" t="s">
-        <v>28</v>
-      </c>
-      <c r="C16" s="14" t="s">
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="14" t="s">
         <v>528</v>
       </c>
-      <c r="D16" s="14" t="s">
+      <c r="B17" s="14" t="s">
         <v>529</v>
       </c>
-    </row>
-    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="14" t="s">
+      <c r="C17" s="14" t="s">
         <v>530</v>
       </c>
-      <c r="B17" s="14" t="s">
+      <c r="D17" s="14" t="s">
         <v>531</v>
       </c>
-      <c r="C17" s="14" t="s">
+    </row>
+    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="14" t="s">
         <v>532</v>
       </c>
-      <c r="D17" s="14" t="s">
+      <c r="B18" s="14" t="s">
         <v>533</v>
       </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="14" t="s">
+      <c r="C18" s="14" t="s">
         <v>534</v>
       </c>
-      <c r="B18" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="C18" s="14" t="s">
+      <c r="D18" s="14" t="s">
         <v>535</v>
-      </c>
-      <c r="D18" s="14" t="s">
-        <v>536</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="14" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="B19" s="14" t="s">
         <v>26</v>
       </c>
       <c r="C19" s="14" t="s">
+        <v>537</v>
+      </c>
+      <c r="D19" s="14" t="s">
         <v>538</v>
       </c>
-      <c r="D19" s="14" t="s">
+    </row>
+    <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="14" t="s">
         <v>539</v>
       </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="14" t="s">
+      <c r="B20" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="C20" s="14" t="s">
         <v>540</v>
       </c>
-      <c r="B20" s="14" t="s">
+      <c r="D20" s="14" t="s">
         <v>541</v>
       </c>
-      <c r="C20" s="14" t="s">
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="14" t="s">
         <v>542</v>
       </c>
-      <c r="D20" s="14" t="s">
+      <c r="B21" s="14" t="s">
+        <v>530</v>
+      </c>
+      <c r="C21" s="14" t="s">
+        <v>537</v>
+      </c>
+      <c r="D21" s="14" t="s">
         <v>543</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="16" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="16" t="s">
         <v>544</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="17" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="9" t="s">
         <v>545</v>
       </c>
-      <c r="B23" s="17" t="s">
+      <c r="B24" s="9" t="s">
         <v>546</v>
       </c>
-      <c r="C23" s="17" t="s">
+      <c r="C24" s="9" t="s">
         <v>547</v>
       </c>
-      <c r="D23" s="17" t="s">
+      <c r="D24" s="9" t="s">
         <v>548</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="14" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="14" t="s">
         <v>549</v>
       </c>
-      <c r="B24" s="18" t="s">
+      <c r="B25" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="C25" s="14" t="s">
         <v>550</v>
       </c>
-      <c r="C24" s="14" t="s">
+      <c r="D25" s="14" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="14" t="s">
         <v>551</v>
       </c>
-      <c r="D24" s="14" t="s">
+      <c r="B26" s="14" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="25" customFormat="false" ht="147" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="14" t="s">
+      <c r="C26" s="14" t="s">
         <v>553</v>
       </c>
-      <c r="B25" s="18" t="s">
+      <c r="D26" s="14" t="s">
         <v>554</v>
       </c>
-      <c r="C25" s="14" t="s">
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="14" t="s">
         <v>555</v>
       </c>
-      <c r="D25" s="14" t="s">
+      <c r="B27" s="14" t="s">
         <v>556</v>
       </c>
-    </row>
-    <row r="26" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="14" t="s">
+      <c r="C27" s="14" t="s">
         <v>557</v>
       </c>
-      <c r="B26" s="18" t="s">
+      <c r="D27" s="14" t="s">
         <v>558</v>
       </c>
-      <c r="C26" s="14" t="s">
+    </row>
+    <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="14" t="s">
         <v>559</v>
       </c>
-      <c r="D26" s="14" t="s">
-        <v>556</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="14" t="s">
+      <c r="B28" s="14" t="s">
         <v>560</v>
       </c>
-      <c r="B27" s="18" t="s">
+      <c r="C28" s="14" t="s">
         <v>561</v>
       </c>
-      <c r="C27" s="14" t="s">
+      <c r="D28" s="14" t="s">
         <v>562</v>
       </c>
-      <c r="D27" s="14" t="s">
-        <v>556</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="14" t="s">
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="14" t="s">
         <v>563</v>
       </c>
-      <c r="B28" s="18" t="s">
+      <c r="B29" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="C29" s="14" t="s">
         <v>564</v>
       </c>
-      <c r="C28" s="14" t="s">
+      <c r="D29" s="14" t="s">
         <v>565</v>
       </c>
-      <c r="D28" s="14" t="s">
-        <v>556</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="13" t="s">
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="14" t="s">
         <v>566</v>
       </c>
+      <c r="B30" s="14" t="s">
+        <v>567</v>
+      </c>
+      <c r="C30" s="14" t="s">
+        <v>568</v>
+      </c>
+      <c r="D30" s="14" t="s">
+        <v>569</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="13" t="s">
-        <v>567</v>
+      <c r="A31" s="14" t="s">
+        <v>570</v>
+      </c>
+      <c r="B31" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="C31" s="14" t="s">
+        <v>571</v>
+      </c>
+      <c r="D31" s="14" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="14" t="s">
+        <v>573</v>
+      </c>
+      <c r="B32" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="C32" s="14" t="s">
+        <v>574</v>
+      </c>
+      <c r="D32" s="14" t="s">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="13" t="s">
+        <v>576</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
My Assets: review handover, report a problem to IT; Handovers: resolve issue
</commit_message>
<xml_diff>
--- a/Claude outputs/IT_Asset_Module_Test_Case_Suite.xlsx
+++ b/Claude outputs/IT_Asset_Module_Test_Case_Suite.xlsx
@@ -13,7 +13,7 @@
     <sheet name="IT Hub Roles &amp; Access" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Test Cases'!$A$1:$O$150</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Test Cases'!$A$1:$O$152</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1785" uniqueCount="751">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1807" uniqueCount="759">
   <si>
     <t xml:space="preserve">IT Asset Management — Test Case Suite</t>
   </si>
@@ -1192,7 +1192,7 @@
     <t xml:space="preserve">Closed year unchanged; open year depreciation recalculated from frozen book value</t>
   </si>
   <si>
-    <t xml:space="preserve">FY25 304279.88 unchanged; FY26 185659.98 → 69731.19</t>
+    <t xml:space="preserve">FY25 399279.92 unchanged; FY26 308613.39 → 129066.69</t>
   </si>
   <si>
     <t xml:space="preserve">DSP-01</t>
@@ -1237,7 +1237,7 @@
     <t xml:space="preserve">Lines present; total debit = total credit; ledgers per asset type</t>
   </si>
   <si>
-    <t xml:space="preserve">Dr = Cr = ₹27784.24</t>
+    <t xml:space="preserve">Dr = Cr = ₹46914.34</t>
   </si>
   <si>
     <t xml:space="preserve">JRN-02</t>
@@ -1277,6 +1277,32 @@
   </si>
   <si>
     <t xml:space="preserve">403; 400; 200 and the year is open again</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HOI-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Employee sends a handover back to IT with the problem</t>
+  </si>
+  <si>
+    <t xml:space="preserve">My Assets › Review &amp; acknowledge › Report a problem › choose 'Damaged or faulty' › describe › Send back to IT. Row shows 'Issue reported'; Acknowledge is not offered; Asset Admin gets an email.
+[API check: Issue an asset to me; My Assets › Review › Report a problem (Damaged) with details]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Status "Issue reported"; history entry; acknowledgement blocked until resolved</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HOI-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IT resolves and sends it back; employee re-reviews and acknowledges</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Handovers › Issues reported › Resolve issue › describe the fix › Send back for acknowledgement. Employee sees 'IT replied: …' in My Assets, gets an email, and acknowledges.
+[API check: Handovers › Issues reported › Resolve issue (note); then My Assets › Review &amp; acknowledge]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pending again with IT reply visible; then Acknowledged</t>
   </si>
   <si>
     <t xml:space="preserve">ARC-05</t>
@@ -3019,27 +3045,27 @@
         <v>21</v>
       </c>
       <c r="C11" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A11,'Test Cases'!$C$2:$C$150,$B11)</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A11,'Test Cases'!$C$2:$C$152,$B11)</f>
         <v>13</v>
       </c>
       <c r="D11" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A11,'Test Cases'!$C$2:$C$150,$B11,'Test Cases'!$J$2:$J$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A11,'Test Cases'!$C$2:$C$152,$B11,'Test Cases'!$J$2:$J$152,"Pass")</f>
         <v>8</v>
       </c>
       <c r="E11" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A11,'Test Cases'!$C$2:$C$150,$B11,'Test Cases'!$J$2:$J$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A11,'Test Cases'!$C$2:$C$152,$B11,'Test Cases'!$J$2:$J$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F11" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A11,'Test Cases'!$C$2:$C$150,$B11,'Test Cases'!$J$2:$J$150,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A11,'Test Cases'!$C$2:$C$152,$B11,'Test Cases'!$J$2:$J$152,"Manual (UAT)")</f>
         <v>5</v>
       </c>
       <c r="G11" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A11,'Test Cases'!$C$2:$C$150,$B11,'Test Cases'!$L$2:$L$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A11,'Test Cases'!$C$2:$C$152,$B11,'Test Cases'!$L$2:$L$152,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H11" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A11,'Test Cases'!$C$2:$C$150,$B11,'Test Cases'!$L$2:$L$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A11,'Test Cases'!$C$2:$C$152,$B11,'Test Cases'!$L$2:$L$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I11" s="6" t="n">
@@ -3055,27 +3081,27 @@
         <v>22</v>
       </c>
       <c r="C12" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A12,'Test Cases'!$C$2:$C$150,$B12)</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A12,'Test Cases'!$C$2:$C$152,$B12)</f>
         <v>3</v>
       </c>
       <c r="D12" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A12,'Test Cases'!$C$2:$C$150,$B12,'Test Cases'!$J$2:$J$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A12,'Test Cases'!$C$2:$C$152,$B12,'Test Cases'!$J$2:$J$152,"Pass")</f>
         <v>2</v>
       </c>
       <c r="E12" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A12,'Test Cases'!$C$2:$C$150,$B12,'Test Cases'!$J$2:$J$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A12,'Test Cases'!$C$2:$C$152,$B12,'Test Cases'!$J$2:$J$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F12" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A12,'Test Cases'!$C$2:$C$150,$B12,'Test Cases'!$J$2:$J$150,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A12,'Test Cases'!$C$2:$C$152,$B12,'Test Cases'!$J$2:$J$152,"Manual (UAT)")</f>
         <v>1</v>
       </c>
       <c r="G12" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A12,'Test Cases'!$C$2:$C$150,$B12,'Test Cases'!$L$2:$L$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A12,'Test Cases'!$C$2:$C$152,$B12,'Test Cases'!$L$2:$L$152,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H12" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A12,'Test Cases'!$C$2:$C$150,$B12,'Test Cases'!$L$2:$L$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A12,'Test Cases'!$C$2:$C$152,$B12,'Test Cases'!$L$2:$L$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I12" s="6" t="n">
@@ -3091,32 +3117,32 @@
         <v>23</v>
       </c>
       <c r="C13" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A13,'Test Cases'!$C$2:$C$150,$B13)</f>
-        <v>8</v>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A13,'Test Cases'!$C$2:$C$152,$B13)</f>
+        <v>9</v>
       </c>
       <c r="D13" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A13,'Test Cases'!$C$2:$C$150,$B13,'Test Cases'!$J$2:$J$150,"Pass")</f>
-        <v>6</v>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A13,'Test Cases'!$C$2:$C$152,$B13,'Test Cases'!$J$2:$J$152,"Pass")</f>
+        <v>7</v>
       </c>
       <c r="E13" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A13,'Test Cases'!$C$2:$C$150,$B13,'Test Cases'!$J$2:$J$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A13,'Test Cases'!$C$2:$C$152,$B13,'Test Cases'!$J$2:$J$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F13" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A13,'Test Cases'!$C$2:$C$150,$B13,'Test Cases'!$J$2:$J$150,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A13,'Test Cases'!$C$2:$C$152,$B13,'Test Cases'!$J$2:$J$152,"Manual (UAT)")</f>
         <v>2</v>
       </c>
       <c r="G13" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A13,'Test Cases'!$C$2:$C$150,$B13,'Test Cases'!$L$2:$L$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A13,'Test Cases'!$C$2:$C$152,$B13,'Test Cases'!$L$2:$L$152,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H13" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A13,'Test Cases'!$C$2:$C$150,$B13,'Test Cases'!$L$2:$L$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A13,'Test Cases'!$C$2:$C$152,$B13,'Test Cases'!$L$2:$L$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I13" s="6" t="n">
         <f aca="false">C13-G13-H13</f>
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3127,27 +3153,27 @@
         <v>24</v>
       </c>
       <c r="C14" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A14,'Test Cases'!$C$2:$C$150,$B14)</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A14,'Test Cases'!$C$2:$C$152,$B14)</f>
         <v>4</v>
       </c>
       <c r="D14" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A14,'Test Cases'!$C$2:$C$150,$B14,'Test Cases'!$J$2:$J$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A14,'Test Cases'!$C$2:$C$152,$B14,'Test Cases'!$J$2:$J$152,"Pass")</f>
         <v>4</v>
       </c>
       <c r="E14" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A14,'Test Cases'!$C$2:$C$150,$B14,'Test Cases'!$J$2:$J$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A14,'Test Cases'!$C$2:$C$152,$B14,'Test Cases'!$J$2:$J$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F14" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A14,'Test Cases'!$C$2:$C$150,$B14,'Test Cases'!$J$2:$J$150,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A14,'Test Cases'!$C$2:$C$152,$B14,'Test Cases'!$J$2:$J$152,"Manual (UAT)")</f>
         <v>0</v>
       </c>
       <c r="G14" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A14,'Test Cases'!$C$2:$C$150,$B14,'Test Cases'!$L$2:$L$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A14,'Test Cases'!$C$2:$C$152,$B14,'Test Cases'!$L$2:$L$152,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H14" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A14,'Test Cases'!$C$2:$C$150,$B14,'Test Cases'!$L$2:$L$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A14,'Test Cases'!$C$2:$C$152,$B14,'Test Cases'!$L$2:$L$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I14" s="6" t="n">
@@ -3163,32 +3189,32 @@
         <v>25</v>
       </c>
       <c r="C15" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A15,'Test Cases'!$C$2:$C$150,$B15)</f>
-        <v>1</v>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A15,'Test Cases'!$C$2:$C$152,$B15)</f>
+        <v>2</v>
       </c>
       <c r="D15" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A15,'Test Cases'!$C$2:$C$150,$B15,'Test Cases'!$J$2:$J$150,"Pass")</f>
-        <v>1</v>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A15,'Test Cases'!$C$2:$C$152,$B15,'Test Cases'!$J$2:$J$152,"Pass")</f>
+        <v>2</v>
       </c>
       <c r="E15" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A15,'Test Cases'!$C$2:$C$150,$B15,'Test Cases'!$J$2:$J$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A15,'Test Cases'!$C$2:$C$152,$B15,'Test Cases'!$J$2:$J$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F15" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A15,'Test Cases'!$C$2:$C$150,$B15,'Test Cases'!$J$2:$J$150,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A15,'Test Cases'!$C$2:$C$152,$B15,'Test Cases'!$J$2:$J$152,"Manual (UAT)")</f>
         <v>0</v>
       </c>
       <c r="G15" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A15,'Test Cases'!$C$2:$C$150,$B15,'Test Cases'!$L$2:$L$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A15,'Test Cases'!$C$2:$C$152,$B15,'Test Cases'!$L$2:$L$152,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H15" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A15,'Test Cases'!$C$2:$C$150,$B15,'Test Cases'!$L$2:$L$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A15,'Test Cases'!$C$2:$C$152,$B15,'Test Cases'!$L$2:$L$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I15" s="6" t="n">
         <f aca="false">C15-G15-H15</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3199,27 +3225,27 @@
         <v>26</v>
       </c>
       <c r="C16" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A16,'Test Cases'!$C$2:$C$150,$B16)</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A16,'Test Cases'!$C$2:$C$152,$B16)</f>
         <v>9</v>
       </c>
       <c r="D16" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A16,'Test Cases'!$C$2:$C$150,$B16,'Test Cases'!$J$2:$J$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A16,'Test Cases'!$C$2:$C$152,$B16,'Test Cases'!$J$2:$J$152,"Pass")</f>
         <v>9</v>
       </c>
       <c r="E16" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A16,'Test Cases'!$C$2:$C$150,$B16,'Test Cases'!$J$2:$J$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A16,'Test Cases'!$C$2:$C$152,$B16,'Test Cases'!$J$2:$J$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F16" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A16,'Test Cases'!$C$2:$C$150,$B16,'Test Cases'!$J$2:$J$150,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A16,'Test Cases'!$C$2:$C$152,$B16,'Test Cases'!$J$2:$J$152,"Manual (UAT)")</f>
         <v>0</v>
       </c>
       <c r="G16" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A16,'Test Cases'!$C$2:$C$150,$B16,'Test Cases'!$L$2:$L$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A16,'Test Cases'!$C$2:$C$152,$B16,'Test Cases'!$L$2:$L$152,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H16" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A16,'Test Cases'!$C$2:$C$150,$B16,'Test Cases'!$L$2:$L$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A16,'Test Cases'!$C$2:$C$152,$B16,'Test Cases'!$L$2:$L$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I16" s="6" t="n">
@@ -3235,27 +3261,27 @@
         <v>27</v>
       </c>
       <c r="C17" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A17,'Test Cases'!$C$2:$C$150,$B17)</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A17,'Test Cases'!$C$2:$C$152,$B17)</f>
         <v>2</v>
       </c>
       <c r="D17" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A17,'Test Cases'!$C$2:$C$150,$B17,'Test Cases'!$J$2:$J$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A17,'Test Cases'!$C$2:$C$152,$B17,'Test Cases'!$J$2:$J$152,"Pass")</f>
         <v>2</v>
       </c>
       <c r="E17" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A17,'Test Cases'!$C$2:$C$150,$B17,'Test Cases'!$J$2:$J$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A17,'Test Cases'!$C$2:$C$152,$B17,'Test Cases'!$J$2:$J$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F17" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A17,'Test Cases'!$C$2:$C$150,$B17,'Test Cases'!$J$2:$J$150,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A17,'Test Cases'!$C$2:$C$152,$B17,'Test Cases'!$J$2:$J$152,"Manual (UAT)")</f>
         <v>0</v>
       </c>
       <c r="G17" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A17,'Test Cases'!$C$2:$C$150,$B17,'Test Cases'!$L$2:$L$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A17,'Test Cases'!$C$2:$C$152,$B17,'Test Cases'!$L$2:$L$152,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H17" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A17,'Test Cases'!$C$2:$C$150,$B17,'Test Cases'!$L$2:$L$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A17,'Test Cases'!$C$2:$C$152,$B17,'Test Cases'!$L$2:$L$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I17" s="6" t="n">
@@ -3271,27 +3297,27 @@
         <v>28</v>
       </c>
       <c r="C18" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A18,'Test Cases'!$C$2:$C$150,$B18)</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A18,'Test Cases'!$C$2:$C$152,$B18)</f>
         <v>5</v>
       </c>
       <c r="D18" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A18,'Test Cases'!$C$2:$C$150,$B18,'Test Cases'!$J$2:$J$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A18,'Test Cases'!$C$2:$C$152,$B18,'Test Cases'!$J$2:$J$152,"Pass")</f>
         <v>4</v>
       </c>
       <c r="E18" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A18,'Test Cases'!$C$2:$C$150,$B18,'Test Cases'!$J$2:$J$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A18,'Test Cases'!$C$2:$C$152,$B18,'Test Cases'!$J$2:$J$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F18" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A18,'Test Cases'!$C$2:$C$150,$B18,'Test Cases'!$J$2:$J$150,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A18,'Test Cases'!$C$2:$C$152,$B18,'Test Cases'!$J$2:$J$152,"Manual (UAT)")</f>
         <v>1</v>
       </c>
       <c r="G18" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A18,'Test Cases'!$C$2:$C$150,$B18,'Test Cases'!$L$2:$L$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A18,'Test Cases'!$C$2:$C$152,$B18,'Test Cases'!$L$2:$L$152,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H18" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A18,'Test Cases'!$C$2:$C$150,$B18,'Test Cases'!$L$2:$L$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A18,'Test Cases'!$C$2:$C$152,$B18,'Test Cases'!$L$2:$L$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I18" s="6" t="n">
@@ -3307,27 +3333,27 @@
         <v>29</v>
       </c>
       <c r="C19" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A19,'Test Cases'!$C$2:$C$150,$B19)</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A19,'Test Cases'!$C$2:$C$152,$B19)</f>
         <v>7</v>
       </c>
       <c r="D19" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A19,'Test Cases'!$C$2:$C$150,$B19,'Test Cases'!$J$2:$J$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A19,'Test Cases'!$C$2:$C$152,$B19,'Test Cases'!$J$2:$J$152,"Pass")</f>
         <v>5</v>
       </c>
       <c r="E19" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A19,'Test Cases'!$C$2:$C$150,$B19,'Test Cases'!$J$2:$J$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A19,'Test Cases'!$C$2:$C$152,$B19,'Test Cases'!$J$2:$J$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F19" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A19,'Test Cases'!$C$2:$C$150,$B19,'Test Cases'!$J$2:$J$150,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A19,'Test Cases'!$C$2:$C$152,$B19,'Test Cases'!$J$2:$J$152,"Manual (UAT)")</f>
         <v>2</v>
       </c>
       <c r="G19" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A19,'Test Cases'!$C$2:$C$150,$B19,'Test Cases'!$L$2:$L$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A19,'Test Cases'!$C$2:$C$152,$B19,'Test Cases'!$L$2:$L$152,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H19" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A19,'Test Cases'!$C$2:$C$150,$B19,'Test Cases'!$L$2:$L$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A19,'Test Cases'!$C$2:$C$152,$B19,'Test Cases'!$L$2:$L$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I19" s="6" t="n">
@@ -3343,27 +3369,27 @@
         <v>30</v>
       </c>
       <c r="C20" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A20,'Test Cases'!$C$2:$C$150,$B20)</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A20,'Test Cases'!$C$2:$C$152,$B20)</f>
         <v>9</v>
       </c>
       <c r="D20" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A20,'Test Cases'!$C$2:$C$150,$B20,'Test Cases'!$J$2:$J$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A20,'Test Cases'!$C$2:$C$152,$B20,'Test Cases'!$J$2:$J$152,"Pass")</f>
         <v>7</v>
       </c>
       <c r="E20" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A20,'Test Cases'!$C$2:$C$150,$B20,'Test Cases'!$J$2:$J$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A20,'Test Cases'!$C$2:$C$152,$B20,'Test Cases'!$J$2:$J$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F20" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A20,'Test Cases'!$C$2:$C$150,$B20,'Test Cases'!$J$2:$J$150,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A20,'Test Cases'!$C$2:$C$152,$B20,'Test Cases'!$J$2:$J$152,"Manual (UAT)")</f>
         <v>2</v>
       </c>
       <c r="G20" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A20,'Test Cases'!$C$2:$C$150,$B20,'Test Cases'!$L$2:$L$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A20,'Test Cases'!$C$2:$C$152,$B20,'Test Cases'!$L$2:$L$152,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H20" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A20,'Test Cases'!$C$2:$C$150,$B20,'Test Cases'!$L$2:$L$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A20,'Test Cases'!$C$2:$C$152,$B20,'Test Cases'!$L$2:$L$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I20" s="6" t="n">
@@ -3379,27 +3405,27 @@
         <v>31</v>
       </c>
       <c r="C21" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A21,'Test Cases'!$C$2:$C$150,$B21)</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A21,'Test Cases'!$C$2:$C$152,$B21)</f>
         <v>11</v>
       </c>
       <c r="D21" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A21,'Test Cases'!$C$2:$C$150,$B21,'Test Cases'!$J$2:$J$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A21,'Test Cases'!$C$2:$C$152,$B21,'Test Cases'!$J$2:$J$152,"Pass")</f>
         <v>9</v>
       </c>
       <c r="E21" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A21,'Test Cases'!$C$2:$C$150,$B21,'Test Cases'!$J$2:$J$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A21,'Test Cases'!$C$2:$C$152,$B21,'Test Cases'!$J$2:$J$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F21" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A21,'Test Cases'!$C$2:$C$150,$B21,'Test Cases'!$J$2:$J$150,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A21,'Test Cases'!$C$2:$C$152,$B21,'Test Cases'!$J$2:$J$152,"Manual (UAT)")</f>
         <v>2</v>
       </c>
       <c r="G21" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A21,'Test Cases'!$C$2:$C$150,$B21,'Test Cases'!$L$2:$L$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A21,'Test Cases'!$C$2:$C$152,$B21,'Test Cases'!$L$2:$L$152,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H21" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A21,'Test Cases'!$C$2:$C$150,$B21,'Test Cases'!$L$2:$L$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A21,'Test Cases'!$C$2:$C$152,$B21,'Test Cases'!$L$2:$L$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I21" s="6" t="n">
@@ -3415,27 +3441,27 @@
         <v>32</v>
       </c>
       <c r="C22" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A22,'Test Cases'!$C$2:$C$150,$B22)</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A22,'Test Cases'!$C$2:$C$152,$B22)</f>
         <v>1</v>
       </c>
       <c r="D22" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A22,'Test Cases'!$C$2:$C$150,$B22,'Test Cases'!$J$2:$J$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A22,'Test Cases'!$C$2:$C$152,$B22,'Test Cases'!$J$2:$J$152,"Pass")</f>
         <v>1</v>
       </c>
       <c r="E22" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A22,'Test Cases'!$C$2:$C$150,$B22,'Test Cases'!$J$2:$J$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A22,'Test Cases'!$C$2:$C$152,$B22,'Test Cases'!$J$2:$J$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F22" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A22,'Test Cases'!$C$2:$C$150,$B22,'Test Cases'!$J$2:$J$150,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A22,'Test Cases'!$C$2:$C$152,$B22,'Test Cases'!$J$2:$J$152,"Manual (UAT)")</f>
         <v>0</v>
       </c>
       <c r="G22" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A22,'Test Cases'!$C$2:$C$150,$B22,'Test Cases'!$L$2:$L$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A22,'Test Cases'!$C$2:$C$152,$B22,'Test Cases'!$L$2:$L$152,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H22" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A22,'Test Cases'!$C$2:$C$150,$B22,'Test Cases'!$L$2:$L$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A22,'Test Cases'!$C$2:$C$152,$B22,'Test Cases'!$L$2:$L$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I22" s="6" t="n">
@@ -3451,27 +3477,27 @@
         <v>33</v>
       </c>
       <c r="C23" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A23,'Test Cases'!$C$2:$C$150,$B23)</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A23,'Test Cases'!$C$2:$C$152,$B23)</f>
         <v>4</v>
       </c>
       <c r="D23" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A23,'Test Cases'!$C$2:$C$150,$B23,'Test Cases'!$J$2:$J$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A23,'Test Cases'!$C$2:$C$152,$B23,'Test Cases'!$J$2:$J$152,"Pass")</f>
         <v>2</v>
       </c>
       <c r="E23" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A23,'Test Cases'!$C$2:$C$150,$B23,'Test Cases'!$J$2:$J$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A23,'Test Cases'!$C$2:$C$152,$B23,'Test Cases'!$J$2:$J$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F23" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A23,'Test Cases'!$C$2:$C$150,$B23,'Test Cases'!$J$2:$J$150,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A23,'Test Cases'!$C$2:$C$152,$B23,'Test Cases'!$J$2:$J$152,"Manual (UAT)")</f>
         <v>2</v>
       </c>
       <c r="G23" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A23,'Test Cases'!$C$2:$C$150,$B23,'Test Cases'!$L$2:$L$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A23,'Test Cases'!$C$2:$C$152,$B23,'Test Cases'!$L$2:$L$152,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H23" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A23,'Test Cases'!$C$2:$C$150,$B23,'Test Cases'!$L$2:$L$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A23,'Test Cases'!$C$2:$C$152,$B23,'Test Cases'!$L$2:$L$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I23" s="6" t="n">
@@ -3487,27 +3513,27 @@
         <v>34</v>
       </c>
       <c r="C24" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A24,'Test Cases'!$C$2:$C$150,$B24)</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A24,'Test Cases'!$C$2:$C$152,$B24)</f>
         <v>10</v>
       </c>
       <c r="D24" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A24,'Test Cases'!$C$2:$C$150,$B24,'Test Cases'!$J$2:$J$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A24,'Test Cases'!$C$2:$C$152,$B24,'Test Cases'!$J$2:$J$152,"Pass")</f>
         <v>7</v>
       </c>
       <c r="E24" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A24,'Test Cases'!$C$2:$C$150,$B24,'Test Cases'!$J$2:$J$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A24,'Test Cases'!$C$2:$C$152,$B24,'Test Cases'!$J$2:$J$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F24" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A24,'Test Cases'!$C$2:$C$150,$B24,'Test Cases'!$J$2:$J$150,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A24,'Test Cases'!$C$2:$C$152,$B24,'Test Cases'!$J$2:$J$152,"Manual (UAT)")</f>
         <v>3</v>
       </c>
       <c r="G24" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A24,'Test Cases'!$C$2:$C$150,$B24,'Test Cases'!$L$2:$L$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A24,'Test Cases'!$C$2:$C$152,$B24,'Test Cases'!$L$2:$L$152,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H24" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A24,'Test Cases'!$C$2:$C$150,$B24,'Test Cases'!$L$2:$L$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A24,'Test Cases'!$C$2:$C$152,$B24,'Test Cases'!$L$2:$L$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I24" s="6" t="n">
@@ -3523,27 +3549,27 @@
         <v>35</v>
       </c>
       <c r="C25" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A25,'Test Cases'!$C$2:$C$150,$B25)</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A25,'Test Cases'!$C$2:$C$152,$B25)</f>
         <v>2</v>
       </c>
       <c r="D25" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A25,'Test Cases'!$C$2:$C$150,$B25,'Test Cases'!$J$2:$J$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A25,'Test Cases'!$C$2:$C$152,$B25,'Test Cases'!$J$2:$J$152,"Pass")</f>
         <v>2</v>
       </c>
       <c r="E25" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A25,'Test Cases'!$C$2:$C$150,$B25,'Test Cases'!$J$2:$J$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A25,'Test Cases'!$C$2:$C$152,$B25,'Test Cases'!$J$2:$J$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F25" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A25,'Test Cases'!$C$2:$C$150,$B25,'Test Cases'!$J$2:$J$150,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A25,'Test Cases'!$C$2:$C$152,$B25,'Test Cases'!$J$2:$J$152,"Manual (UAT)")</f>
         <v>0</v>
       </c>
       <c r="G25" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A25,'Test Cases'!$C$2:$C$150,$B25,'Test Cases'!$L$2:$L$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A25,'Test Cases'!$C$2:$C$152,$B25,'Test Cases'!$L$2:$L$152,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H25" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A25,'Test Cases'!$C$2:$C$150,$B25,'Test Cases'!$L$2:$L$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A25,'Test Cases'!$C$2:$C$152,$B25,'Test Cases'!$L$2:$L$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I25" s="6" t="n">
@@ -3559,27 +3585,27 @@
         <v>36</v>
       </c>
       <c r="C26" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A26,'Test Cases'!$C$2:$C$150,$B26)</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A26,'Test Cases'!$C$2:$C$152,$B26)</f>
         <v>16</v>
       </c>
       <c r="D26" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A26,'Test Cases'!$C$2:$C$150,$B26,'Test Cases'!$J$2:$J$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A26,'Test Cases'!$C$2:$C$152,$B26,'Test Cases'!$J$2:$J$152,"Pass")</f>
         <v>13</v>
       </c>
       <c r="E26" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A26,'Test Cases'!$C$2:$C$150,$B26,'Test Cases'!$J$2:$J$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A26,'Test Cases'!$C$2:$C$152,$B26,'Test Cases'!$J$2:$J$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F26" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A26,'Test Cases'!$C$2:$C$150,$B26,'Test Cases'!$J$2:$J$150,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A26,'Test Cases'!$C$2:$C$152,$B26,'Test Cases'!$J$2:$J$152,"Manual (UAT)")</f>
         <v>3</v>
       </c>
       <c r="G26" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A26,'Test Cases'!$C$2:$C$150,$B26,'Test Cases'!$L$2:$L$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A26,'Test Cases'!$C$2:$C$152,$B26,'Test Cases'!$L$2:$L$152,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H26" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A26,'Test Cases'!$C$2:$C$150,$B26,'Test Cases'!$L$2:$L$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A26,'Test Cases'!$C$2:$C$152,$B26,'Test Cases'!$L$2:$L$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I26" s="6" t="n">
@@ -3595,27 +3621,27 @@
         <v>37</v>
       </c>
       <c r="C27" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A27,'Test Cases'!$C$2:$C$150,$B27)</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A27,'Test Cases'!$C$2:$C$152,$B27)</f>
         <v>3</v>
       </c>
       <c r="D27" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A27,'Test Cases'!$C$2:$C$150,$B27,'Test Cases'!$J$2:$J$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A27,'Test Cases'!$C$2:$C$152,$B27,'Test Cases'!$J$2:$J$152,"Pass")</f>
         <v>0</v>
       </c>
       <c r="E27" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A27,'Test Cases'!$C$2:$C$150,$B27,'Test Cases'!$J$2:$J$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A27,'Test Cases'!$C$2:$C$152,$B27,'Test Cases'!$J$2:$J$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F27" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A27,'Test Cases'!$C$2:$C$150,$B27,'Test Cases'!$J$2:$J$150,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A27,'Test Cases'!$C$2:$C$152,$B27,'Test Cases'!$J$2:$J$152,"Manual (UAT)")</f>
         <v>3</v>
       </c>
       <c r="G27" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A27,'Test Cases'!$C$2:$C$150,$B27,'Test Cases'!$L$2:$L$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A27,'Test Cases'!$C$2:$C$152,$B27,'Test Cases'!$L$2:$L$152,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H27" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A27,'Test Cases'!$C$2:$C$150,$B27,'Test Cases'!$L$2:$L$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A27,'Test Cases'!$C$2:$C$152,$B27,'Test Cases'!$L$2:$L$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I27" s="6" t="n">
@@ -3631,27 +3657,27 @@
         <v>38</v>
       </c>
       <c r="C28" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A28,'Test Cases'!$C$2:$C$150,$B28)</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A28,'Test Cases'!$C$2:$C$152,$B28)</f>
         <v>1</v>
       </c>
       <c r="D28" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A28,'Test Cases'!$C$2:$C$150,$B28,'Test Cases'!$J$2:$J$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A28,'Test Cases'!$C$2:$C$152,$B28,'Test Cases'!$J$2:$J$152,"Pass")</f>
         <v>0</v>
       </c>
       <c r="E28" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A28,'Test Cases'!$C$2:$C$150,$B28,'Test Cases'!$J$2:$J$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A28,'Test Cases'!$C$2:$C$152,$B28,'Test Cases'!$J$2:$J$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F28" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A28,'Test Cases'!$C$2:$C$150,$B28,'Test Cases'!$J$2:$J$150,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A28,'Test Cases'!$C$2:$C$152,$B28,'Test Cases'!$J$2:$J$152,"Manual (UAT)")</f>
         <v>1</v>
       </c>
       <c r="G28" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A28,'Test Cases'!$C$2:$C$150,$B28,'Test Cases'!$L$2:$L$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A28,'Test Cases'!$C$2:$C$152,$B28,'Test Cases'!$L$2:$L$152,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H28" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A28,'Test Cases'!$C$2:$C$150,$B28,'Test Cases'!$L$2:$L$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A28,'Test Cases'!$C$2:$C$152,$B28,'Test Cases'!$L$2:$L$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I28" s="6" t="n">
@@ -3667,27 +3693,27 @@
         <v>39</v>
       </c>
       <c r="C29" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A29,'Test Cases'!$C$2:$C$150,$B29)</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A29,'Test Cases'!$C$2:$C$152,$B29)</f>
         <v>1</v>
       </c>
       <c r="D29" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A29,'Test Cases'!$C$2:$C$150,$B29,'Test Cases'!$J$2:$J$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A29,'Test Cases'!$C$2:$C$152,$B29,'Test Cases'!$J$2:$J$152,"Pass")</f>
         <v>0</v>
       </c>
       <c r="E29" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A29,'Test Cases'!$C$2:$C$150,$B29,'Test Cases'!$J$2:$J$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A29,'Test Cases'!$C$2:$C$152,$B29,'Test Cases'!$J$2:$J$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F29" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A29,'Test Cases'!$C$2:$C$150,$B29,'Test Cases'!$J$2:$J$150,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A29,'Test Cases'!$C$2:$C$152,$B29,'Test Cases'!$J$2:$J$152,"Manual (UAT)")</f>
         <v>1</v>
       </c>
       <c r="G29" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A29,'Test Cases'!$C$2:$C$150,$B29,'Test Cases'!$L$2:$L$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A29,'Test Cases'!$C$2:$C$152,$B29,'Test Cases'!$L$2:$L$152,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H29" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A29,'Test Cases'!$C$2:$C$150,$B29,'Test Cases'!$L$2:$L$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A29,'Test Cases'!$C$2:$C$152,$B29,'Test Cases'!$L$2:$L$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I29" s="6" t="n">
@@ -3703,27 +3729,27 @@
         <v>40</v>
       </c>
       <c r="C30" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A30,'Test Cases'!$C$2:$C$150,$B30)</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A30,'Test Cases'!$C$2:$C$152,$B30)</f>
         <v>1</v>
       </c>
       <c r="D30" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A30,'Test Cases'!$C$2:$C$150,$B30,'Test Cases'!$J$2:$J$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A30,'Test Cases'!$C$2:$C$152,$B30,'Test Cases'!$J$2:$J$152,"Pass")</f>
         <v>0</v>
       </c>
       <c r="E30" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A30,'Test Cases'!$C$2:$C$150,$B30,'Test Cases'!$J$2:$J$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A30,'Test Cases'!$C$2:$C$152,$B30,'Test Cases'!$J$2:$J$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F30" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A30,'Test Cases'!$C$2:$C$150,$B30,'Test Cases'!$J$2:$J$150,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A30,'Test Cases'!$C$2:$C$152,$B30,'Test Cases'!$J$2:$J$152,"Manual (UAT)")</f>
         <v>1</v>
       </c>
       <c r="G30" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A30,'Test Cases'!$C$2:$C$150,$B30,'Test Cases'!$L$2:$L$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A30,'Test Cases'!$C$2:$C$152,$B30,'Test Cases'!$L$2:$L$152,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H30" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A30,'Test Cases'!$C$2:$C$150,$B30,'Test Cases'!$L$2:$L$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A30,'Test Cases'!$C$2:$C$152,$B30,'Test Cases'!$L$2:$L$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I30" s="6" t="n">
@@ -3739,27 +3765,27 @@
         <v>41</v>
       </c>
       <c r="C31" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A31,'Test Cases'!$C$2:$C$150,$B31)</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A31,'Test Cases'!$C$2:$C$152,$B31)</f>
         <v>1</v>
       </c>
       <c r="D31" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A31,'Test Cases'!$C$2:$C$150,$B31,'Test Cases'!$J$2:$J$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A31,'Test Cases'!$C$2:$C$152,$B31,'Test Cases'!$J$2:$J$152,"Pass")</f>
         <v>0</v>
       </c>
       <c r="E31" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A31,'Test Cases'!$C$2:$C$150,$B31,'Test Cases'!$J$2:$J$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A31,'Test Cases'!$C$2:$C$152,$B31,'Test Cases'!$J$2:$J$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F31" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A31,'Test Cases'!$C$2:$C$150,$B31,'Test Cases'!$J$2:$J$150,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A31,'Test Cases'!$C$2:$C$152,$B31,'Test Cases'!$J$2:$J$152,"Manual (UAT)")</f>
         <v>1</v>
       </c>
       <c r="G31" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A31,'Test Cases'!$C$2:$C$150,$B31,'Test Cases'!$L$2:$L$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A31,'Test Cases'!$C$2:$C$152,$B31,'Test Cases'!$L$2:$L$152,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H31" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A31,'Test Cases'!$C$2:$C$150,$B31,'Test Cases'!$L$2:$L$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A31,'Test Cases'!$C$2:$C$152,$B31,'Test Cases'!$L$2:$L$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I31" s="6" t="n">
@@ -3775,27 +3801,27 @@
         <v>42</v>
       </c>
       <c r="C32" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A32,'Test Cases'!$C$2:$C$150,$B32)</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A32,'Test Cases'!$C$2:$C$152,$B32)</f>
         <v>2</v>
       </c>
       <c r="D32" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A32,'Test Cases'!$C$2:$C$150,$B32,'Test Cases'!$J$2:$J$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A32,'Test Cases'!$C$2:$C$152,$B32,'Test Cases'!$J$2:$J$152,"Pass")</f>
         <v>0</v>
       </c>
       <c r="E32" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A32,'Test Cases'!$C$2:$C$150,$B32,'Test Cases'!$J$2:$J$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A32,'Test Cases'!$C$2:$C$152,$B32,'Test Cases'!$J$2:$J$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F32" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A32,'Test Cases'!$C$2:$C$150,$B32,'Test Cases'!$J$2:$J$150,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A32,'Test Cases'!$C$2:$C$152,$B32,'Test Cases'!$J$2:$J$152,"Manual (UAT)")</f>
         <v>2</v>
       </c>
       <c r="G32" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A32,'Test Cases'!$C$2:$C$150,$B32,'Test Cases'!$L$2:$L$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A32,'Test Cases'!$C$2:$C$152,$B32,'Test Cases'!$L$2:$L$152,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H32" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A32,'Test Cases'!$C$2:$C$150,$B32,'Test Cases'!$L$2:$L$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A32,'Test Cases'!$C$2:$C$152,$B32,'Test Cases'!$L$2:$L$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I32" s="6" t="n">
@@ -3811,27 +3837,27 @@
         <v>43</v>
       </c>
       <c r="C33" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A33,'Test Cases'!$C$2:$C$150,$B33)</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A33,'Test Cases'!$C$2:$C$152,$B33)</f>
         <v>1</v>
       </c>
       <c r="D33" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A33,'Test Cases'!$C$2:$C$150,$B33,'Test Cases'!$J$2:$J$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A33,'Test Cases'!$C$2:$C$152,$B33,'Test Cases'!$J$2:$J$152,"Pass")</f>
         <v>0</v>
       </c>
       <c r="E33" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A33,'Test Cases'!$C$2:$C$150,$B33,'Test Cases'!$J$2:$J$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A33,'Test Cases'!$C$2:$C$152,$B33,'Test Cases'!$J$2:$J$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F33" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A33,'Test Cases'!$C$2:$C$150,$B33,'Test Cases'!$J$2:$J$150,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A33,'Test Cases'!$C$2:$C$152,$B33,'Test Cases'!$J$2:$J$152,"Manual (UAT)")</f>
         <v>1</v>
       </c>
       <c r="G33" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A33,'Test Cases'!$C$2:$C$150,$B33,'Test Cases'!$L$2:$L$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A33,'Test Cases'!$C$2:$C$152,$B33,'Test Cases'!$L$2:$L$152,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H33" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A33,'Test Cases'!$C$2:$C$150,$B33,'Test Cases'!$L$2:$L$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A33,'Test Cases'!$C$2:$C$152,$B33,'Test Cases'!$L$2:$L$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I33" s="6" t="n">
@@ -3846,11 +3872,11 @@
       <c r="B34" s="7"/>
       <c r="C34" s="8" t="n">
         <f aca="false">SUM(C11:C33)</f>
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D34" s="8" t="n">
         <f aca="false">SUM(D11:D33)</f>
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E34" s="8" t="n">
         <f aca="false">SUM(E11:E33)</f>
@@ -3870,7 +3896,7 @@
       </c>
       <c r="I34" s="8" t="n">
         <f aca="false">SUM(I11:I33)</f>
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3881,27 +3907,27 @@
         <v>46</v>
       </c>
       <c r="C35" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A35,'Test Cases'!$C$2:$C$150,$B35)</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A35,'Test Cases'!$C$2:$C$152,$B35)</f>
         <v>21</v>
       </c>
       <c r="D35" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A35,'Test Cases'!$C$2:$C$150,$B35,'Test Cases'!$J$2:$J$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A35,'Test Cases'!$C$2:$C$152,$B35,'Test Cases'!$J$2:$J$152,"Pass")</f>
         <v>17</v>
       </c>
       <c r="E35" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A35,'Test Cases'!$C$2:$C$150,$B35,'Test Cases'!$J$2:$J$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A35,'Test Cases'!$C$2:$C$152,$B35,'Test Cases'!$J$2:$J$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F35" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A35,'Test Cases'!$C$2:$C$150,$B35,'Test Cases'!$J$2:$J$150,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A35,'Test Cases'!$C$2:$C$152,$B35,'Test Cases'!$J$2:$J$152,"Manual (UAT)")</f>
         <v>4</v>
       </c>
       <c r="G35" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A35,'Test Cases'!$C$2:$C$150,$B35,'Test Cases'!$L$2:$L$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A35,'Test Cases'!$C$2:$C$152,$B35,'Test Cases'!$L$2:$L$152,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H35" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A35,'Test Cases'!$C$2:$C$150,$B35,'Test Cases'!$L$2:$L$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A35,'Test Cases'!$C$2:$C$152,$B35,'Test Cases'!$L$2:$L$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I35" s="6" t="n">
@@ -3917,27 +3943,27 @@
         <v>47</v>
       </c>
       <c r="C36" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A36,'Test Cases'!$C$2:$C$150,$B36)</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A36,'Test Cases'!$C$2:$C$152,$B36)</f>
         <v>10</v>
       </c>
       <c r="D36" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A36,'Test Cases'!$C$2:$C$150,$B36,'Test Cases'!$J$2:$J$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A36,'Test Cases'!$C$2:$C$152,$B36,'Test Cases'!$J$2:$J$152,"Pass")</f>
         <v>10</v>
       </c>
       <c r="E36" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A36,'Test Cases'!$C$2:$C$150,$B36,'Test Cases'!$J$2:$J$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A36,'Test Cases'!$C$2:$C$152,$B36,'Test Cases'!$J$2:$J$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F36" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A36,'Test Cases'!$C$2:$C$150,$B36,'Test Cases'!$J$2:$J$150,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A36,'Test Cases'!$C$2:$C$152,$B36,'Test Cases'!$J$2:$J$152,"Manual (UAT)")</f>
         <v>0</v>
       </c>
       <c r="G36" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A36,'Test Cases'!$C$2:$C$150,$B36,'Test Cases'!$L$2:$L$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A36,'Test Cases'!$C$2:$C$152,$B36,'Test Cases'!$L$2:$L$152,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H36" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A36,'Test Cases'!$C$2:$C$150,$B36,'Test Cases'!$L$2:$L$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A36,'Test Cases'!$C$2:$C$152,$B36,'Test Cases'!$L$2:$L$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I36" s="6" t="n">
@@ -3953,27 +3979,27 @@
         <v>48</v>
       </c>
       <c r="C37" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A37,'Test Cases'!$C$2:$C$150,$B37)</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A37,'Test Cases'!$C$2:$C$152,$B37)</f>
         <v>2</v>
       </c>
       <c r="D37" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A37,'Test Cases'!$C$2:$C$150,$B37,'Test Cases'!$J$2:$J$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A37,'Test Cases'!$C$2:$C$152,$B37,'Test Cases'!$J$2:$J$152,"Pass")</f>
         <v>2</v>
       </c>
       <c r="E37" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A37,'Test Cases'!$C$2:$C$150,$B37,'Test Cases'!$J$2:$J$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A37,'Test Cases'!$C$2:$C$152,$B37,'Test Cases'!$J$2:$J$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F37" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A37,'Test Cases'!$C$2:$C$150,$B37,'Test Cases'!$J$2:$J$150,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A37,'Test Cases'!$C$2:$C$152,$B37,'Test Cases'!$J$2:$J$152,"Manual (UAT)")</f>
         <v>0</v>
       </c>
       <c r="G37" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A37,'Test Cases'!$C$2:$C$150,$B37,'Test Cases'!$L$2:$L$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A37,'Test Cases'!$C$2:$C$152,$B37,'Test Cases'!$L$2:$L$152,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H37" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A37,'Test Cases'!$C$2:$C$150,$B37,'Test Cases'!$L$2:$L$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A37,'Test Cases'!$C$2:$C$152,$B37,'Test Cases'!$L$2:$L$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I37" s="6" t="n">
@@ -3989,27 +4015,27 @@
         <v>49</v>
       </c>
       <c r="C38" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A38,'Test Cases'!$C$2:$C$150,$B38)</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A38,'Test Cases'!$C$2:$C$152,$B38)</f>
         <v>1</v>
       </c>
       <c r="D38" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A38,'Test Cases'!$C$2:$C$150,$B38,'Test Cases'!$J$2:$J$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A38,'Test Cases'!$C$2:$C$152,$B38,'Test Cases'!$J$2:$J$152,"Pass")</f>
         <v>0</v>
       </c>
       <c r="E38" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A38,'Test Cases'!$C$2:$C$150,$B38,'Test Cases'!$J$2:$J$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A38,'Test Cases'!$C$2:$C$152,$B38,'Test Cases'!$J$2:$J$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="F38" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A38,'Test Cases'!$C$2:$C$150,$B38,'Test Cases'!$J$2:$J$150,"Manual (UAT)")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A38,'Test Cases'!$C$2:$C$152,$B38,'Test Cases'!$J$2:$J$152,"Manual (UAT)")</f>
         <v>1</v>
       </c>
       <c r="G38" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A38,'Test Cases'!$C$2:$C$150,$B38,'Test Cases'!$L$2:$L$150,"Pass")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A38,'Test Cases'!$C$2:$C$152,$B38,'Test Cases'!$L$2:$L$152,"Pass")</f>
         <v>0</v>
       </c>
       <c r="H38" s="6" t="n">
-        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$150,$A38,'Test Cases'!$C$2:$C$150,$B38,'Test Cases'!$L$2:$L$150,"Fail")</f>
+        <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$152,$A38,'Test Cases'!$C$2:$C$152,$B38,'Test Cases'!$L$2:$L$152,"Fail")</f>
         <v>0</v>
       </c>
       <c r="I38" s="6" t="n">
@@ -4058,11 +4084,11 @@
       <c r="B40" s="9"/>
       <c r="C40" s="10" t="n">
         <f aca="false">C11+C12+C13+C14+C15+C16+C17+C18+C19+C20+C21+C22+C23+C24+C25+C26+C27+C28+C29+C30+C31+C32+C33+C35+C36+C37+C38</f>
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D40" s="10" t="n">
         <f aca="false">D11+D12+D13+D14+D15+D16+D17+D18+D19+D20+D21+D22+D23+D24+D25+D26+D27+D28+D29+D30+D31+D32+D33+D35+D36+D37+D38</f>
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E40" s="10" t="n">
         <f aca="false">E11+E12+E13+E14+E15+E16+E17+E18+E19+E20+E21+E22+E23+E24+E25+E26+E27+E28+E29+E30+E31+E32+E33+E35+E36+E37+E38</f>
@@ -4082,7 +4108,7 @@
       </c>
       <c r="I40" s="10" t="n">
         <f aca="false">I11+I12+I13+I14+I15+I16+I17+I18+I19+I20+I21+I22+I23+I24+I25+I26+I27+I28+I29+I30+I31+I32+I33+I35+I36+I37+I38</f>
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4149,7 +4175,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O150"/>
+  <dimension ref="A1:O152"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -7297,7 +7323,7 @@
       <c r="N80" s="15"/>
       <c r="O80" s="15"/>
     </row>
-    <row r="81" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="81" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="14" t="s">
         <v>391</v>
       </c>
@@ -7305,7 +7331,7 @@
         <v>20</v>
       </c>
       <c r="C81" s="14" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="D81" s="14" t="s">
         <v>392</v>
@@ -7336,7 +7362,7 @@
       <c r="N81" s="15"/>
       <c r="O81" s="15"/>
     </row>
-    <row r="82" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="82" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="14" t="s">
         <v>395</v>
       </c>
@@ -7344,7 +7370,7 @@
         <v>20</v>
       </c>
       <c r="C82" s="14" t="s">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="D82" s="14" t="s">
         <v>396</v>
@@ -7375,7 +7401,7 @@
       <c r="N82" s="15"/>
       <c r="O82" s="15"/>
     </row>
-    <row r="83" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="83" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="14" t="s">
         <v>399</v>
       </c>
@@ -7395,7 +7421,7 @@
         <v>401</v>
       </c>
       <c r="G83" s="14" t="s">
-        <v>203</v>
+        <v>402</v>
       </c>
       <c r="H83" s="14" t="s">
         <v>164</v>
@@ -7414,21 +7440,21 @@
       <c r="N83" s="15"/>
       <c r="O83" s="15"/>
     </row>
-    <row r="84" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="84" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="14" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="B84" s="14" t="s">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="C84" s="14" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="D84" s="14" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="E84" s="14" t="s">
-        <v>404</v>
+        <v>75</v>
       </c>
       <c r="F84" s="14" t="s">
         <v>405</v>
@@ -7437,7 +7463,7 @@
         <v>406</v>
       </c>
       <c r="H84" s="14" t="s">
-        <v>78</v>
+        <v>164</v>
       </c>
       <c r="I84" s="14" t="s">
         <v>79</v>
@@ -7453,30 +7479,30 @@
       <c r="N84" s="15"/>
       <c r="O84" s="15"/>
     </row>
-    <row r="85" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="85" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="14" t="s">
         <v>407</v>
       </c>
       <c r="B85" s="14" t="s">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="C85" s="14" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="D85" s="14" t="s">
         <v>408</v>
       </c>
       <c r="E85" s="14" t="s">
-        <v>404</v>
+        <v>75</v>
       </c>
       <c r="F85" s="14" t="s">
         <v>409</v>
       </c>
       <c r="G85" s="14" t="s">
-        <v>410</v>
+        <v>203</v>
       </c>
       <c r="H85" s="14" t="s">
-        <v>78</v>
+        <v>164</v>
       </c>
       <c r="I85" s="14" t="s">
         <v>79</v>
@@ -7494,7 +7520,7 @@
     </row>
     <row r="86" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="14" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="B86" s="14" t="s">
         <v>45</v>
@@ -7503,10 +7529,10 @@
         <v>46</v>
       </c>
       <c r="D86" s="14" t="s">
+        <v>411</v>
+      </c>
+      <c r="E86" s="14" t="s">
         <v>412</v>
-      </c>
-      <c r="E86" s="14" t="s">
-        <v>404</v>
       </c>
       <c r="F86" s="14" t="s">
         <v>413</v>
@@ -7518,7 +7544,7 @@
         <v>78</v>
       </c>
       <c r="I86" s="14" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="J86" s="14" t="s">
         <v>80</v>
@@ -7545,7 +7571,7 @@
         <v>416</v>
       </c>
       <c r="E87" s="14" t="s">
-        <v>404</v>
+        <v>412</v>
       </c>
       <c r="F87" s="14" t="s">
         <v>417</v>
@@ -7584,7 +7610,7 @@
         <v>420</v>
       </c>
       <c r="E88" s="14" t="s">
-        <v>404</v>
+        <v>412</v>
       </c>
       <c r="F88" s="14" t="s">
         <v>421</v>
@@ -7623,7 +7649,7 @@
         <v>424</v>
       </c>
       <c r="E89" s="14" t="s">
-        <v>404</v>
+        <v>412</v>
       </c>
       <c r="F89" s="14" t="s">
         <v>425</v>
@@ -7635,7 +7661,7 @@
         <v>78</v>
       </c>
       <c r="I89" s="14" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="J89" s="14" t="s">
         <v>80</v>
@@ -7662,7 +7688,7 @@
         <v>428</v>
       </c>
       <c r="E90" s="14" t="s">
-        <v>404</v>
+        <v>412</v>
       </c>
       <c r="F90" s="14" t="s">
         <v>429</v>
@@ -7701,7 +7727,7 @@
         <v>432</v>
       </c>
       <c r="E91" s="14" t="s">
-        <v>404</v>
+        <v>412</v>
       </c>
       <c r="F91" s="14" t="s">
         <v>433</v>
@@ -7713,7 +7739,7 @@
         <v>78</v>
       </c>
       <c r="I91" s="14" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="J91" s="14" t="s">
         <v>80</v>
@@ -7726,7 +7752,7 @@
       <c r="N91" s="15"/>
       <c r="O91" s="15"/>
     </row>
-    <row r="92" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="92" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="14" t="s">
         <v>435</v>
       </c>
@@ -7734,25 +7760,25 @@
         <v>45</v>
       </c>
       <c r="C92" s="14" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D92" s="14" t="s">
         <v>436</v>
       </c>
       <c r="E92" s="14" t="s">
+        <v>412</v>
+      </c>
+      <c r="F92" s="14" t="s">
         <v>437</v>
       </c>
-      <c r="F92" s="14" t="s">
+      <c r="G92" s="14" t="s">
         <v>438</v>
-      </c>
-      <c r="G92" s="14" t="s">
-        <v>439</v>
       </c>
       <c r="H92" s="14" t="s">
         <v>78</v>
       </c>
       <c r="I92" s="14" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="J92" s="14" t="s">
         <v>80</v>
@@ -7765,33 +7791,33 @@
       <c r="N92" s="15"/>
       <c r="O92" s="15"/>
     </row>
-    <row r="93" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="93" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="14" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="B93" s="14" t="s">
         <v>45</v>
       </c>
       <c r="C93" s="14" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D93" s="14" t="s">
+        <v>440</v>
+      </c>
+      <c r="E93" s="14" t="s">
+        <v>412</v>
+      </c>
+      <c r="F93" s="14" t="s">
         <v>441</v>
       </c>
-      <c r="E93" s="14" t="s">
-        <v>437</v>
-      </c>
-      <c r="F93" s="14" t="s">
+      <c r="G93" s="14" t="s">
         <v>442</v>
-      </c>
-      <c r="G93" s="14" t="s">
-        <v>443</v>
       </c>
       <c r="H93" s="14" t="s">
         <v>78</v>
       </c>
       <c r="I93" s="14" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="J93" s="14" t="s">
         <v>80</v>
@@ -7804,9 +7830,9 @@
       <c r="N93" s="15"/>
       <c r="O93" s="15"/>
     </row>
-    <row r="94" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="94" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="14" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="B94" s="14" t="s">
         <v>45</v>
@@ -7815,22 +7841,22 @@
         <v>47</v>
       </c>
       <c r="D94" s="14" t="s">
+        <v>444</v>
+      </c>
+      <c r="E94" s="14" t="s">
         <v>445</v>
-      </c>
-      <c r="E94" s="14" t="s">
-        <v>437</v>
       </c>
       <c r="F94" s="14" t="s">
         <v>446</v>
       </c>
       <c r="G94" s="14" t="s">
-        <v>203</v>
+        <v>447</v>
       </c>
       <c r="H94" s="14" t="s">
         <v>78</v>
       </c>
       <c r="I94" s="14" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="J94" s="14" t="s">
         <v>80</v>
@@ -7845,7 +7871,7 @@
     </row>
     <row r="95" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="14" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="B95" s="14" t="s">
         <v>45</v>
@@ -7854,16 +7880,16 @@
         <v>47</v>
       </c>
       <c r="D95" s="14" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="E95" s="14" t="s">
-        <v>437</v>
+        <v>445</v>
       </c>
       <c r="F95" s="14" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="G95" s="14" t="s">
-        <v>203</v>
+        <v>451</v>
       </c>
       <c r="H95" s="14" t="s">
         <v>78</v>
@@ -7884,7 +7910,7 @@
     </row>
     <row r="96" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="14" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="B96" s="14" t="s">
         <v>45</v>
@@ -7893,13 +7919,13 @@
         <v>47</v>
       </c>
       <c r="D96" s="14" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="E96" s="14" t="s">
-        <v>437</v>
+        <v>445</v>
       </c>
       <c r="F96" s="14" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="G96" s="14" t="s">
         <v>203</v>
@@ -7921,9 +7947,9 @@
       <c r="N96" s="15"/>
       <c r="O96" s="15"/>
     </row>
-    <row r="97" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="97" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="14" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="B97" s="14" t="s">
         <v>45</v>
@@ -7932,22 +7958,22 @@
         <v>47</v>
       </c>
       <c r="D97" s="14" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="E97" s="14" t="s">
-        <v>437</v>
+        <v>445</v>
       </c>
       <c r="F97" s="14" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="G97" s="14" t="s">
-        <v>456</v>
+        <v>203</v>
       </c>
       <c r="H97" s="14" t="s">
         <v>78</v>
       </c>
       <c r="I97" s="14" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="J97" s="14" t="s">
         <v>80</v>
@@ -7962,7 +7988,7 @@
     </row>
     <row r="98" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="14" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="B98" s="14" t="s">
         <v>45</v>
@@ -7971,22 +7997,22 @@
         <v>47</v>
       </c>
       <c r="D98" s="14" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="E98" s="14" t="s">
-        <v>437</v>
+        <v>445</v>
       </c>
       <c r="F98" s="14" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="G98" s="14" t="s">
-        <v>460</v>
+        <v>203</v>
       </c>
       <c r="H98" s="14" t="s">
         <v>78</v>
       </c>
       <c r="I98" s="14" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="J98" s="14" t="s">
         <v>80</v>
@@ -7999,7 +8025,7 @@
       <c r="N98" s="15"/>
       <c r="O98" s="15"/>
     </row>
-    <row r="99" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="99" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="14" t="s">
         <v>461</v>
       </c>
@@ -8013,19 +8039,19 @@
         <v>462</v>
       </c>
       <c r="E99" s="14" t="s">
-        <v>437</v>
+        <v>445</v>
       </c>
       <c r="F99" s="14" t="s">
         <v>463</v>
       </c>
       <c r="G99" s="14" t="s">
-        <v>203</v>
+        <v>464</v>
       </c>
       <c r="H99" s="14" t="s">
         <v>78</v>
       </c>
       <c r="I99" s="14" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="J99" s="14" t="s">
         <v>80</v>
@@ -8040,7 +8066,7 @@
     </row>
     <row r="100" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="14" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="B100" s="14" t="s">
         <v>45</v>
@@ -8049,16 +8075,16 @@
         <v>47</v>
       </c>
       <c r="D100" s="14" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="E100" s="14" t="s">
-        <v>437</v>
+        <v>445</v>
       </c>
       <c r="F100" s="14" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="G100" s="14" t="s">
-        <v>439</v>
+        <v>468</v>
       </c>
       <c r="H100" s="14" t="s">
         <v>78</v>
@@ -8077,33 +8103,33 @@
       <c r="N100" s="15"/>
       <c r="O100" s="15"/>
     </row>
-    <row r="101" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="101" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="14" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="B101" s="14" t="s">
         <v>45</v>
       </c>
       <c r="C101" s="14" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D101" s="14" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="E101" s="14" t="s">
-        <v>404</v>
+        <v>445</v>
       </c>
       <c r="F101" s="14" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="G101" s="14" t="s">
-        <v>470</v>
+        <v>203</v>
       </c>
       <c r="H101" s="14" t="s">
         <v>78</v>
       </c>
       <c r="I101" s="14" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="J101" s="14" t="s">
         <v>80</v>
@@ -8116,27 +8142,27 @@
       <c r="N101" s="15"/>
       <c r="O101" s="15"/>
     </row>
-    <row r="102" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="102" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="14" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="B102" s="14" t="s">
         <v>45</v>
       </c>
       <c r="C102" s="14" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D102" s="14" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="E102" s="14" t="s">
-        <v>404</v>
+        <v>445</v>
       </c>
       <c r="F102" s="14" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="G102" s="14" t="s">
-        <v>474</v>
+        <v>447</v>
       </c>
       <c r="H102" s="14" t="s">
         <v>78</v>
@@ -8169,7 +8195,7 @@
         <v>476</v>
       </c>
       <c r="E103" s="14" t="s">
-        <v>404</v>
+        <v>412</v>
       </c>
       <c r="F103" s="14" t="s">
         <v>477</v>
@@ -8208,7 +8234,7 @@
         <v>480</v>
       </c>
       <c r="E104" s="14" t="s">
-        <v>404</v>
+        <v>412</v>
       </c>
       <c r="F104" s="14" t="s">
         <v>481</v>
@@ -8247,7 +8273,7 @@
         <v>484</v>
       </c>
       <c r="E105" s="14" t="s">
-        <v>404</v>
+        <v>412</v>
       </c>
       <c r="F105" s="14" t="s">
         <v>485</v>
@@ -8259,7 +8285,7 @@
         <v>78</v>
       </c>
       <c r="I105" s="14" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="J105" s="14" t="s">
         <v>80</v>
@@ -8286,7 +8312,7 @@
         <v>488</v>
       </c>
       <c r="E106" s="14" t="s">
-        <v>404</v>
+        <v>412</v>
       </c>
       <c r="F106" s="14" t="s">
         <v>489</v>
@@ -8298,7 +8324,7 @@
         <v>78</v>
       </c>
       <c r="I106" s="14" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="J106" s="14" t="s">
         <v>80</v>
@@ -8325,7 +8351,7 @@
         <v>492</v>
       </c>
       <c r="E107" s="14" t="s">
-        <v>404</v>
+        <v>412</v>
       </c>
       <c r="F107" s="14" t="s">
         <v>493</v>
@@ -8337,7 +8363,7 @@
         <v>78</v>
       </c>
       <c r="I107" s="14" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="J107" s="14" t="s">
         <v>80</v>
@@ -8364,7 +8390,7 @@
         <v>496</v>
       </c>
       <c r="E108" s="14" t="s">
-        <v>404</v>
+        <v>412</v>
       </c>
       <c r="F108" s="14" t="s">
         <v>497</v>
@@ -8389,7 +8415,7 @@
       <c r="N108" s="15"/>
       <c r="O108" s="15"/>
     </row>
-    <row r="109" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="109" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="14" t="s">
         <v>499</v>
       </c>
@@ -8397,19 +8423,19 @@
         <v>45</v>
       </c>
       <c r="C109" s="14" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D109" s="14" t="s">
         <v>500</v>
       </c>
       <c r="E109" s="14" t="s">
+        <v>412</v>
+      </c>
+      <c r="F109" s="14" t="s">
         <v>501</v>
       </c>
-      <c r="F109" s="14" t="s">
+      <c r="G109" s="14" t="s">
         <v>502</v>
-      </c>
-      <c r="G109" s="14" t="s">
-        <v>503</v>
       </c>
       <c r="H109" s="14" t="s">
         <v>78</v>
@@ -8428,33 +8454,33 @@
       <c r="N109" s="15"/>
       <c r="O109" s="15"/>
     </row>
-    <row r="110" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="110" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="14" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="B110" s="14" t="s">
         <v>45</v>
       </c>
       <c r="C110" s="14" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D110" s="14" t="s">
+        <v>504</v>
+      </c>
+      <c r="E110" s="14" t="s">
+        <v>412</v>
+      </c>
+      <c r="F110" s="14" t="s">
         <v>505</v>
       </c>
-      <c r="E110" s="14" t="s">
-        <v>501</v>
-      </c>
-      <c r="F110" s="14" t="s">
+      <c r="G110" s="14" t="s">
         <v>506</v>
-      </c>
-      <c r="G110" s="14" t="s">
-        <v>507</v>
       </c>
       <c r="H110" s="14" t="s">
         <v>78</v>
       </c>
       <c r="I110" s="14" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="J110" s="14" t="s">
         <v>80</v>
@@ -8467,27 +8493,27 @@
       <c r="N110" s="15"/>
       <c r="O110" s="15"/>
     </row>
-    <row r="111" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="111" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="14" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="B111" s="14" t="s">
         <v>45</v>
       </c>
       <c r="C111" s="14" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D111" s="14" t="s">
+        <v>508</v>
+      </c>
+      <c r="E111" s="14" t="s">
         <v>509</v>
       </c>
-      <c r="E111" s="14" t="s">
+      <c r="F111" s="14" t="s">
         <v>510</v>
       </c>
-      <c r="F111" s="14" t="s">
+      <c r="G111" s="14" t="s">
         <v>511</v>
-      </c>
-      <c r="G111" s="14" t="s">
-        <v>512</v>
       </c>
       <c r="H111" s="14" t="s">
         <v>78</v>
@@ -8499,7 +8525,7 @@
         <v>80</v>
       </c>
       <c r="K111" s="14" t="s">
-        <v>513</v>
+        <v>81</v>
       </c>
       <c r="L111" s="15"/>
       <c r="M111" s="15"/>
@@ -8508,25 +8534,25 @@
     </row>
     <row r="112" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="14" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
       <c r="B112" s="14" t="s">
         <v>45</v>
       </c>
       <c r="C112" s="14" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D112" s="14" t="s">
+        <v>513</v>
+      </c>
+      <c r="E112" s="14" t="s">
+        <v>509</v>
+      </c>
+      <c r="F112" s="14" t="s">
+        <v>514</v>
+      </c>
+      <c r="G112" s="14" t="s">
         <v>515</v>
-      </c>
-      <c r="E112" s="14" t="s">
-        <v>510</v>
-      </c>
-      <c r="F112" s="14" t="s">
-        <v>516</v>
-      </c>
-      <c r="G112" s="14" t="s">
-        <v>517</v>
       </c>
       <c r="H112" s="14" t="s">
         <v>78</v>
@@ -8538,82 +8564,86 @@
         <v>80</v>
       </c>
       <c r="K112" s="14" t="s">
-        <v>518</v>
+        <v>81</v>
       </c>
       <c r="L112" s="15"/>
       <c r="M112" s="15"/>
       <c r="N112" s="15"/>
       <c r="O112" s="15"/>
     </row>
-    <row r="113" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="113" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="14" t="s">
+        <v>516</v>
+      </c>
+      <c r="B113" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="C113" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="D113" s="14" t="s">
+        <v>517</v>
+      </c>
+      <c r="E113" s="14" t="s">
+        <v>518</v>
+      </c>
+      <c r="F113" s="14" t="s">
         <v>519</v>
       </c>
-      <c r="B113" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="C113" s="14" t="s">
-        <v>37</v>
-      </c>
-      <c r="D113" s="14" t="s">
+      <c r="G113" s="14" t="s">
         <v>520</v>
-      </c>
-      <c r="E113" s="14" t="s">
-        <v>521</v>
-      </c>
-      <c r="F113" s="14" t="s">
-        <v>522</v>
-      </c>
-      <c r="G113" s="14" t="s">
-        <v>523</v>
       </c>
       <c r="H113" s="14" t="s">
         <v>78</v>
       </c>
       <c r="I113" s="14" t="s">
-        <v>524</v>
+        <v>79</v>
       </c>
       <c r="J113" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="K113" s="14"/>
+        <v>80</v>
+      </c>
+      <c r="K113" s="14" t="s">
+        <v>521</v>
+      </c>
       <c r="L113" s="15"/>
       <c r="M113" s="15"/>
       <c r="N113" s="15"/>
       <c r="O113" s="15"/>
     </row>
-    <row r="114" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="114" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="14" t="s">
+        <v>522</v>
+      </c>
+      <c r="B114" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="C114" s="14" t="s">
+        <v>46</v>
+      </c>
+      <c r="D114" s="14" t="s">
+        <v>523</v>
+      </c>
+      <c r="E114" s="14" t="s">
+        <v>518</v>
+      </c>
+      <c r="F114" s="14" t="s">
+        <v>524</v>
+      </c>
+      <c r="G114" s="14" t="s">
         <v>525</v>
-      </c>
-      <c r="B114" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="C114" s="14" t="s">
-        <v>37</v>
-      </c>
-      <c r="D114" s="14" t="s">
-        <v>526</v>
-      </c>
-      <c r="E114" s="14" t="s">
-        <v>521</v>
-      </c>
-      <c r="F114" s="14" t="s">
-        <v>527</v>
-      </c>
-      <c r="G114" s="14" t="s">
-        <v>528</v>
       </c>
       <c r="H114" s="14" t="s">
         <v>78</v>
       </c>
       <c r="I114" s="14" t="s">
-        <v>524</v>
+        <v>79</v>
       </c>
       <c r="J114" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="K114" s="14"/>
+        <v>80</v>
+      </c>
+      <c r="K114" s="14" t="s">
+        <v>526</v>
+      </c>
       <c r="L114" s="15"/>
       <c r="M114" s="15"/>
       <c r="N114" s="15"/>
@@ -8621,7 +8651,7 @@
     </row>
     <row r="115" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="14" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="B115" s="14" t="s">
         <v>20</v>
@@ -8630,22 +8660,22 @@
         <v>37</v>
       </c>
       <c r="D115" s="14" t="s">
+        <v>528</v>
+      </c>
+      <c r="E115" s="14" t="s">
+        <v>529</v>
+      </c>
+      <c r="F115" s="14" t="s">
         <v>530</v>
       </c>
-      <c r="E115" s="14" t="s">
-        <v>521</v>
-      </c>
-      <c r="F115" s="14" t="s">
+      <c r="G115" s="14" t="s">
         <v>531</v>
-      </c>
-      <c r="G115" s="14" t="s">
-        <v>532</v>
       </c>
       <c r="H115" s="14" t="s">
         <v>78</v>
       </c>
       <c r="I115" s="14" t="s">
-        <v>524</v>
+        <v>532</v>
       </c>
       <c r="J115" s="14" t="s">
         <v>16</v>
@@ -8664,13 +8694,13 @@
         <v>20</v>
       </c>
       <c r="C116" s="14" t="s">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="D116" s="14" t="s">
         <v>534</v>
       </c>
       <c r="E116" s="14" t="s">
-        <v>521</v>
+        <v>529</v>
       </c>
       <c r="F116" s="14" t="s">
         <v>535</v>
@@ -8679,10 +8709,10 @@
         <v>536</v>
       </c>
       <c r="H116" s="14" t="s">
-        <v>164</v>
+        <v>78</v>
       </c>
       <c r="I116" s="14" t="s">
-        <v>524</v>
+        <v>532</v>
       </c>
       <c r="J116" s="14" t="s">
         <v>16</v>
@@ -8701,13 +8731,13 @@
         <v>20</v>
       </c>
       <c r="C117" s="14" t="s">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="D117" s="14" t="s">
         <v>538</v>
       </c>
       <c r="E117" s="14" t="s">
-        <v>521</v>
+        <v>529</v>
       </c>
       <c r="F117" s="14" t="s">
         <v>539</v>
@@ -8716,10 +8746,10 @@
         <v>540</v>
       </c>
       <c r="H117" s="14" t="s">
-        <v>164</v>
+        <v>78</v>
       </c>
       <c r="I117" s="14" t="s">
-        <v>524</v>
+        <v>532</v>
       </c>
       <c r="J117" s="14" t="s">
         <v>16</v>
@@ -8738,13 +8768,13 @@
         <v>20</v>
       </c>
       <c r="C118" s="14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D118" s="14" t="s">
         <v>542</v>
       </c>
       <c r="E118" s="14" t="s">
-        <v>521</v>
+        <v>529</v>
       </c>
       <c r="F118" s="14" t="s">
         <v>543</v>
@@ -8756,7 +8786,7 @@
         <v>164</v>
       </c>
       <c r="I118" s="14" t="s">
-        <v>524</v>
+        <v>532</v>
       </c>
       <c r="J118" s="14" t="s">
         <v>16</v>
@@ -8781,7 +8811,7 @@
         <v>546</v>
       </c>
       <c r="E119" s="14" t="s">
-        <v>521</v>
+        <v>529</v>
       </c>
       <c r="F119" s="14" t="s">
         <v>547</v>
@@ -8790,10 +8820,10 @@
         <v>548</v>
       </c>
       <c r="H119" s="14" t="s">
-        <v>78</v>
+        <v>164</v>
       </c>
       <c r="I119" s="14" t="s">
-        <v>549</v>
+        <v>532</v>
       </c>
       <c r="J119" s="14" t="s">
         <v>16</v>
@@ -8806,31 +8836,31 @@
     </row>
     <row r="120" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="14" t="s">
+        <v>549</v>
+      </c>
+      <c r="B120" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="C120" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="D120" s="14" t="s">
         <v>550</v>
       </c>
-      <c r="B120" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="C120" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="D120" s="14" t="s">
+      <c r="E120" s="14" t="s">
+        <v>529</v>
+      </c>
+      <c r="F120" s="14" t="s">
         <v>551</v>
       </c>
-      <c r="E120" s="14" t="s">
-        <v>521</v>
-      </c>
-      <c r="F120" s="14" t="s">
+      <c r="G120" s="14" t="s">
         <v>552</v>
       </c>
-      <c r="G120" s="14" t="s">
-        <v>553</v>
-      </c>
       <c r="H120" s="14" t="s">
-        <v>78</v>
+        <v>164</v>
       </c>
       <c r="I120" s="14" t="s">
-        <v>554</v>
+        <v>532</v>
       </c>
       <c r="J120" s="14" t="s">
         <v>16</v>
@@ -8843,31 +8873,31 @@
     </row>
     <row r="121" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="14" t="s">
+        <v>553</v>
+      </c>
+      <c r="B121" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="C121" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="D121" s="14" t="s">
+        <v>554</v>
+      </c>
+      <c r="E121" s="14" t="s">
+        <v>529</v>
+      </c>
+      <c r="F121" s="14" t="s">
         <v>555</v>
       </c>
-      <c r="B121" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="C121" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="D121" s="14" t="s">
+      <c r="G121" s="14" t="s">
         <v>556</v>
       </c>
-      <c r="E121" s="14" t="s">
-        <v>521</v>
-      </c>
-      <c r="F121" s="14" t="s">
+      <c r="H121" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="I121" s="14" t="s">
         <v>557</v>
-      </c>
-      <c r="G121" s="14" t="s">
-        <v>558</v>
-      </c>
-      <c r="H121" s="14" t="s">
-        <v>164</v>
-      </c>
-      <c r="I121" s="14" t="s">
-        <v>524</v>
       </c>
       <c r="J121" s="14" t="s">
         <v>16</v>
@@ -8880,31 +8910,31 @@
     </row>
     <row r="122" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="14" t="s">
+        <v>558</v>
+      </c>
+      <c r="B122" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="C122" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="D122" s="14" t="s">
         <v>559</v>
       </c>
-      <c r="B122" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="C122" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="D122" s="14" t="s">
+      <c r="E122" s="14" t="s">
+        <v>529</v>
+      </c>
+      <c r="F122" s="14" t="s">
         <v>560</v>
       </c>
-      <c r="E122" s="14" t="s">
-        <v>521</v>
-      </c>
-      <c r="F122" s="14" t="s">
+      <c r="G122" s="14" t="s">
         <v>561</v>
       </c>
-      <c r="G122" s="14" t="s">
+      <c r="H122" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="I122" s="14" t="s">
         <v>562</v>
-      </c>
-      <c r="H122" s="14" t="s">
-        <v>164</v>
-      </c>
-      <c r="I122" s="14" t="s">
-        <v>524</v>
       </c>
       <c r="J122" s="14" t="s">
         <v>16</v>
@@ -8923,13 +8953,13 @@
         <v>20</v>
       </c>
       <c r="C123" s="14" t="s">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="D123" s="14" t="s">
         <v>564</v>
       </c>
       <c r="E123" s="14" t="s">
-        <v>521</v>
+        <v>529</v>
       </c>
       <c r="F123" s="14" t="s">
         <v>565</v>
@@ -8941,7 +8971,7 @@
         <v>164</v>
       </c>
       <c r="I123" s="14" t="s">
-        <v>524</v>
+        <v>532</v>
       </c>
       <c r="J123" s="14" t="s">
         <v>16</v>
@@ -8960,13 +8990,13 @@
         <v>20</v>
       </c>
       <c r="C124" s="14" t="s">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="D124" s="14" t="s">
         <v>568</v>
       </c>
       <c r="E124" s="14" t="s">
-        <v>521</v>
+        <v>529</v>
       </c>
       <c r="F124" s="14" t="s">
         <v>569</v>
@@ -8975,10 +9005,10 @@
         <v>570</v>
       </c>
       <c r="H124" s="14" t="s">
-        <v>78</v>
+        <v>164</v>
       </c>
       <c r="I124" s="14" t="s">
-        <v>571</v>
+        <v>532</v>
       </c>
       <c r="J124" s="14" t="s">
         <v>16</v>
@@ -8991,31 +9021,31 @@
     </row>
     <row r="125" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="14" t="s">
+        <v>571</v>
+      </c>
+      <c r="B125" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="C125" s="14" t="s">
+        <v>38</v>
+      </c>
+      <c r="D125" s="14" t="s">
         <v>572</v>
       </c>
-      <c r="B125" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="C125" s="14" t="s">
-        <v>28</v>
-      </c>
-      <c r="D125" s="14" t="s">
+      <c r="E125" s="14" t="s">
+        <v>529</v>
+      </c>
+      <c r="F125" s="14" t="s">
         <v>573</v>
       </c>
-      <c r="E125" s="14" t="s">
-        <v>521</v>
-      </c>
-      <c r="F125" s="14" t="s">
+      <c r="G125" s="14" t="s">
         <v>574</v>
-      </c>
-      <c r="G125" s="14" t="s">
-        <v>575</v>
       </c>
       <c r="H125" s="14" t="s">
         <v>164</v>
       </c>
       <c r="I125" s="14" t="s">
-        <v>524</v>
+        <v>532</v>
       </c>
       <c r="J125" s="14" t="s">
         <v>16</v>
@@ -9028,31 +9058,31 @@
     </row>
     <row r="126" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="14" t="s">
+        <v>575</v>
+      </c>
+      <c r="B126" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="C126" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="D126" s="14" t="s">
         <v>576</v>
       </c>
-      <c r="B126" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="C126" s="14" t="s">
-        <v>29</v>
-      </c>
-      <c r="D126" s="14" t="s">
+      <c r="E126" s="14" t="s">
+        <v>529</v>
+      </c>
+      <c r="F126" s="14" t="s">
         <v>577</v>
       </c>
-      <c r="E126" s="14" t="s">
-        <v>521</v>
-      </c>
-      <c r="F126" s="14" t="s">
+      <c r="G126" s="14" t="s">
         <v>578</v>
       </c>
-      <c r="G126" s="14" t="s">
+      <c r="H126" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="I126" s="14" t="s">
         <v>579</v>
-      </c>
-      <c r="H126" s="14" t="s">
-        <v>164</v>
-      </c>
-      <c r="I126" s="14" t="s">
-        <v>524</v>
       </c>
       <c r="J126" s="14" t="s">
         <v>16</v>
@@ -9071,13 +9101,13 @@
         <v>20</v>
       </c>
       <c r="C127" s="14" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D127" s="14" t="s">
         <v>581</v>
       </c>
       <c r="E127" s="14" t="s">
-        <v>521</v>
+        <v>529</v>
       </c>
       <c r="F127" s="14" t="s">
         <v>582</v>
@@ -9089,7 +9119,7 @@
         <v>164</v>
       </c>
       <c r="I127" s="14" t="s">
-        <v>524</v>
+        <v>532</v>
       </c>
       <c r="J127" s="14" t="s">
         <v>16</v>
@@ -9108,13 +9138,13 @@
         <v>20</v>
       </c>
       <c r="C128" s="14" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D128" s="14" t="s">
         <v>585</v>
       </c>
       <c r="E128" s="14" t="s">
-        <v>521</v>
+        <v>529</v>
       </c>
       <c r="F128" s="14" t="s">
         <v>586</v>
@@ -9126,7 +9156,7 @@
         <v>164</v>
       </c>
       <c r="I128" s="14" t="s">
-        <v>524</v>
+        <v>532</v>
       </c>
       <c r="J128" s="14" t="s">
         <v>16</v>
@@ -9145,13 +9175,13 @@
         <v>20</v>
       </c>
       <c r="C129" s="14" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D129" s="14" t="s">
         <v>589</v>
       </c>
       <c r="E129" s="14" t="s">
-        <v>521</v>
+        <v>529</v>
       </c>
       <c r="F129" s="14" t="s">
         <v>590</v>
@@ -9163,7 +9193,7 @@
         <v>164</v>
       </c>
       <c r="I129" s="14" t="s">
-        <v>524</v>
+        <v>532</v>
       </c>
       <c r="J129" s="14" t="s">
         <v>16</v>
@@ -9182,13 +9212,13 @@
         <v>20</v>
       </c>
       <c r="C130" s="14" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D130" s="14" t="s">
         <v>593</v>
       </c>
       <c r="E130" s="14" t="s">
-        <v>521</v>
+        <v>529</v>
       </c>
       <c r="F130" s="14" t="s">
         <v>594</v>
@@ -9200,7 +9230,7 @@
         <v>164</v>
       </c>
       <c r="I130" s="14" t="s">
-        <v>524</v>
+        <v>532</v>
       </c>
       <c r="J130" s="14" t="s">
         <v>16</v>
@@ -9219,13 +9249,13 @@
         <v>20</v>
       </c>
       <c r="C131" s="14" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D131" s="14" t="s">
         <v>597</v>
       </c>
       <c r="E131" s="14" t="s">
-        <v>521</v>
+        <v>529</v>
       </c>
       <c r="F131" s="14" t="s">
         <v>598</v>
@@ -9234,10 +9264,10 @@
         <v>599</v>
       </c>
       <c r="H131" s="14" t="s">
-        <v>600</v>
+        <v>164</v>
       </c>
       <c r="I131" s="14" t="s">
-        <v>549</v>
+        <v>532</v>
       </c>
       <c r="J131" s="14" t="s">
         <v>16</v>
@@ -9250,31 +9280,31 @@
     </row>
     <row r="132" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="14" t="s">
+        <v>600</v>
+      </c>
+      <c r="B132" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="C132" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D132" s="14" t="s">
         <v>601</v>
       </c>
-      <c r="B132" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="C132" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="D132" s="14" t="s">
+      <c r="E132" s="14" t="s">
+        <v>529</v>
+      </c>
+      <c r="F132" s="14" t="s">
         <v>602</v>
       </c>
-      <c r="E132" s="14" t="s">
-        <v>521</v>
-      </c>
-      <c r="F132" s="14" t="s">
+      <c r="G132" s="14" t="s">
         <v>603</v>
       </c>
-      <c r="G132" s="14" t="s">
-        <v>604</v>
-      </c>
       <c r="H132" s="14" t="s">
-        <v>78</v>
+        <v>164</v>
       </c>
       <c r="I132" s="14" t="s">
-        <v>524</v>
+        <v>532</v>
       </c>
       <c r="J132" s="14" t="s">
         <v>16</v>
@@ -9287,31 +9317,31 @@
     </row>
     <row r="133" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="14" t="s">
+        <v>604</v>
+      </c>
+      <c r="B133" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="C133" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D133" s="14" t="s">
         <v>605</v>
       </c>
-      <c r="B133" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="C133" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="D133" s="14" t="s">
+      <c r="E133" s="14" t="s">
+        <v>529</v>
+      </c>
+      <c r="F133" s="14" t="s">
         <v>606</v>
       </c>
-      <c r="E133" s="14" t="s">
-        <v>521</v>
-      </c>
-      <c r="F133" s="14" t="s">
+      <c r="G133" s="14" t="s">
         <v>607</v>
       </c>
-      <c r="G133" s="14" t="s">
+      <c r="H133" s="14" t="s">
         <v>608</v>
       </c>
-      <c r="H133" s="14" t="s">
-        <v>600</v>
-      </c>
       <c r="I133" s="14" t="s">
-        <v>549</v>
+        <v>557</v>
       </c>
       <c r="J133" s="14" t="s">
         <v>16</v>
@@ -9322,7 +9352,7 @@
       <c r="N133" s="15"/>
       <c r="O133" s="15"/>
     </row>
-    <row r="134" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="134" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="14" t="s">
         <v>609</v>
       </c>
@@ -9330,13 +9360,13 @@
         <v>20</v>
       </c>
       <c r="C134" s="14" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="D134" s="14" t="s">
         <v>610</v>
       </c>
       <c r="E134" s="14" t="s">
-        <v>521</v>
+        <v>529</v>
       </c>
       <c r="F134" s="14" t="s">
         <v>611</v>
@@ -9345,10 +9375,10 @@
         <v>612</v>
       </c>
       <c r="H134" s="14" t="s">
-        <v>164</v>
+        <v>78</v>
       </c>
       <c r="I134" s="14" t="s">
-        <v>524</v>
+        <v>532</v>
       </c>
       <c r="J134" s="14" t="s">
         <v>16</v>
@@ -9359,7 +9389,7 @@
       <c r="N134" s="15"/>
       <c r="O134" s="15"/>
     </row>
-    <row r="135" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="135" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="14" t="s">
         <v>613</v>
       </c>
@@ -9367,13 +9397,13 @@
         <v>20</v>
       </c>
       <c r="C135" s="14" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D135" s="14" t="s">
         <v>614</v>
       </c>
       <c r="E135" s="14" t="s">
-        <v>521</v>
+        <v>529</v>
       </c>
       <c r="F135" s="14" t="s">
         <v>615</v>
@@ -9382,10 +9412,10 @@
         <v>616</v>
       </c>
       <c r="H135" s="14" t="s">
-        <v>78</v>
+        <v>608</v>
       </c>
       <c r="I135" s="14" t="s">
-        <v>524</v>
+        <v>557</v>
       </c>
       <c r="J135" s="14" t="s">
         <v>16</v>
@@ -9396,7 +9426,7 @@
       <c r="N135" s="15"/>
       <c r="O135" s="15"/>
     </row>
-    <row r="136" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="136" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="14" t="s">
         <v>617</v>
       </c>
@@ -9404,13 +9434,13 @@
         <v>20</v>
       </c>
       <c r="C136" s="14" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="D136" s="14" t="s">
         <v>618</v>
       </c>
       <c r="E136" s="14" t="s">
-        <v>521</v>
+        <v>529</v>
       </c>
       <c r="F136" s="14" t="s">
         <v>619</v>
@@ -9422,7 +9452,7 @@
         <v>164</v>
       </c>
       <c r="I136" s="14" t="s">
-        <v>524</v>
+        <v>532</v>
       </c>
       <c r="J136" s="14" t="s">
         <v>16</v>
@@ -9441,13 +9471,13 @@
         <v>20</v>
       </c>
       <c r="C137" s="14" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="D137" s="14" t="s">
         <v>622</v>
       </c>
       <c r="E137" s="14" t="s">
-        <v>521</v>
+        <v>529</v>
       </c>
       <c r="F137" s="14" t="s">
         <v>623</v>
@@ -9456,10 +9486,10 @@
         <v>624</v>
       </c>
       <c r="H137" s="14" t="s">
-        <v>164</v>
+        <v>78</v>
       </c>
       <c r="I137" s="14" t="s">
-        <v>524</v>
+        <v>532</v>
       </c>
       <c r="J137" s="14" t="s">
         <v>16</v>
@@ -9484,7 +9514,7 @@
         <v>626</v>
       </c>
       <c r="E138" s="14" t="s">
-        <v>521</v>
+        <v>529</v>
       </c>
       <c r="F138" s="14" t="s">
         <v>627</v>
@@ -9496,7 +9526,7 @@
         <v>164</v>
       </c>
       <c r="I138" s="14" t="s">
-        <v>524</v>
+        <v>532</v>
       </c>
       <c r="J138" s="14" t="s">
         <v>16</v>
@@ -9515,13 +9545,13 @@
         <v>20</v>
       </c>
       <c r="C139" s="14" t="s">
-        <v>41</v>
+        <v>21</v>
       </c>
       <c r="D139" s="14" t="s">
         <v>630</v>
       </c>
       <c r="E139" s="14" t="s">
-        <v>521</v>
+        <v>529</v>
       </c>
       <c r="F139" s="14" t="s">
         <v>631</v>
@@ -9530,10 +9560,10 @@
         <v>632</v>
       </c>
       <c r="H139" s="14" t="s">
-        <v>78</v>
+        <v>164</v>
       </c>
       <c r="I139" s="14" t="s">
-        <v>554</v>
+        <v>532</v>
       </c>
       <c r="J139" s="14" t="s">
         <v>16</v>
@@ -9544,21 +9574,21 @@
       <c r="N139" s="15"/>
       <c r="O139" s="15"/>
     </row>
-    <row r="140" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="140" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="14" t="s">
         <v>633</v>
       </c>
       <c r="B140" s="14" t="s">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="C140" s="14" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="D140" s="14" t="s">
         <v>634</v>
       </c>
       <c r="E140" s="14" t="s">
-        <v>521</v>
+        <v>529</v>
       </c>
       <c r="F140" s="14" t="s">
         <v>635</v>
@@ -9570,7 +9600,7 @@
         <v>164</v>
       </c>
       <c r="I140" s="14" t="s">
-        <v>554</v>
+        <v>532</v>
       </c>
       <c r="J140" s="14" t="s">
         <v>16</v>
@@ -9581,7 +9611,7 @@
       <c r="N140" s="15"/>
       <c r="O140" s="15"/>
     </row>
-    <row r="141" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="141" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="14" t="s">
         <v>637</v>
       </c>
@@ -9589,13 +9619,13 @@
         <v>20</v>
       </c>
       <c r="C141" s="14" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D141" s="14" t="s">
         <v>638</v>
       </c>
       <c r="E141" s="14" t="s">
-        <v>521</v>
+        <v>529</v>
       </c>
       <c r="F141" s="14" t="s">
         <v>639</v>
@@ -9604,10 +9634,10 @@
         <v>640</v>
       </c>
       <c r="H141" s="14" t="s">
-        <v>164</v>
+        <v>78</v>
       </c>
       <c r="I141" s="14" t="s">
-        <v>549</v>
+        <v>562</v>
       </c>
       <c r="J141" s="14" t="s">
         <v>16</v>
@@ -9618,21 +9648,21 @@
       <c r="N141" s="15"/>
       <c r="O141" s="15"/>
     </row>
-    <row r="142" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="142" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="14" t="s">
         <v>641</v>
       </c>
       <c r="B142" s="14" t="s">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="C142" s="14" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="D142" s="14" t="s">
         <v>642</v>
       </c>
       <c r="E142" s="14" t="s">
-        <v>521</v>
+        <v>529</v>
       </c>
       <c r="F142" s="14" t="s">
         <v>643</v>
@@ -9641,10 +9671,10 @@
         <v>644</v>
       </c>
       <c r="H142" s="14" t="s">
-        <v>600</v>
+        <v>164</v>
       </c>
       <c r="I142" s="14" t="s">
-        <v>549</v>
+        <v>562</v>
       </c>
       <c r="J142" s="14" t="s">
         <v>16</v>
@@ -9660,16 +9690,16 @@
         <v>645</v>
       </c>
       <c r="B143" s="14" t="s">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="C143" s="14" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="D143" s="14" t="s">
         <v>646</v>
       </c>
       <c r="E143" s="14" t="s">
-        <v>521</v>
+        <v>529</v>
       </c>
       <c r="F143" s="14" t="s">
         <v>647</v>
@@ -9678,10 +9708,10 @@
         <v>648</v>
       </c>
       <c r="H143" s="14" t="s">
-        <v>78</v>
+        <v>164</v>
       </c>
       <c r="I143" s="14" t="s">
-        <v>554</v>
+        <v>557</v>
       </c>
       <c r="J143" s="14" t="s">
         <v>16</v>
@@ -9697,16 +9727,16 @@
         <v>649</v>
       </c>
       <c r="B144" s="14" t="s">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="C144" s="14" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="D144" s="14" t="s">
         <v>650</v>
       </c>
       <c r="E144" s="14" t="s">
-        <v>521</v>
+        <v>529</v>
       </c>
       <c r="F144" s="14" t="s">
         <v>651</v>
@@ -9715,10 +9745,10 @@
         <v>652</v>
       </c>
       <c r="H144" s="14" t="s">
-        <v>78</v>
+        <v>608</v>
       </c>
       <c r="I144" s="14" t="s">
-        <v>554</v>
+        <v>557</v>
       </c>
       <c r="J144" s="14" t="s">
         <v>16</v>
@@ -9743,7 +9773,7 @@
         <v>654</v>
       </c>
       <c r="E145" s="14" t="s">
-        <v>521</v>
+        <v>529</v>
       </c>
       <c r="F145" s="14" t="s">
         <v>655</v>
@@ -9755,7 +9785,7 @@
         <v>78</v>
       </c>
       <c r="I145" s="14" t="s">
-        <v>554</v>
+        <v>562</v>
       </c>
       <c r="J145" s="14" t="s">
         <v>16</v>
@@ -9780,7 +9810,7 @@
         <v>658</v>
       </c>
       <c r="E146" s="14" t="s">
-        <v>521</v>
+        <v>529</v>
       </c>
       <c r="F146" s="14" t="s">
         <v>659</v>
@@ -9789,10 +9819,10 @@
         <v>660</v>
       </c>
       <c r="H146" s="14" t="s">
-        <v>164</v>
+        <v>78</v>
       </c>
       <c r="I146" s="14" t="s">
-        <v>554</v>
+        <v>562</v>
       </c>
       <c r="J146" s="14" t="s">
         <v>16</v>
@@ -9808,16 +9838,16 @@
         <v>661</v>
       </c>
       <c r="B147" s="14" t="s">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="C147" s="14" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="D147" s="14" t="s">
         <v>662</v>
       </c>
       <c r="E147" s="14" t="s">
-        <v>521</v>
+        <v>529</v>
       </c>
       <c r="F147" s="14" t="s">
         <v>663</v>
@@ -9826,10 +9856,10 @@
         <v>664</v>
       </c>
       <c r="H147" s="14" t="s">
-        <v>164</v>
+        <v>78</v>
       </c>
       <c r="I147" s="14" t="s">
-        <v>43</v>
+        <v>562</v>
       </c>
       <c r="J147" s="14" t="s">
         <v>16</v>
@@ -9845,16 +9875,16 @@
         <v>665</v>
       </c>
       <c r="B148" s="14" t="s">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="C148" s="14" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="D148" s="14" t="s">
         <v>666</v>
       </c>
       <c r="E148" s="14" t="s">
-        <v>521</v>
+        <v>529</v>
       </c>
       <c r="F148" s="14" t="s">
         <v>667</v>
@@ -9863,10 +9893,10 @@
         <v>668</v>
       </c>
       <c r="H148" s="14" t="s">
-        <v>78</v>
+        <v>164</v>
       </c>
       <c r="I148" s="14" t="s">
-        <v>79</v>
+        <v>562</v>
       </c>
       <c r="J148" s="14" t="s">
         <v>16</v>
@@ -9885,13 +9915,13 @@
         <v>20</v>
       </c>
       <c r="C149" s="14" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="D149" s="14" t="s">
         <v>670</v>
       </c>
       <c r="E149" s="14" t="s">
-        <v>521</v>
+        <v>529</v>
       </c>
       <c r="F149" s="14" t="s">
         <v>671</v>
@@ -9900,10 +9930,10 @@
         <v>672</v>
       </c>
       <c r="H149" s="14" t="s">
-        <v>78</v>
+        <v>164</v>
       </c>
       <c r="I149" s="14" t="s">
-        <v>79</v>
+        <v>43</v>
       </c>
       <c r="J149" s="14" t="s">
         <v>16</v>
@@ -9928,7 +9958,7 @@
         <v>674</v>
       </c>
       <c r="E150" s="14" t="s">
-        <v>521</v>
+        <v>529</v>
       </c>
       <c r="F150" s="14" t="s">
         <v>675</v>
@@ -9937,7 +9967,7 @@
         <v>676</v>
       </c>
       <c r="H150" s="14" t="s">
-        <v>164</v>
+        <v>78</v>
       </c>
       <c r="I150" s="14" t="s">
         <v>79</v>
@@ -9951,9 +9981,83 @@
       <c r="N150" s="15"/>
       <c r="O150" s="15"/>
     </row>
+    <row r="151" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A151" s="14" t="s">
+        <v>677</v>
+      </c>
+      <c r="B151" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="C151" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="D151" s="14" t="s">
+        <v>678</v>
+      </c>
+      <c r="E151" s="14" t="s">
+        <v>529</v>
+      </c>
+      <c r="F151" s="14" t="s">
+        <v>679</v>
+      </c>
+      <c r="G151" s="14" t="s">
+        <v>680</v>
+      </c>
+      <c r="H151" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="I151" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="J151" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="K151" s="14"/>
+      <c r="L151" s="15"/>
+      <c r="M151" s="15"/>
+      <c r="N151" s="15"/>
+      <c r="O151" s="15"/>
+    </row>
+    <row r="152" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A152" s="14" t="s">
+        <v>681</v>
+      </c>
+      <c r="B152" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="C152" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="D152" s="14" t="s">
+        <v>682</v>
+      </c>
+      <c r="E152" s="14" t="s">
+        <v>529</v>
+      </c>
+      <c r="F152" s="14" t="s">
+        <v>683</v>
+      </c>
+      <c r="G152" s="14" t="s">
+        <v>684</v>
+      </c>
+      <c r="H152" s="14" t="s">
+        <v>164</v>
+      </c>
+      <c r="I152" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="J152" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="K152" s="14"/>
+      <c r="L152" s="15"/>
+      <c r="M152" s="15"/>
+      <c r="N152" s="15"/>
+      <c r="O152" s="15"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O150"/>
-  <conditionalFormatting sqref="J2:J150">
+  <autoFilter ref="A1:O152"/>
+  <conditionalFormatting sqref="J2:J152">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
       <formula>"Pass"</formula>
     </cfRule>
@@ -9964,7 +10068,7 @@
       <formula>"Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L2:L150">
+  <conditionalFormatting sqref="L2:L152">
     <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
       <formula>"Pass"</formula>
     </cfRule>
@@ -9976,11 +10080,11 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L2:L150" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L2:L152" type="list">
       <formula1>"Pass,Fail,Blocked,Not Run"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H2:H150" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H2:H152" type="list">
       <formula1>"High,Medium,Low"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -10012,318 +10116,318 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="16" t="s">
-        <v>677</v>
+        <v>685</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="13" t="s">
-        <v>678</v>
+        <v>686</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="13" t="s">
-        <v>679</v>
+        <v>687</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>680</v>
+        <v>688</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>681</v>
+        <v>689</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>682</v>
+        <v>690</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>683</v>
+        <v>691</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>684</v>
+        <v>692</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>685</v>
+        <v>693</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>686</v>
+        <v>694</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>687</v>
+        <v>695</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>688</v>
+        <v>696</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>689</v>
+        <v>697</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>690</v>
+        <v>698</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>692</v>
+        <v>700</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>693</v>
+        <v>701</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="16" t="s">
-        <v>694</v>
+        <v>702</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
-        <v>695</v>
+        <v>703</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>696</v>
+        <v>704</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>697</v>
+        <v>705</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>698</v>
+        <v>706</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="14" t="s">
-        <v>699</v>
+        <v>707</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>700</v>
+        <v>708</v>
       </c>
       <c r="C17" s="14" t="s">
-        <v>701</v>
+        <v>709</v>
       </c>
       <c r="D17" s="14" t="s">
-        <v>702</v>
+        <v>710</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
-        <v>703</v>
+        <v>711</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>704</v>
+        <v>712</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>701</v>
+        <v>709</v>
       </c>
       <c r="D18" s="14" t="s">
-        <v>705</v>
+        <v>713</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="14" t="s">
-        <v>706</v>
+        <v>714</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>707</v>
+        <v>715</v>
       </c>
       <c r="C19" s="14" t="s">
-        <v>708</v>
+        <v>716</v>
       </c>
       <c r="D19" s="14" t="s">
-        <v>709</v>
+        <v>717</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="14" t="s">
-        <v>710</v>
+        <v>718</v>
       </c>
       <c r="B20" s="14" t="s">
         <v>28</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>711</v>
+        <v>719</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>712</v>
+        <v>720</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="14" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="B21" s="14" t="s">
         <v>30</v>
       </c>
       <c r="C21" s="14" t="s">
-        <v>714</v>
+        <v>722</v>
       </c>
       <c r="D21" s="14" t="s">
-        <v>715</v>
+        <v>723</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="14" t="s">
-        <v>716</v>
+        <v>724</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>701</v>
+        <v>709</v>
       </c>
       <c r="C22" s="14" t="s">
-        <v>711</v>
+        <v>719</v>
       </c>
       <c r="D22" s="14" t="s">
-        <v>717</v>
+        <v>725</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="16" t="s">
-        <v>718</v>
+        <v>726</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="9" t="s">
-        <v>719</v>
+        <v>727</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>720</v>
+        <v>728</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>721</v>
+        <v>729</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>722</v>
+        <v>730</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="14" t="s">
-        <v>723</v>
+        <v>731</v>
       </c>
       <c r="B26" s="14" t="s">
         <v>33</v>
       </c>
       <c r="C26" s="14" t="s">
-        <v>724</v>
+        <v>732</v>
       </c>
       <c r="D26" s="14" t="s">
-        <v>701</v>
+        <v>709</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="14" t="s">
-        <v>725</v>
+        <v>733</v>
       </c>
       <c r="B27" s="14" t="s">
-        <v>726</v>
+        <v>734</v>
       </c>
       <c r="C27" s="14" t="s">
-        <v>727</v>
+        <v>735</v>
       </c>
       <c r="D27" s="14" t="s">
-        <v>728</v>
+        <v>736</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="14" t="s">
-        <v>729</v>
+        <v>737</v>
       </c>
       <c r="B28" s="14" t="s">
-        <v>730</v>
+        <v>738</v>
       </c>
       <c r="C28" s="14" t="s">
-        <v>731</v>
+        <v>739</v>
       </c>
       <c r="D28" s="14" t="s">
-        <v>732</v>
+        <v>740</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="14" t="s">
-        <v>733</v>
+        <v>741</v>
       </c>
       <c r="B29" s="14" t="s">
-        <v>734</v>
+        <v>742</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>735</v>
+        <v>743</v>
       </c>
       <c r="D29" s="14" t="s">
-        <v>736</v>
+        <v>744</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="14" t="s">
-        <v>737</v>
+        <v>745</v>
       </c>
       <c r="B30" s="14" t="s">
         <v>30</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>738</v>
+        <v>746</v>
       </c>
       <c r="D30" s="14" t="s">
-        <v>739</v>
+        <v>747</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="14" t="s">
-        <v>740</v>
+        <v>748</v>
       </c>
       <c r="B31" s="14" t="s">
-        <v>741</v>
+        <v>749</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>742</v>
+        <v>750</v>
       </c>
       <c r="D31" s="14" t="s">
-        <v>743</v>
+        <v>751</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="14" t="s">
-        <v>744</v>
+        <v>752</v>
       </c>
       <c r="B32" s="14" t="s">
         <v>32</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>745</v>
+        <v>753</v>
       </c>
       <c r="D32" s="14" t="s">
-        <v>746</v>
+        <v>754</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="14" t="s">
-        <v>747</v>
+        <v>755</v>
       </c>
       <c r="B33" s="14" t="s">
         <v>28</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>748</v>
+        <v>756</v>
       </c>
       <c r="D33" s="14" t="s">
-        <v>749</v>
+        <v>757</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="13" t="s">
-        <v>750</v>
+        <v>758</v>
       </c>
     </row>
   </sheetData>

</xml_diff>